<commit_message>
feat: add core IT asset management components, services, and database seed
</commit_message>
<xml_diff>
--- a/database/IT_Asset_Database.xlsx
+++ b/database/IT_Asset_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\AnjeloPrograms\ITSystem\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E6EE5F-3E39-4649-84BF-E0810E932658}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BED2086A-9A2A-4C67-B8BF-8CC8C12C0DCA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="273">
   <si>
     <t>Name</t>
   </si>
@@ -398,28 +398,31 @@
     <t>AssetID</t>
   </si>
   <si>
+    <t>Printer</t>
+  </si>
+  <si>
+    <t>CANON</t>
+  </si>
+  <si>
+    <t>MF645C ufr ii</t>
+  </si>
+  <si>
+    <t>Assigned</t>
+  </si>
+  <si>
+    <t>AST-0057</t>
+  </si>
+  <si>
+    <t>KMN/CH/CP/016</t>
+  </si>
+  <si>
     <t>Laptop</t>
   </si>
   <si>
-    <t>CANON</t>
-  </si>
-  <si>
-    <t>MF645C ufr ii</t>
-  </si>
-  <si>
-    <t>Assigned</t>
-  </si>
-  <si>
-    <t>AST-0057</t>
-  </si>
-  <si>
-    <t>KMN/CH/CP/016</t>
-  </si>
-  <si>
     <t>Dell</t>
   </si>
   <si>
-    <t>NONE</t>
+    <t>Business Laptop</t>
   </si>
   <si>
     <t>AST-0056</t>
@@ -431,6 +434,12 @@
     <t>Mouse</t>
   </si>
   <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>Optical USB Mouse</t>
+  </si>
+  <si>
     <t>AST-0055</t>
   </si>
   <si>
@@ -446,18 +455,30 @@
     <t>Keyboard</t>
   </si>
   <si>
+    <t>Standard Keyboard</t>
+  </si>
+  <si>
     <t>AST-0053</t>
   </si>
   <si>
     <t>Desktop</t>
   </si>
   <si>
+    <t>Desktop PC Workstation</t>
+  </si>
+  <si>
     <t>AST-0052</t>
   </si>
   <si>
     <t>UPS</t>
   </si>
   <si>
+    <t>Office Standard</t>
+  </si>
+  <si>
+    <t>Office UPS Backup Unit</t>
+  </si>
+  <si>
     <t>AST-0051</t>
   </si>
   <si>
@@ -470,12 +491,18 @@
     <t>BRUKER</t>
   </si>
   <si>
+    <t>Laboratory Testing Machine</t>
+  </si>
+  <si>
     <t>AST-0050</t>
   </si>
   <si>
     <t>GAP/ATT/CP/011</t>
   </si>
   <si>
+    <t>Generic</t>
+  </si>
+  <si>
     <t>NIR MACHINE LAPTOP</t>
   </si>
   <si>
@@ -485,6 +512,9 @@
     <t>GAP/ATT/CP/012</t>
   </si>
   <si>
+    <t>Office UPS Backup (GAP/ATT/CP/012)</t>
+  </si>
+  <si>
     <t>AST-0048</t>
   </si>
   <si>
@@ -512,6 +542,9 @@
     <t>KMN/CH/CP/013</t>
   </si>
   <si>
+    <t>Office UPS Backup (KMN/CH/CP/013)</t>
+  </si>
+  <si>
     <t>AST-0043</t>
   </si>
   <si>
@@ -539,12 +572,18 @@
     <t>Monitor</t>
   </si>
   <si>
+    <t>Display Monitor</t>
+  </si>
+  <si>
     <t>AST-0039</t>
   </si>
   <si>
     <t>KMN/CH/CP/018</t>
   </si>
   <si>
+    <t>Office UPS Backup (KMN/CH/CP/018)</t>
+  </si>
+  <si>
     <t>AST-0038</t>
   </si>
   <si>
@@ -563,6 +602,9 @@
     <t>KMN/CH/CP/032</t>
   </si>
   <si>
+    <t>Office UPS Backup (KMN/CH/CP/032)</t>
+  </si>
+  <si>
     <t>AST-0034</t>
   </si>
   <si>
@@ -704,6 +746,9 @@
     <t>KMN/CH/CP/047</t>
   </si>
   <si>
+    <t>Office UPS Backup (KMN/CH/CP/047)</t>
+  </si>
+  <si>
     <t>AST-0007</t>
   </si>
   <si>
@@ -713,9 +758,6 @@
     <t>AST-0006</t>
   </si>
   <si>
-    <t>Printer</t>
-  </si>
-  <si>
     <t>EPSON</t>
   </si>
   <si>
@@ -741,6 +783,75 @@
   </si>
   <si>
     <t>AST-0001</t>
+  </si>
+  <si>
+    <t>RepairID</t>
+  </si>
+  <si>
+    <t>RepairDate</t>
+  </si>
+  <si>
+    <t>ProblemDescription</t>
+  </si>
+  <si>
+    <t>Diagnosis</t>
+  </si>
+  <si>
+    <t>ActionTaken</t>
+  </si>
+  <si>
+    <t>PartsReplaced</t>
+  </si>
+  <si>
+    <t>RepairSupplier</t>
+  </si>
+  <si>
+    <t>Technician</t>
+  </si>
+  <si>
+    <t>RepairCost</t>
+  </si>
+  <si>
+    <t>WarrantyCovered</t>
+  </si>
+  <si>
+    <t>CompletedDate</t>
+  </si>
+  <si>
+    <t>LastServiceDate</t>
+  </si>
+  <si>
+    <t>NextServiceDate</t>
+  </si>
+  <si>
+    <t>InvoiceID</t>
+  </si>
+  <si>
+    <t>REP-0001</t>
+  </si>
+  <si>
+    <t>UPS GIVE SOME BEEP SOUND</t>
+  </si>
+  <si>
+    <t>CHECKED BUY YOHAN</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>KMN IT Solution</t>
+  </si>
+  <si>
+    <t>KMN IT Service Specialist</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Warning / Under Observation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THIS IS AUTO FIXED BUT NEAD TO CHECK </t>
   </si>
 </sst>
 </file>
@@ -776,8 +887,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1118,9 +1230,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1155,7 +1267,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1190,7 +1302,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -1225,7 +1337,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -1260,7 +1372,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -1295,7 +1407,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1330,7 +1442,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -1365,7 +1477,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>41</v>
       </c>
@@ -1400,7 +1512,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>44</v>
       </c>
@@ -1435,7 +1547,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -1470,7 +1582,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>50</v>
       </c>
@@ -1505,7 +1617,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>53</v>
       </c>
@@ -1540,7 +1652,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>56</v>
       </c>
@@ -1575,7 +1687,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>60</v>
       </c>
@@ -1610,7 +1722,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>63</v>
       </c>
@@ -1645,7 +1757,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>66</v>
       </c>
@@ -1691,7 +1803,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1703,7 +1815,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1715,7 +1827,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1727,7 +1839,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1739,7 +1851,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1751,9 +1863,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1767,7 +1879,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1781,7 +1893,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -1795,7 +1907,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -1809,7 +1921,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -1823,7 +1935,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -1837,7 +1949,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1862,9 +1974,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>84</v>
       </c>
@@ -1887,7 +1999,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1910,7 +2022,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>94</v>
       </c>
@@ -1933,7 +2045,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>100</v>
       </c>
@@ -1956,7 +2068,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>104</v>
       </c>
@@ -1990,9 +2102,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:O58"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>108</v>
       </c>
@@ -2039,12 +2151,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>226</v>
+        <v>121</v>
       </c>
       <c r="C2" t="s">
         <v>122</v>
@@ -2086,18 +2198,18 @@
         <v>125</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>126</v>
       </c>
       <c r="B3" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E3" t="s">
         <v>14</v>
@@ -2130,21 +2242,21 @@
         <v>14</v>
       </c>
       <c r="O3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C4" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D4" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E4" t="s">
         <v>14</v>
@@ -2177,21 +2289,21 @@
         <v>14</v>
       </c>
       <c r="O4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="C5" t="s">
         <v>133</v>
       </c>
-      <c r="B5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C5" t="s">
-        <v>128</v>
-      </c>
       <c r="D5" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E5" t="s">
         <v>14</v>
@@ -2224,21 +2336,21 @@
         <v>14</v>
       </c>
       <c r="O5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D6" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
@@ -2271,21 +2383,21 @@
         <v>14</v>
       </c>
       <c r="O6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D7" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="E7" t="s">
         <v>14</v>
@@ -2318,21 +2430,21 @@
         <v>14</v>
       </c>
       <c r="O7" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C8" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D8" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E8" t="s">
         <v>14</v>
@@ -2365,21 +2477,21 @@
         <v>14</v>
       </c>
       <c r="O8" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B9" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C9" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="D9" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="E9" t="s">
         <v>14</v>
@@ -2412,21 +2524,21 @@
         <v>14</v>
       </c>
       <c r="O9" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B10" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="D10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E10" t="s">
         <v>14</v>
@@ -2456,24 +2568,24 @@
         <v>15</v>
       </c>
       <c r="N10" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="O10" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="B11" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C11" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D11" t="s">
-        <v>128</v>
+        <v>159</v>
       </c>
       <c r="E11" t="s">
         <v>14</v>
@@ -2506,68 +2618,68 @@
         <v>14</v>
       </c>
       <c r="O11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="B12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D12" t="s">
+        <v>134</v>
+      </c>
+      <c r="E12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J12" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" t="s">
+        <v>162</v>
+      </c>
+      <c r="L12" t="s">
+        <v>14</v>
+      </c>
+      <c r="M12" t="s">
+        <v>15</v>
+      </c>
+      <c r="N12" t="s">
+        <v>14</v>
+      </c>
+      <c r="O12" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>127</v>
+      </c>
+      <c r="C13" t="s">
         <v>128</v>
       </c>
-      <c r="D12" t="s">
-        <v>128</v>
-      </c>
-      <c r="E12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
-      </c>
-      <c r="I12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J12" t="s">
-        <v>14</v>
-      </c>
-      <c r="K12" t="s">
-        <v>152</v>
-      </c>
-      <c r="L12" t="s">
-        <v>14</v>
-      </c>
-      <c r="M12" t="s">
-        <v>15</v>
-      </c>
-      <c r="N12" t="s">
-        <v>14</v>
-      </c>
-      <c r="O12" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" t="s">
-        <v>127</v>
-      </c>
       <c r="D13" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E13" t="s">
         <v>14</v>
@@ -2588,7 +2700,7 @@
         <v>14</v>
       </c>
       <c r="K13" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="L13" t="s">
         <v>14</v>
@@ -2600,21 +2712,21 @@
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C14" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D14" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E14" t="s">
         <v>14</v>
@@ -2647,21 +2759,21 @@
         <v>14</v>
       </c>
       <c r="O14" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C15" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E15" t="s">
         <v>14</v>
@@ -2694,21 +2806,21 @@
         <v>14</v>
       </c>
       <c r="O15" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="B16" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C16" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D16" t="s">
-        <v>128</v>
+        <v>169</v>
       </c>
       <c r="E16" t="s">
         <v>14</v>
@@ -2741,21 +2853,21 @@
         <v>14</v>
       </c>
       <c r="O16" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C17" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="D17" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E17" t="s">
         <v>14</v>
@@ -2788,21 +2900,21 @@
         <v>14</v>
       </c>
       <c r="O17" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="B18" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C18" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D18" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="E18" t="s">
         <v>14</v>
@@ -2835,21 +2947,21 @@
         <v>14</v>
       </c>
       <c r="O18" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="B19" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D19" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E19" t="s">
         <v>14</v>
@@ -2882,21 +2994,21 @@
         <v>14</v>
       </c>
       <c r="O19" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="B20" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="C20" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D20" t="s">
-        <v>128</v>
+        <v>179</v>
       </c>
       <c r="E20" t="s">
         <v>14</v>
@@ -2929,21 +3041,21 @@
         <v>14</v>
       </c>
       <c r="O20" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="B21" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C21" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D21" t="s">
-        <v>128</v>
+        <v>182</v>
       </c>
       <c r="E21" t="s">
         <v>14</v>
@@ -2976,21 +3088,21 @@
         <v>14</v>
       </c>
       <c r="O21" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C22" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="D22" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="E22" t="s">
         <v>14</v>
@@ -3023,21 +3135,21 @@
         <v>14</v>
       </c>
       <c r="O22" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C23" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D23" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="E23" t="s">
         <v>14</v>
@@ -3070,21 +3182,21 @@
         <v>14</v>
       </c>
       <c r="O23" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>14</v>
       </c>
       <c r="B24" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="C24" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D24" t="s">
-        <v>128</v>
+        <v>179</v>
       </c>
       <c r="E24" t="s">
         <v>14</v>
@@ -3117,21 +3229,21 @@
         <v>14</v>
       </c>
       <c r="O24" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="B25" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C25" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D25" t="s">
-        <v>128</v>
+        <v>189</v>
       </c>
       <c r="E25" t="s">
         <v>14</v>
@@ -3164,21 +3276,21 @@
         <v>14</v>
       </c>
       <c r="O25" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>14</v>
       </c>
       <c r="B26" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="C26" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="D26" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="E26" t="s">
         <v>14</v>
@@ -3211,21 +3323,21 @@
         <v>14</v>
       </c>
       <c r="O26" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C27" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D27" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E27" t="s">
         <v>14</v>
@@ -3258,21 +3370,21 @@
         <v>14</v>
       </c>
       <c r="O27" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="B28" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C28" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D28" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="E28" t="s">
         <v>14</v>
@@ -3302,24 +3414,24 @@
         <v>15</v>
       </c>
       <c r="N28" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="O28" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="B29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C29" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D29" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E29" t="s">
         <v>14</v>
@@ -3352,21 +3464,21 @@
         <v>14</v>
       </c>
       <c r="O29" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C30" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D30" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E30" t="s">
         <v>14</v>
@@ -3399,21 +3511,21 @@
         <v>14</v>
       </c>
       <c r="O30" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="B31" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C31" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D31" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E31" t="s">
         <v>14</v>
@@ -3446,21 +3558,21 @@
         <v>14</v>
       </c>
       <c r="O31" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="B32" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D32" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E32" t="s">
         <v>14</v>
@@ -3493,21 +3605,21 @@
         <v>14</v>
       </c>
       <c r="O32" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>14</v>
       </c>
       <c r="B33" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="C33" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="D33" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="E33" t="s">
         <v>14</v>
@@ -3540,21 +3652,21 @@
         <v>14</v>
       </c>
       <c r="O33" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>14</v>
       </c>
       <c r="B34" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C34" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D34" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E34" t="s">
         <v>14</v>
@@ -3587,21 +3699,21 @@
         <v>14</v>
       </c>
       <c r="O34" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>14</v>
       </c>
       <c r="B35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C35" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D35" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E35" t="s">
         <v>14</v>
@@ -3634,21 +3746,21 @@
         <v>14</v>
       </c>
       <c r="O35" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>14</v>
       </c>
       <c r="B36" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C36" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D36" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="E36" t="s">
         <v>14</v>
@@ -3681,21 +3793,21 @@
         <v>14</v>
       </c>
       <c r="O36" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="B37" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C37" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D37" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E37" t="s">
         <v>14</v>
@@ -3728,21 +3840,21 @@
         <v>14</v>
       </c>
       <c r="O37" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="B38" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C38" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="D38" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="E38" t="s">
         <v>14</v>
@@ -3775,21 +3887,21 @@
         <v>14</v>
       </c>
       <c r="O38" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>14</v>
       </c>
       <c r="B39" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C39" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D39" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E39" t="s">
         <v>14</v>
@@ -3822,21 +3934,21 @@
         <v>14</v>
       </c>
       <c r="O39" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>14</v>
       </c>
       <c r="B40" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C40" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D40" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E40" t="s">
         <v>14</v>
@@ -3869,21 +3981,21 @@
         <v>14</v>
       </c>
       <c r="O40" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>14</v>
       </c>
       <c r="B41" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C41" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D41" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E41" t="s">
         <v>14</v>
@@ -3916,21 +4028,21 @@
         <v>14</v>
       </c>
       <c r="O41" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>14</v>
-      </c>
-      <c r="B42" t="s">
-        <v>191</v>
-      </c>
       <c r="C42" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D42" t="s">
-        <v>128</v>
+        <v>205</v>
       </c>
       <c r="E42" t="s">
         <v>14</v>
@@ -3963,21 +4075,21 @@
         <v>14</v>
       </c>
       <c r="O42" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C43" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D43" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E43" t="s">
         <v>14</v>
@@ -4010,21 +4122,21 @@
         <v>14</v>
       </c>
       <c r="O43" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C44" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D44" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E44" t="s">
         <v>14</v>
@@ -4057,21 +4169,21 @@
         <v>14</v>
       </c>
       <c r="O44" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>14</v>
       </c>
       <c r="B45" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C45" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E45" t="s">
         <v>14</v>
@@ -4104,21 +4216,21 @@
         <v>14</v>
       </c>
       <c r="O45" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="B46" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="C46" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="D46" t="s">
-        <v>128</v>
+        <v>205</v>
       </c>
       <c r="E46" t="s">
         <v>14</v>
@@ -4151,21 +4263,21 @@
         <v>14</v>
       </c>
       <c r="O46" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="B47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C47" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D47" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E47" t="s">
         <v>14</v>
@@ -4198,21 +4310,21 @@
         <v>14</v>
       </c>
       <c r="O47" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="B48" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C48" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="D48" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E48" t="s">
         <v>14</v>
@@ -4245,21 +4357,21 @@
         <v>14</v>
       </c>
       <c r="O48" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="B49" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C49" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D49" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="E49" t="s">
         <v>14</v>
@@ -4292,21 +4404,21 @@
         <v>14</v>
       </c>
       <c r="O49" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="B50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C50" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D50" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E50" t="s">
         <v>14</v>
@@ -4339,21 +4451,21 @@
         <v>14</v>
       </c>
       <c r="O50" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="B51" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C51" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D51" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E51" t="s">
         <v>14</v>
@@ -4386,21 +4498,21 @@
         <v>14</v>
       </c>
       <c r="O51" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="B52" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C52" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D52" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="E52" t="s">
         <v>14</v>
@@ -4433,21 +4545,21 @@
         <v>14</v>
       </c>
       <c r="O52" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="B53" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="C53" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="D53" t="s">
-        <v>128</v>
+        <v>179</v>
       </c>
       <c r="E53" t="s">
         <v>14</v>
@@ -4480,21 +4592,21 @@
         <v>14</v>
       </c>
       <c r="O53" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>14</v>
       </c>
       <c r="B54" t="s">
-        <v>226</v>
+        <v>121</v>
       </c>
       <c r="C54" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="D54" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="E54" t="s">
         <v>14</v>
@@ -4527,21 +4639,21 @@
         <v>14</v>
       </c>
       <c r="O54" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>14</v>
       </c>
       <c r="B55" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C55" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D55" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E55" t="s">
         <v>14</v>
@@ -4574,21 +4686,21 @@
         <v>14</v>
       </c>
       <c r="O55" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="B56" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C56" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E56" t="s">
         <v>14</v>
@@ -4621,21 +4733,21 @@
         <v>14</v>
       </c>
       <c r="O56" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="B57" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="C57" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="D57" t="s">
-        <v>128</v>
+        <v>179</v>
       </c>
       <c r="E57" t="s">
         <v>14</v>
@@ -4668,21 +4780,21 @@
         <v>14</v>
       </c>
       <c r="O57" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="B58" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C58" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D58" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E58" t="s">
         <v>14</v>
@@ -4715,13 +4827,13 @@
         <v>14</v>
       </c>
       <c r="O58" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:O1 A3:O58 A2 C2:O2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:O58" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4729,7 +4841,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -4741,7 +4853,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -4753,7 +4865,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -4765,7 +4877,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -4776,12 +4888,122 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="22.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C1" t="s">
+        <v>251</v>
+      </c>
+      <c r="D1" t="s">
+        <v>252</v>
+      </c>
+      <c r="E1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F1" t="s">
+        <v>254</v>
+      </c>
+      <c r="G1" t="s">
+        <v>255</v>
+      </c>
+      <c r="H1" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1" t="s">
+        <v>257</v>
+      </c>
+      <c r="J1" t="s">
+        <v>258</v>
+      </c>
+      <c r="K1" t="s">
+        <v>259</v>
+      </c>
+      <c r="L1" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" t="s">
+        <v>260</v>
+      </c>
+      <c r="N1" t="s">
+        <v>261</v>
+      </c>
+      <c r="O1" t="s">
+        <v>262</v>
+      </c>
+      <c r="P1" t="s">
+        <v>263</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C2" s="1">
+        <v>46270</v>
+      </c>
+      <c r="D2" t="s">
+        <v>265</v>
+      </c>
+      <c r="E2" t="s">
+        <v>265</v>
+      </c>
+      <c r="F2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G2" t="s">
+        <v>267</v>
+      </c>
+      <c r="H2" t="s">
+        <v>268</v>
+      </c>
+      <c r="I2" t="s">
+        <v>269</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>270</v>
+      </c>
+      <c r="L2" t="s">
+        <v>271</v>
+      </c>
+      <c r="M2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" t="s">
+        <v>17</v>
+      </c>
+      <c r="O2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P2" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:Q1 A2:B2 D2:Q2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add core IT system application with CCTV management, global search, and Excel database integration
</commit_message>
<xml_diff>
--- a/database/IT_Asset_Database.xlsx
+++ b/database/IT_Asset_Database.xlsx
@@ -16,7 +16,8 @@
     <sheet name="Expenses" sheetId="11" r:id="rId11"/>
     <sheet name="Invoices" sheetId="12" r:id="rId12"/>
     <sheet name="Suppliers" sheetId="13" r:id="rId13"/>
-    <sheet name="LegacyRawImport" sheetId="14" r:id="rId14"/>
+    <sheet name="CCTVBills" sheetId="14" r:id="rId14"/>
+    <sheet name="LegacyRawImport" sheetId="15" r:id="rId15"/>
   </sheets>
 </workbook>
 </file>
@@ -1440,7 +1441,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1485,98 +1486,98 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EXP-0009</v>
+        <v>EXP-0012</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-23</v>
       </c>
       <c r="C2" t="str">
-        <v>Consumable / Toner</v>
+        <v>CCTV Bill (Palawiya)</v>
       </c>
       <c r="D2" t="str">
-        <v>AST-0057</v>
+        <v/>
       </c>
       <c r="E2" t="str">
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>AST-0057</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>DEP-0002</v>
+        <v>DEP-0004</v>
       </c>
       <c r="H2" t="str">
-        <v>KMN IT Solution</v>
+        <v>KMN IT</v>
       </c>
       <c r="I2" t="str">
-        <v>Black Toner Replacement (Cartridge 337 / 047)</v>
+        <v>[CCTV - Palawiya] 32 TV and wireless 2 mouse (Bill: 09.09.2026.)</v>
       </c>
       <c r="J2">
-        <v>4800</v>
+        <v>38000</v>
       </c>
       <c r="K2" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L2" t="str">
-        <v>INV-0007</v>
+        <v>CCTV-0003</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>Categorized under General / Other for Palawiya CCTV surveillance</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EXP-0008</v>
+        <v>EXP-0011</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-07-23</v>
+        <v>2026-09-11</v>
       </c>
       <c r="C3" t="str">
-        <v>Consumable / Toner</v>
+        <v>CCTV Bill (Palawiya)</v>
       </c>
       <c r="D3" t="str">
-        <v>AST-0059</v>
+        <v/>
       </c>
       <c r="E3" t="str">
         <v/>
       </c>
       <c r="F3" t="str">
-        <v>AST-0059</v>
+        <v/>
       </c>
       <c r="G3" t="str">
-        <v>DEP-0002</v>
+        <v>DEP-0004</v>
       </c>
       <c r="H3" t="str">
-        <v>KMN IT Solution</v>
+        <v>Dilex Computer System</v>
       </c>
       <c r="I3" t="str">
-        <v>Black Toner Replacement (Standard Toner)</v>
+        <v>[CCTV - Palawiya] 2TB HDD, Wall mount Tv stand ,5M HDMI Cable (Bill: DI61077)</v>
       </c>
       <c r="J3">
-        <v>8000</v>
+        <v>59100</v>
       </c>
       <c r="K3" t="str">
-        <v>Company Cheque</v>
+        <v>Bank Transfer</v>
       </c>
       <c r="L3" t="str">
-        <v>INV-0006</v>
+        <v>CCTV-0002</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>Categorized under Internet &amp; Remote Access for Palawiya CCTV surveillance</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EXP-0007</v>
+        <v>EXP-0010</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-08-14</v>
+        <v>2026-09-08</v>
       </c>
       <c r="C4" t="str">
-        <v>Hardware Upgrade / RAM</v>
+        <v>CCTV Bill (Chilaw Portion)</v>
       </c>
       <c r="D4" t="str">
-        <v>AST-0056</v>
+        <v/>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -1588,83 +1589,83 @@
         <v>DEP-0004</v>
       </c>
       <c r="H4" t="str">
-        <v>KMN IT Solution</v>
+        <v>Dilex Computer System</v>
       </c>
       <c r="I4" t="str">
-        <v>DDR4 4GB RAM Upgrade for Laptop (S/N: K06G00013812690D7C - Invoice 1641)</v>
+        <v>[CCTV - Chilaw Share] BAT-CMO-0002 CR 1220 MAXELL LITHIUM BATTERY (Bill: DI61042)</v>
       </c>
       <c r="J4">
-        <v>7000</v>
+        <v>550</v>
       </c>
       <c r="K4" t="str">
-        <v>Company Cheque</v>
+        <v>Bank Transfer</v>
       </c>
       <c r="L4" t="str">
-        <v>INV-0005</v>
+        <v>CCTV-0001</v>
       </c>
       <c r="M4" t="str">
-        <v>kalpana laptop (4gb ram) DDR4 4GB RAM - One Year Warranty</v>
+        <v>Split portion for Chilaw Office CCTV</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EXP-0006</v>
+        <v>EXP-0010</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-08-14</v>
+        <v>2026-09-08</v>
       </c>
       <c r="C5" t="str">
-        <v>Consumable / Toner</v>
+        <v>CCTV Bill (Palawiya Portion)</v>
       </c>
       <c r="D5" t="str">
-        <v>AST-0060</v>
+        <v/>
       </c>
       <c r="E5" t="str">
         <v/>
       </c>
       <c r="F5" t="str">
-        <v>AST-0060</v>
+        <v/>
       </c>
       <c r="G5" t="str">
-        <v>DEP-0002</v>
+        <v>DEP-0004</v>
       </c>
       <c r="H5" t="str">
-        <v>KMN IT Solution</v>
+        <v>Dilex Computer System</v>
       </c>
       <c r="I5" t="str">
-        <v>Black Toner Replacement (Standard Toner)</v>
+        <v>[CCTV - Palawiya Share] MOUSE, TECHNICAL SERVICE, CR123A BATTERY (Bill: DI61042)</v>
       </c>
       <c r="J5">
-        <v>2200</v>
+        <v>10450</v>
       </c>
       <c r="K5" t="str">
-        <v>Company Cheque</v>
+        <v>Bank Transfer</v>
       </c>
       <c r="L5" t="str">
-        <v>INV-0005</v>
+        <v>CCTV-0001</v>
       </c>
       <c r="M5" t="str">
-        <v>ASTA 337/83X TONER</v>
+        <v>Split portion for Palawiya Office CCTV</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EXP-0005</v>
+        <v>EXP-0009</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-07-01</v>
+        <v>2026-09-17</v>
       </c>
       <c r="C6" t="str">
         <v>Consumable / Toner</v>
       </c>
       <c r="D6" t="str">
-        <v>AST-0063</v>
+        <v>AST-0057</v>
       </c>
       <c r="E6" t="str">
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>AST-0063</v>
+        <v>AST-0057</v>
       </c>
       <c r="G6" t="str">
         <v>DEP-0002</v>
@@ -1673,16 +1674,16 @@
         <v>KMN IT Solution</v>
       </c>
       <c r="I6" t="str">
-        <v>Color Toner Replacement (Standard Toner)</v>
+        <v>Black Toner Replacement (Cartridge 337 / 047)</v>
       </c>
       <c r="J6">
-        <v>2850</v>
+        <v>4800</v>
       </c>
       <c r="K6" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L6" t="str">
-        <v>INV-0004</v>
+        <v>INV-0007</v>
       </c>
       <c r="M6" t="str">
         <v/>
@@ -1690,22 +1691,22 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EXP-0004</v>
+        <v>EXP-0008</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-07-01</v>
+        <v>2026-07-23</v>
       </c>
       <c r="C7" t="str">
         <v>Consumable / Toner</v>
       </c>
       <c r="D7" t="str">
-        <v>AST-0063</v>
+        <v>AST-0059</v>
       </c>
       <c r="E7" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>AST-0063</v>
+        <v>AST-0059</v>
       </c>
       <c r="G7" t="str">
         <v>DEP-0002</v>
@@ -1717,13 +1718,13 @@
         <v>Black Toner Replacement (Standard Toner)</v>
       </c>
       <c r="J7">
-        <v>2800</v>
+        <v>8000</v>
       </c>
       <c r="K7" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L7" t="str">
-        <v>INV-0004</v>
+        <v>INV-0006</v>
       </c>
       <c r="M7" t="str">
         <v/>
@@ -1731,19 +1732,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EXP-0003</v>
+        <v>EXP-0007</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-09-07</v>
+        <v>2026-08-14</v>
       </c>
       <c r="C8" t="str">
-        <v>Repair</v>
+        <v>Hardware Upgrade / RAM</v>
       </c>
       <c r="D8" t="str">
-        <v>AST-0052</v>
+        <v>AST-0056</v>
       </c>
       <c r="E8" t="str">
-        <v>USR-0014</v>
+        <v/>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -1755,106 +1756,270 @@
         <v>KMN IT Solution</v>
       </c>
       <c r="I8" t="str">
-        <v>Repair for Desktop PC Workstation: HAVEN'T A MOUSE</v>
+        <v>DDR4 4GB RAM Upgrade for Laptop (S/N: K06G00013812690D7C - Invoice 1641)</v>
       </c>
       <c r="J8">
-        <v>1000</v>
+        <v>7000</v>
       </c>
       <c r="K8" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L8" t="str">
-        <v>INV-0003</v>
+        <v>INV-0005</v>
       </c>
       <c r="M8" t="str">
-        <v/>
+        <v>kalpana laptop (4gb ram) DDR4 4GB RAM - One Year Warranty</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EXP-0002</v>
+        <v>EXP-0006</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-09-10</v>
+        <v>2026-08-14</v>
       </c>
       <c r="C9" t="str">
-        <v>Repair</v>
+        <v>Consumable / Toner</v>
       </c>
       <c r="D9" t="str">
-        <v>AST-0052</v>
+        <v>AST-0060</v>
       </c>
       <c r="E9" t="str">
-        <v>USR-0014</v>
+        <v/>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>AST-0060</v>
       </c>
       <c r="G9" t="str">
-        <v>DEP-0004</v>
+        <v>DEP-0002</v>
       </c>
       <c r="H9" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="I9" t="str">
-        <v>Repair for Desktop PC Workstation: STUCK &amp; SLOW (2 parts replaced)</v>
+        <v>Black Toner Replacement (Standard Toner)</v>
       </c>
       <c r="J9">
-        <v>30000</v>
+        <v>2200</v>
       </c>
       <c r="K9" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L9" t="str">
-        <v>INV-0002</v>
+        <v>INV-0005</v>
       </c>
       <c r="M9" t="str">
-        <v/>
+        <v>ASTA 337/83X TONER</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>EXP-0001</v>
+        <v>EXP-0005</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-09-08</v>
+        <v>2026-07-01</v>
       </c>
       <c r="C10" t="str">
-        <v>Repair</v>
+        <v>Consumable / Toner</v>
       </c>
       <c r="D10" t="str">
-        <v>AST-0041</v>
+        <v>AST-0063</v>
       </c>
       <c r="E10" t="str">
-        <v>USR-0010</v>
+        <v/>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>AST-0063</v>
       </c>
       <c r="G10" t="str">
-        <v>DEP-0004</v>
+        <v>DEP-0002</v>
       </c>
       <c r="H10" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="I10" t="str">
-        <v>Repair for Desktop PC Workstation: STUCK &amp; SLOW (2 parts replaced)</v>
+        <v>Color Toner Replacement (Standard Toner)</v>
       </c>
       <c r="J10">
-        <v>36000</v>
+        <v>2850</v>
       </c>
       <c r="K10" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L10" t="str">
+        <v>INV-0004</v>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>EXP-0004</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Consumable / Toner</v>
+      </c>
+      <c r="D11" t="str">
+        <v>AST-0063</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v>AST-0063</v>
+      </c>
+      <c r="G11" t="str">
+        <v>DEP-0002</v>
+      </c>
+      <c r="H11" t="str">
+        <v>KMN IT Solution</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Black Toner Replacement (Standard Toner)</v>
+      </c>
+      <c r="J11">
+        <v>2800</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Company Cheque</v>
+      </c>
+      <c r="L11" t="str">
+        <v>INV-0004</v>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>EXP-0003</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Repair</v>
+      </c>
+      <c r="D12" t="str">
+        <v>AST-0052</v>
+      </c>
+      <c r="E12" t="str">
+        <v>USR-0014</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v>DEP-0004</v>
+      </c>
+      <c r="H12" t="str">
+        <v>KMN IT Solution</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Repair for Desktop PC Workstation: HAVEN'T A MOUSE</v>
+      </c>
+      <c r="J12">
+        <v>1000</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Company Cheque</v>
+      </c>
+      <c r="L12" t="str">
+        <v>INV-0003</v>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>EXP-0002</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-09-10</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Repair</v>
+      </c>
+      <c r="D13" t="str">
+        <v>AST-0052</v>
+      </c>
+      <c r="E13" t="str">
+        <v>USR-0014</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v>DEP-0004</v>
+      </c>
+      <c r="H13" t="str">
+        <v>KMN IT Solution</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Repair for Desktop PC Workstation: STUCK &amp; SLOW (2 parts replaced)</v>
+      </c>
+      <c r="J13">
+        <v>30000</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Company Cheque</v>
+      </c>
+      <c r="L13" t="str">
+        <v>INV-0002</v>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>EXP-0001</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Repair</v>
+      </c>
+      <c r="D14" t="str">
+        <v>AST-0041</v>
+      </c>
+      <c r="E14" t="str">
+        <v>USR-0010</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v>DEP-0004</v>
+      </c>
+      <c r="H14" t="str">
+        <v>KMN IT Solution</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Repair for Desktop PC Workstation: STUCK &amp; SLOW (2 parts replaced)</v>
+      </c>
+      <c r="J14">
+        <v>36000</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Company Cheque</v>
+      </c>
+      <c r="L14" t="str">
         <v>INV-0001</v>
       </c>
-      <c r="M10" t="str">
+      <c r="M14" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2233,6 +2398,265 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>BillID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Office</v>
+      </c>
+      <c r="C1" t="str">
+        <v>LocationID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>BillNumber</v>
+      </c>
+      <c r="E1" t="str">
+        <v>BillDate</v>
+      </c>
+      <c r="F1" t="str">
+        <v>BillPeriod</v>
+      </c>
+      <c r="G1" t="str">
+        <v>BillCategory</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Supplier</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Amount</v>
+      </c>
+      <c r="J1" t="str">
+        <v>ChilawAmount</v>
+      </c>
+      <c r="K1" t="str">
+        <v>PalawiyaAmount</v>
+      </c>
+      <c r="L1" t="str">
+        <v>ChilawDescription</v>
+      </c>
+      <c r="M1" t="str">
+        <v>PalawiyaDescription</v>
+      </c>
+      <c r="N1" t="str">
+        <v>PaymentStatus</v>
+      </c>
+      <c r="O1" t="str">
+        <v>PaymentMethod</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="R1" t="str">
+        <v>FileName</v>
+      </c>
+      <c r="S1" t="str">
+        <v>FilePath</v>
+      </c>
+      <c r="T1" t="str">
+        <v>FileSize</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>CCTV-0003</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Palawiya</v>
+      </c>
+      <c r="C2" t="str">
+        <v>LOC-0002</v>
+      </c>
+      <c r="D2" t="str">
+        <v>09.09.2026.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="F2" t="str">
+        <v>September 2026</v>
+      </c>
+      <c r="G2" t="str">
+        <v>General / Other</v>
+      </c>
+      <c r="H2" t="str">
+        <v>KMN IT</v>
+      </c>
+      <c r="I2">
+        <v>38000</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>38000</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Company Cheque</v>
+      </c>
+      <c r="P2" t="str">
+        <v>32 TV and wireless 2 mouse</v>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v>09.09.2026..pdf</v>
+      </c>
+      <c r="S2" t="str">
+        <v>/invoices/09.09.2026..pdf</v>
+      </c>
+      <c r="T2" t="str">
+        <v>643 KB</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>CCTV-0002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Palawiya</v>
+      </c>
+      <c r="C3" t="str">
+        <v>LOC-0002</v>
+      </c>
+      <c r="D3" t="str">
+        <v>DI61077</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="F3" t="str">
+        <v>September 2026</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Internet &amp; Remote Access</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Dilex Computer System</v>
+      </c>
+      <c r="I3">
+        <v>59100</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>59100</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Bank Transfer</v>
+      </c>
+      <c r="P3" t="str">
+        <v>2TB HDD, Wall mount Tv stand ,5M HDMI Cable</v>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v>DI61077.pdf</v>
+      </c>
+      <c r="S3" t="str">
+        <v>/invoices/DI61077.pdf</v>
+      </c>
+      <c r="T3" t="str">
+        <v>679 KB</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>CCTV-0001</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Split</v>
+      </c>
+      <c r="C4" t="str">
+        <v>LOC-BOTH</v>
+      </c>
+      <c r="D4" t="str">
+        <v>DI61042</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="F4" t="str">
+        <v>September 2026</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Internet &amp; Remote Access</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Dilex Computer System</v>
+      </c>
+      <c r="I4">
+        <v>11000</v>
+      </c>
+      <c r="J4">
+        <v>550</v>
+      </c>
+      <c r="K4">
+        <v>10450</v>
+      </c>
+      <c r="L4" t="str">
+        <v>BAT-CMO-0002 CR 1220 MAXELL LITHIUM BATTERY</v>
+      </c>
+      <c r="M4" t="str">
+        <v>MOUSE, TECHNICAL SERVICE, CR123A BATTERY</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Bank Transfer</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Split Bill: Chilaw (Rs. 550) &amp; Palawiya (Rs. 10,450)</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v>DI61042.pdf</v>
+      </c>
+      <c r="S4" t="str">
+        <v>/invoices/DI61042.pdf</v>
+      </c>
+      <c r="T4" t="str">
+        <v>677 KB</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:T4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetData/>

</xml_diff>

<commit_message>
feat: add cctvService and invoiceService modules for CCTV management and billing
</commit_message>
<xml_diff>
--- a/database/IT_Asset_Database.xlsx
+++ b/database/IT_Asset_Database.xlsx
@@ -1441,7 +1441,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1486,19 +1486,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EXP-0012</v>
+        <v>EXP-0014</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-23</v>
+        <v>2026-08-04</v>
       </c>
       <c r="C2" t="str">
-        <v>CCTV Bill (Palawiya)</v>
+        <v>Repair</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>AST-0052</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>USR-0014</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -1507,30 +1507,30 @@
         <v>DEP-0004</v>
       </c>
       <c r="H2" t="str">
-        <v>KMN IT</v>
+        <v>KMN IT Solution</v>
       </c>
       <c r="I2" t="str">
-        <v>[CCTV - Palawiya] 32 TV and wireless 2 mouse (Bill: 09.09.2026.)</v>
+        <v xml:space="preserve">Repair for Desktop PC Workstation: Power cable not worked </v>
       </c>
       <c r="J2">
-        <v>38000</v>
+        <v>1000</v>
       </c>
       <c r="K2" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L2" t="str">
-        <v>CCTV-0003</v>
+        <v>INV-0008</v>
       </c>
       <c r="M2" t="str">
-        <v>Categorized under General / Other for Palawiya CCTV surveillance</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EXP-0011</v>
+        <v>EXP-0012</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-23</v>
       </c>
       <c r="C3" t="str">
         <v>CCTV Bill (Palawiya)</v>
@@ -1548,33 +1548,33 @@
         <v>DEP-0004</v>
       </c>
       <c r="H3" t="str">
-        <v>Dilex Computer System</v>
+        <v>KMN IT</v>
       </c>
       <c r="I3" t="str">
-        <v>[CCTV - Palawiya] 2TB HDD, Wall mount Tv stand ,5M HDMI Cable (Bill: DI61077)</v>
+        <v>[CCTV - Palawiya] 32 TV and wireless 2 mouse (Bill: 09.09.2026.)</v>
       </c>
       <c r="J3">
-        <v>59100</v>
+        <v>38000</v>
       </c>
       <c r="K3" t="str">
-        <v>Bank Transfer</v>
+        <v>Company Cheque</v>
       </c>
       <c r="L3" t="str">
-        <v>CCTV-0002</v>
+        <v>CCTV-0003</v>
       </c>
       <c r="M3" t="str">
-        <v>Categorized under Internet &amp; Remote Access for Palawiya CCTV surveillance</v>
+        <v>Categorized under General / Other for Palawiya CCTV surveillance</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EXP-0010</v>
+        <v>EXP-0011</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-11</v>
       </c>
       <c r="C4" t="str">
-        <v>CCTV Bill (Chilaw Portion)</v>
+        <v>CCTV Bill (Palawiya)</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -1592,19 +1592,19 @@
         <v>Dilex Computer System</v>
       </c>
       <c r="I4" t="str">
-        <v>[CCTV - Chilaw Share] BAT-CMO-0002 CR 1220 MAXELL LITHIUM BATTERY (Bill: DI61042)</v>
+        <v>[CCTV - Palawiya] 2TB HDD, Wall mount Tv stand ,5M HDMI Cable (Bill: DI61077)</v>
       </c>
       <c r="J4">
-        <v>550</v>
+        <v>59100</v>
       </c>
       <c r="K4" t="str">
         <v>Bank Transfer</v>
       </c>
       <c r="L4" t="str">
-        <v>CCTV-0001</v>
+        <v>CCTV-0002</v>
       </c>
       <c r="M4" t="str">
-        <v>Split portion for Chilaw Office CCTV</v>
+        <v>Categorized under Internet &amp; Remote Access for Palawiya CCTV surveillance</v>
       </c>
     </row>
     <row r="5">
@@ -1615,7 +1615,7 @@
         <v>2026-09-08</v>
       </c>
       <c r="C5" t="str">
-        <v>CCTV Bill (Palawiya Portion)</v>
+        <v>CCTV Bill (Chilaw Portion)</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -1633,10 +1633,10 @@
         <v>Dilex Computer System</v>
       </c>
       <c r="I5" t="str">
-        <v>[CCTV - Palawiya Share] MOUSE, TECHNICAL SERVICE, CR123A BATTERY (Bill: DI61042)</v>
+        <v>[CCTV - Chilaw Share] BAT-CMO-0002 CR 1220 MAXELL LITHIUM BATTERY (Bill: DI61042)</v>
       </c>
       <c r="J5">
-        <v>10450</v>
+        <v>550</v>
       </c>
       <c r="K5" t="str">
         <v>Bank Transfer</v>
@@ -1645,68 +1645,68 @@
         <v>CCTV-0001</v>
       </c>
       <c r="M5" t="str">
-        <v>Split portion for Palawiya Office CCTV</v>
+        <v>Split portion for Chilaw Office CCTV</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EXP-0009</v>
+        <v>EXP-0010</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-08</v>
       </c>
       <c r="C6" t="str">
-        <v>Consumable / Toner</v>
+        <v>CCTV Bill (Palawiya Portion)</v>
       </c>
       <c r="D6" t="str">
-        <v>AST-0057</v>
+        <v/>
       </c>
       <c r="E6" t="str">
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>AST-0057</v>
+        <v/>
       </c>
       <c r="G6" t="str">
-        <v>DEP-0002</v>
+        <v>DEP-0004</v>
       </c>
       <c r="H6" t="str">
-        <v>KMN IT Solution</v>
+        <v>Dilex Computer System</v>
       </c>
       <c r="I6" t="str">
-        <v>Black Toner Replacement (Cartridge 337 / 047)</v>
+        <v>[CCTV - Palawiya Share] MOUSE, TECHNICAL SERVICE, CR123A BATTERY (Bill: DI61042)</v>
       </c>
       <c r="J6">
-        <v>4800</v>
+        <v>10450</v>
       </c>
       <c r="K6" t="str">
-        <v>Company Cheque</v>
+        <v>Bank Transfer</v>
       </c>
       <c r="L6" t="str">
-        <v>INV-0007</v>
+        <v>CCTV-0001</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>Split portion for Palawiya Office CCTV</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EXP-0008</v>
+        <v>EXP-0009</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-07-23</v>
+        <v>2026-09-17</v>
       </c>
       <c r="C7" t="str">
         <v>Consumable / Toner</v>
       </c>
       <c r="D7" t="str">
-        <v>AST-0059</v>
+        <v>AST-0057</v>
       </c>
       <c r="E7" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>AST-0059</v>
+        <v>AST-0057</v>
       </c>
       <c r="G7" t="str">
         <v>DEP-0002</v>
@@ -1715,16 +1715,16 @@
         <v>KMN IT Solution</v>
       </c>
       <c r="I7" t="str">
-        <v>Black Toner Replacement (Standard Toner)</v>
+        <v>Black Toner Replacement (Cartridge 337 / 047)</v>
       </c>
       <c r="J7">
-        <v>8000</v>
+        <v>4800</v>
       </c>
       <c r="K7" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L7" t="str">
-        <v>INV-0006</v>
+        <v>INV-0007</v>
       </c>
       <c r="M7" t="str">
         <v/>
@@ -1732,75 +1732,75 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EXP-0007</v>
+        <v>EXP-0008</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-08-14</v>
+        <v>2026-07-23</v>
       </c>
       <c r="C8" t="str">
-        <v>Hardware Upgrade / RAM</v>
+        <v>Consumable / Toner</v>
       </c>
       <c r="D8" t="str">
-        <v>AST-0056</v>
+        <v>AST-0059</v>
       </c>
       <c r="E8" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>AST-0059</v>
       </c>
       <c r="G8" t="str">
-        <v>DEP-0004</v>
+        <v>DEP-0002</v>
       </c>
       <c r="H8" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="I8" t="str">
-        <v>DDR4 4GB RAM Upgrade for Laptop (S/N: K06G00013812690D7C - Invoice 1641)</v>
+        <v>Black Toner Replacement (Standard Toner)</v>
       </c>
       <c r="J8">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="K8" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L8" t="str">
-        <v>INV-0005</v>
+        <v>INV-0006</v>
       </c>
       <c r="M8" t="str">
-        <v>kalpana laptop (4gb ram) DDR4 4GB RAM - One Year Warranty</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EXP-0006</v>
+        <v>EXP-0007</v>
       </c>
       <c r="B9" t="str">
         <v>2026-08-14</v>
       </c>
       <c r="C9" t="str">
-        <v>Consumable / Toner</v>
+        <v>Hardware Upgrade / RAM</v>
       </c>
       <c r="D9" t="str">
-        <v>AST-0060</v>
+        <v>AST-0056</v>
       </c>
       <c r="E9" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>AST-0060</v>
+        <v/>
       </c>
       <c r="G9" t="str">
-        <v>DEP-0002</v>
+        <v>DEP-0004</v>
       </c>
       <c r="H9" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="I9" t="str">
-        <v>Black Toner Replacement (Standard Toner)</v>
+        <v>DDR4 4GB RAM Upgrade for Laptop (S/N: K06G00013812690D7C - Invoice 1641)</v>
       </c>
       <c r="J9">
-        <v>2200</v>
+        <v>7000</v>
       </c>
       <c r="K9" t="str">
         <v>Company Cheque</v>
@@ -1809,27 +1809,27 @@
         <v>INV-0005</v>
       </c>
       <c r="M9" t="str">
-        <v>ASTA 337/83X TONER</v>
+        <v>kalpana laptop (4gb ram) DDR4 4GB RAM - One Year Warranty</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>EXP-0005</v>
+        <v>EXP-0006</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-07-01</v>
+        <v>2026-08-14</v>
       </c>
       <c r="C10" t="str">
         <v>Consumable / Toner</v>
       </c>
       <c r="D10" t="str">
-        <v>AST-0063</v>
+        <v>AST-0060</v>
       </c>
       <c r="E10" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>AST-0063</v>
+        <v>AST-0060</v>
       </c>
       <c r="G10" t="str">
         <v>DEP-0002</v>
@@ -1838,24 +1838,24 @@
         <v>KMN IT Solution</v>
       </c>
       <c r="I10" t="str">
-        <v>Color Toner Replacement (Standard Toner)</v>
+        <v>Black Toner Replacement (Standard Toner)</v>
       </c>
       <c r="J10">
-        <v>2850</v>
+        <v>2200</v>
       </c>
       <c r="K10" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L10" t="str">
-        <v>INV-0004</v>
+        <v>INV-0005</v>
       </c>
       <c r="M10" t="str">
-        <v/>
+        <v>ASTA 337/83X TONER</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>EXP-0004</v>
+        <v>EXP-0005</v>
       </c>
       <c r="B11" t="str">
         <v>2026-07-01</v>
@@ -1879,10 +1879,10 @@
         <v>KMN IT Solution</v>
       </c>
       <c r="I11" t="str">
-        <v>Black Toner Replacement (Standard Toner)</v>
+        <v>Color Toner Replacement (Standard Toner)</v>
       </c>
       <c r="J11">
-        <v>2800</v>
+        <v>2850</v>
       </c>
       <c r="K11" t="str">
         <v>Company Cheque</v>
@@ -1896,40 +1896,40 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>EXP-0003</v>
+        <v>EXP-0004</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-09-07</v>
+        <v>2026-07-01</v>
       </c>
       <c r="C12" t="str">
-        <v>Repair</v>
+        <v>Consumable / Toner</v>
       </c>
       <c r="D12" t="str">
-        <v>AST-0052</v>
+        <v>AST-0063</v>
       </c>
       <c r="E12" t="str">
-        <v>USR-0014</v>
+        <v/>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>AST-0063</v>
       </c>
       <c r="G12" t="str">
-        <v>DEP-0004</v>
+        <v>DEP-0002</v>
       </c>
       <c r="H12" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="I12" t="str">
-        <v>Repair for Desktop PC Workstation: HAVEN'T A MOUSE</v>
+        <v>Black Toner Replacement (Standard Toner)</v>
       </c>
       <c r="J12">
-        <v>1000</v>
+        <v>2800</v>
       </c>
       <c r="K12" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L12" t="str">
-        <v>INV-0003</v>
+        <v>INV-0004</v>
       </c>
       <c r="M12" t="str">
         <v/>
@@ -1937,10 +1937,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>EXP-0002</v>
+        <v>EXP-0003</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-07</v>
       </c>
       <c r="C13" t="str">
         <v>Repair</v>
@@ -1961,16 +1961,16 @@
         <v>KMN IT Solution</v>
       </c>
       <c r="I13" t="str">
-        <v>Repair for Desktop PC Workstation: STUCK &amp; SLOW (2 parts replaced)</v>
+        <v>Repair for Desktop PC Workstation: HAVEN'T A MOUSE</v>
       </c>
       <c r="J13">
-        <v>30000</v>
+        <v>1000</v>
       </c>
       <c r="K13" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L13" t="str">
-        <v>INV-0002</v>
+        <v>INV-0003</v>
       </c>
       <c r="M13" t="str">
         <v/>
@@ -1978,19 +1978,19 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>EXP-0001</v>
+        <v>EXP-0002</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-10</v>
       </c>
       <c r="C14" t="str">
         <v>Repair</v>
       </c>
       <c r="D14" t="str">
-        <v>AST-0041</v>
+        <v>AST-0052</v>
       </c>
       <c r="E14" t="str">
-        <v>USR-0010</v>
+        <v>USR-0014</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -2005,28 +2005,69 @@
         <v>Repair for Desktop PC Workstation: STUCK &amp; SLOW (2 parts replaced)</v>
       </c>
       <c r="J14">
-        <v>36000</v>
+        <v>30000</v>
       </c>
       <c r="K14" t="str">
         <v>Company Cheque</v>
       </c>
       <c r="L14" t="str">
+        <v>INV-0002</v>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>EXP-0001</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Repair</v>
+      </c>
+      <c r="D15" t="str">
+        <v>AST-0041</v>
+      </c>
+      <c r="E15" t="str">
+        <v>USR-0010</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v>DEP-0004</v>
+      </c>
+      <c r="H15" t="str">
+        <v>KMN IT Solution</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Repair for Desktop PC Workstation: STUCK &amp; SLOW (2 parts replaced)</v>
+      </c>
+      <c r="J15">
+        <v>36000</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Company Cheque</v>
+      </c>
+      <c r="L15" t="str">
         <v>INV-0001</v>
       </c>
-      <c r="M14" t="str">
+      <c r="M15" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2074,87 +2115,87 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>INV-0007</v>
+        <v>INV-0008</v>
       </c>
       <c r="B2" t="str">
-        <v>kmn_aqua</v>
+        <v>04_08_2026_</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-09-17</v>
+        <v>2026-08-04</v>
       </c>
       <c r="D2" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E2">
-        <v>4800</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="str">
-        <v>AST-0057</v>
+        <v>AST-0052</v>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>AST-0057</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>
       </c>
       <c r="J2" t="str">
-        <v>17.09.26.pdf</v>
+        <v>04.08.2026..pdf</v>
       </c>
       <c r="K2" t="str">
-        <v>/invoices/17.09.26.pdf</v>
+        <v>/invoices/04.08.2026..pdf</v>
       </c>
       <c r="L2" t="str">
         <v>545 KB</v>
       </c>
       <c r="M2" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-23</v>
       </c>
       <c r="N2" t="str">
-        <v>Black Toner for printer</v>
+        <v xml:space="preserve">Invoice for repair/service: Power cable not worked </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>INV-0006</v>
+        <v>INV-0007</v>
       </c>
       <c r="B3" t="str">
-        <v>23_07_2026_</v>
+        <v>kmn_aqua</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-07-23</v>
+        <v>2026-09-17</v>
       </c>
       <c r="D3" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E3">
-        <v>8000</v>
+        <v>4800</v>
       </c>
       <c r="F3" t="str">
-        <v>AST-0059</v>
+        <v>AST-0057</v>
       </c>
       <c r="G3" t="str">
         <v/>
       </c>
       <c r="H3" t="str">
-        <v>AST-0059</v>
+        <v>AST-0057</v>
       </c>
       <c r="I3" t="str">
         <v/>
       </c>
       <c r="J3" t="str">
-        <v>23.07.2026..pdf</v>
+        <v>17.09.26.pdf</v>
       </c>
       <c r="K3" t="str">
-        <v>/invoices/23.07.2026..pdf</v>
+        <v>/invoices/17.09.26.pdf</v>
       </c>
       <c r="L3" t="str">
-        <v>633 KB</v>
+        <v>545 KB</v>
       </c>
       <c r="M3" t="str">
-        <v>2026-07-23</v>
+        <v>2026-09-17</v>
       </c>
       <c r="N3" t="str">
         <v>Black Toner for printer</v>
@@ -2162,69 +2203,69 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>INV-0005</v>
+        <v>INV-0006</v>
       </c>
       <c r="B4" t="str">
-        <v>14.08.2026.</v>
+        <v>23_07_2026_</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-08-14</v>
+        <v>2026-07-23</v>
       </c>
       <c r="D4" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E4">
-        <v>9200</v>
+        <v>8000</v>
       </c>
       <c r="F4" t="str">
-        <v>AST-0060</v>
+        <v>AST-0059</v>
       </c>
       <c r="G4" t="str">
         <v/>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>AST-0059</v>
       </c>
       <c r="I4" t="str">
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>14.08.2026..pdf</v>
+        <v>23.07.2026..pdf</v>
       </c>
       <c r="K4" t="str">
-        <v>/invoices/14.08.2026..pdf</v>
+        <v>/invoices/23.07.2026..pdf</v>
       </c>
       <c r="L4" t="str">
-        <v>641 KB</v>
+        <v>633 KB</v>
       </c>
       <c r="M4" t="str">
-        <v>2026-09-22</v>
+        <v>2026-07-23</v>
       </c>
       <c r="N4" t="str">
-        <v>Uploaded Invoice: 14.08.2026..pdf</v>
+        <v>Black Toner for printer</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>INV-0004</v>
+        <v>INV-0005</v>
       </c>
       <c r="B5" t="str">
-        <v>01.07.2026.</v>
+        <v>14.08.2026.</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-07-01</v>
+        <v>2026-08-14</v>
       </c>
       <c r="D5" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E5">
-        <v>5650</v>
+        <v>9200</v>
       </c>
       <c r="F5" t="str">
-        <v>AST-0063</v>
+        <v>AST-0060</v>
       </c>
       <c r="G5" t="str">
-        <v>USR-0016</v>
+        <v/>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -2233,42 +2274,42 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>01.07.2026..pdf</v>
+        <v>14.08.2026..pdf</v>
       </c>
       <c r="K5" t="str">
-        <v>/invoices/01.07.2026..pdf</v>
+        <v>/invoices/14.08.2026..pdf</v>
       </c>
       <c r="L5" t="str">
-        <v>494 KB</v>
+        <v>641 KB</v>
       </c>
       <c r="M5" t="str">
         <v>2026-09-22</v>
       </c>
       <c r="N5" t="str">
-        <v>ADD TO TONNER 680 BLACK AND COLOUR</v>
+        <v>Uploaded Invoice: 14.08.2026..pdf</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>INV-0003</v>
+        <v>INV-0004</v>
       </c>
       <c r="B6" t="str">
-        <v>07_09_2026_</v>
+        <v>01.07.2026.</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-09-07</v>
+        <v>2026-07-01</v>
       </c>
       <c r="D6" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E6">
-        <v>1000</v>
+        <v>5650</v>
       </c>
       <c r="F6" t="str">
-        <v>AST-0052</v>
+        <v>AST-0063</v>
       </c>
       <c r="G6" t="str">
-        <v/>
+        <v>USR-0016</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -2277,36 +2318,36 @@
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>07.09.2026..pdf</v>
+        <v>01.07.2026..pdf</v>
       </c>
       <c r="K6" t="str">
-        <v>/invoices/07.09.2026..pdf</v>
+        <v>/invoices/01.07.2026..pdf</v>
       </c>
       <c r="L6" t="str">
-        <v>638 KB</v>
+        <v>494 KB</v>
       </c>
       <c r="M6" t="str">
         <v>2026-09-22</v>
       </c>
       <c r="N6" t="str">
-        <v>Invoice for repair/service: HAVEN'T A MOUSE</v>
+        <v>ADD TO TONNER 680 BLACK AND COLOUR</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>INV-0002</v>
+        <v>INV-0003</v>
       </c>
       <c r="B7" t="str">
-        <v>10_09_2026_</v>
+        <v>07_09_2026_</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-07</v>
       </c>
       <c r="D7" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E7">
-        <v>30000</v>
+        <v>1000</v>
       </c>
       <c r="F7" t="str">
         <v>AST-0052</v>
@@ -2321,39 +2362,39 @@
         <v/>
       </c>
       <c r="J7" t="str">
-        <v>10.09.2026..pdf</v>
+        <v>07.09.2026..pdf</v>
       </c>
       <c r="K7" t="str">
-        <v>/invoices/10.09.2026..pdf</v>
+        <v>/invoices/07.09.2026..pdf</v>
       </c>
       <c r="L7" t="str">
-        <v>633 KB</v>
+        <v>638 KB</v>
       </c>
       <c r="M7" t="str">
         <v>2026-09-22</v>
       </c>
       <c r="N7" t="str">
-        <v>Invoice for repair/service: STUCK &amp; SLOW</v>
+        <v>Invoice for repair/service: HAVEN'T A MOUSE</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>INV-0001</v>
+        <v>INV-0002</v>
       </c>
       <c r="B8" t="str">
-        <v>05_09_2026_</v>
+        <v>10_09_2026_</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-10</v>
       </c>
       <c r="D8" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E8">
-        <v>36000</v>
+        <v>30000</v>
       </c>
       <c r="F8" t="str">
-        <v>AST-0041</v>
+        <v>AST-0052</v>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -2365,13 +2406,13 @@
         <v/>
       </c>
       <c r="J8" t="str">
-        <v>05.09.2026..pdf</v>
+        <v>10.09.2026..pdf</v>
       </c>
       <c r="K8" t="str">
-        <v>/invoices/05.09.2026..pdf</v>
+        <v>/invoices/10.09.2026..pdf</v>
       </c>
       <c r="L8" t="str">
-        <v>639 KB</v>
+        <v>633 KB</v>
       </c>
       <c r="M8" t="str">
         <v>2026-09-22</v>
@@ -2380,9 +2421,53 @@
         <v>Invoice for repair/service: STUCK &amp; SLOW</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>INV-0001</v>
+      </c>
+      <c r="B9" t="str">
+        <v>05_09_2026_</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="D9" t="str">
+        <v>KMN IT Solution</v>
+      </c>
+      <c r="E9">
+        <v>36000</v>
+      </c>
+      <c r="F9" t="str">
+        <v>AST-0041</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v>05.09.2026..pdf</v>
+      </c>
+      <c r="K9" t="str">
+        <v>/invoices/05.09.2026..pdf</v>
+      </c>
+      <c r="L9" t="str">
+        <v>639 KB</v>
+      </c>
+      <c r="M9" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Invoice for repair/service: STUCK &amp; SLOW</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3472,7 +3557,7 @@
         <v>LOC-0001</v>
       </c>
       <c r="N12" t="str">
-        <v>[⚠️ Warning Logged 2026-09-10: S] [⚠️ Warning Logged 2026-09-07: G]</v>
+        <v>[⚠️ Warning Logged 2026-09-10: S] [⚠️ Warning Logged 2026-09-07: G] [⚠️ Warning Logged 2026-08-04: p]</v>
       </c>
       <c r="O12" t="str">
         <v>AST-0052</v>
@@ -3481,10 +3566,10 @@
         <v>Warning</v>
       </c>
       <c r="Q12" t="str">
-        <v>G</v>
+        <v>p</v>
       </c>
       <c r="R12" t="str">
-        <v>2026-09-07</v>
+        <v>2026-08-04</v>
       </c>
     </row>
     <row r="13">
@@ -6529,7 +6614,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:Q6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6586,25 +6671,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>REP-0004</v>
+        <v>REP-0005</v>
       </c>
       <c r="B2" t="str">
         <v>AST-0052</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-09-07</v>
+        <v>2026-08-04</v>
       </c>
       <c r="D2" t="str">
-        <v>HAVEN'T A MOUSE</v>
+        <v xml:space="preserve">Power cable not worked </v>
       </c>
       <c r="E2" t="str">
-        <v>HAVEN'T A MOUSE</v>
+        <v xml:space="preserve">Power cable not worked </v>
       </c>
       <c r="F2" t="str">
-        <v>GIVE NEW ONE</v>
+        <v>Anjitha</v>
       </c>
       <c r="G2" t="str">
-        <v>Keyboard &amp; Mouse: Standard USB Mouse</v>
+        <v>N/A</v>
       </c>
       <c r="H2" t="str">
         <v>KMN IT Solution</v>
@@ -6622,16 +6707,16 @@
         <v>Completed</v>
       </c>
       <c r="M2" t="str">
-        <v>2026-09-22</v>
+        <v>2026-09-23</v>
       </c>
       <c r="N2" t="str">
-        <v>2026-09-07</v>
+        <v>2026-08-04</v>
       </c>
       <c r="O2" t="str">
         <v/>
       </c>
       <c r="P2" t="str">
-        <v>INV-0003</v>
+        <v>INV-0008</v>
       </c>
       <c r="Q2" t="str">
         <v/>
@@ -6639,25 +6724,25 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>REP-0003</v>
+        <v>REP-0004</v>
       </c>
       <c r="B3" t="str">
         <v>AST-0052</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-07</v>
       </c>
       <c r="D3" t="str">
-        <v>STUCK &amp; SLOW</v>
+        <v>HAVEN'T A MOUSE</v>
       </c>
       <c r="E3" t="str">
-        <v>STUCK &amp; SLOW</v>
+        <v>HAVEN'T A MOUSE</v>
       </c>
       <c r="F3" t="str">
-        <v>ADD NEW PARTS</v>
+        <v>GIVE NEW ONE</v>
       </c>
       <c r="G3" t="str">
-        <v>RAM: 4 GB; Storage / SSD: 256 GB</v>
+        <v>Keyboard &amp; Mouse: Standard USB Mouse</v>
       </c>
       <c r="H3" t="str">
         <v>KMN IT Solution</v>
@@ -6666,7 +6751,7 @@
         <v>KMN IT Service Specialist</v>
       </c>
       <c r="J3">
-        <v>30000</v>
+        <v>1000</v>
       </c>
       <c r="K3" t="str">
         <v>Yes</v>
@@ -6675,16 +6760,16 @@
         <v>Completed</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>2026-09-22</v>
       </c>
       <c r="N3" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-07</v>
       </c>
       <c r="O3" t="str">
         <v/>
       </c>
       <c r="P3" t="str">
-        <v>INV-0002</v>
+        <v>INV-0003</v>
       </c>
       <c r="Q3" t="str">
         <v/>
@@ -6692,13 +6777,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>REP-0002</v>
+        <v>REP-0003</v>
       </c>
       <c r="B4" t="str">
-        <v>AST-0041</v>
+        <v>AST-0052</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-10</v>
       </c>
       <c r="D4" t="str">
         <v>STUCK &amp; SLOW</v>
@@ -6710,7 +6795,7 @@
         <v>ADD NEW PARTS</v>
       </c>
       <c r="G4" t="str">
-        <v>RAM: 4GB DDR4; Storage / SSD: 256 GB</v>
+        <v>RAM: 4 GB; Storage / SSD: 256 GB</v>
       </c>
       <c r="H4" t="str">
         <v>KMN IT Solution</v>
@@ -6719,7 +6804,7 @@
         <v>KMN IT Service Specialist</v>
       </c>
       <c r="J4">
-        <v>36000</v>
+        <v>30000</v>
       </c>
       <c r="K4" t="str">
         <v>Yes</v>
@@ -6728,16 +6813,16 @@
         <v>Completed</v>
       </c>
       <c r="M4" t="str">
-        <v>2026-09-22</v>
+        <v/>
       </c>
       <c r="N4" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-10</v>
       </c>
       <c r="O4" t="str">
         <v/>
       </c>
       <c r="P4" t="str">
-        <v>INV-0001</v>
+        <v>INV-0002</v>
       </c>
       <c r="Q4" t="str">
         <v/>
@@ -6745,25 +6830,25 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>REP-0001</v>
+        <v>REP-0002</v>
       </c>
       <c r="B5" t="str">
-        <v>AST-0048</v>
+        <v>AST-0041</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-08</v>
       </c>
       <c r="D5" t="str">
-        <v>UPS GIVE SOME BEEP SOUND</v>
+        <v>STUCK &amp; SLOW</v>
       </c>
       <c r="E5" t="str">
-        <v>UPS GIVE SOME BEEP SOUND</v>
+        <v>STUCK &amp; SLOW</v>
       </c>
       <c r="F5" t="str">
-        <v>CHECKED BUY YOHAN</v>
+        <v>ADD NEW PARTS</v>
       </c>
       <c r="G5" t="str">
-        <v>N/A</v>
+        <v>RAM: 4GB DDR4; Storage / SSD: 256 GB</v>
       </c>
       <c r="H5" t="str">
         <v>KMN IT Solution</v>
@@ -6772,33 +6857,86 @@
         <v>KMN IT Service Specialist</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>36000</v>
       </c>
       <c r="K5" t="str">
         <v>Yes</v>
       </c>
       <c r="L5" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M5" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="N5" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v>INV-0001</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>REP-0001</v>
+      </c>
+      <c r="B6" t="str">
+        <v>AST-0048</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-09-05</v>
+      </c>
+      <c r="D6" t="str">
+        <v>UPS GIVE SOME BEEP SOUND</v>
+      </c>
+      <c r="E6" t="str">
+        <v>UPS GIVE SOME BEEP SOUND</v>
+      </c>
+      <c r="F6" t="str">
+        <v>CHECKED BUY YOHAN</v>
+      </c>
+      <c r="G6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H6" t="str">
+        <v>KMN IT Solution</v>
+      </c>
+      <c r="I6" t="str">
+        <v>KMN IT Service Specialist</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L6" t="str">
         <v>Warning / Under Observation</v>
       </c>
-      <c r="M5" t="str">
-        <v/>
-      </c>
-      <c r="N5" t="str">
-        <v>2026-09-21</v>
-      </c>
-      <c r="O5" t="str">
-        <v/>
-      </c>
-      <c r="P5" t="str">
-        <v/>
-      </c>
-      <c r="Q5" t="str">
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
         <v xml:space="preserve">THIS IS AUTO FIXED BUT NEAD TO CHECK </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add relational database repository, Excel file synchronization, and assignment management UI
</commit_message>
<xml_diff>
--- a/database/IT_Asset_Database.xlsx
+++ b/database/IT_Asset_Database.xlsx
@@ -2988,7 +2988,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R63"/>
+  <dimension ref="A1:R64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3048,16 +3048,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>KMN/CH/CP/024</v>
       </c>
       <c r="B2" t="str">
-        <v>Printer</v>
+        <v>Desktop</v>
       </c>
       <c r="C2" t="str">
-        <v>HP</v>
+        <v>Dell</v>
       </c>
       <c r="D2" t="str">
-        <v>DeskJet Link Advantage 3835</v>
+        <v>N/A</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -3066,13 +3066,13 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2026-09-22</v>
+        <v>2026-09-23</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-09-22</v>
+        <v>2026-09-23</v>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -3081,7 +3081,7 @@
         <v>Assigned</v>
       </c>
       <c r="L2" t="str">
-        <v>USR-0016</v>
+        <v>USR-0002</v>
       </c>
       <c r="M2" t="str">
         <v>LOC-0001</v>
@@ -3090,21 +3090,21 @@
         <v/>
       </c>
       <c r="O2" t="str">
-        <v>AST-0063</v>
+        <v>AST-0064</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>KMN/CH/CP/061</v>
+        <v/>
       </c>
       <c r="B3" t="str">
-        <v>Mouse</v>
+        <v>Printer</v>
       </c>
       <c r="C3" t="str">
-        <v>Standard</v>
+        <v>HP</v>
       </c>
       <c r="D3" t="str">
-        <v>Optical USB Mouse</v>
+        <v>DeskJet Link Advantage 3835</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -3137,21 +3137,21 @@
         <v/>
       </c>
       <c r="O3" t="str">
-        <v>AST-0062</v>
+        <v>AST-0063</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>KMN/CH/CP/037</v>
+        <v>KMN/CH/CP/061</v>
       </c>
       <c r="B4" t="str">
-        <v>Laptop</v>
+        <v>Mouse</v>
       </c>
       <c r="C4" t="str">
-        <v>Dell</v>
+        <v>Standard</v>
       </c>
       <c r="D4" t="str">
-        <v>Business Laptop</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -3184,21 +3184,21 @@
         <v/>
       </c>
       <c r="O4" t="str">
-        <v>AST-0061</v>
+        <v>AST-0062</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>KMN/CH/CP/005</v>
+        <v>KMN/CH/CP/037</v>
       </c>
       <c r="B5" t="str">
-        <v>Printer</v>
+        <v>Laptop</v>
       </c>
       <c r="C5" t="str">
-        <v>CANON</v>
+        <v>Dell</v>
       </c>
       <c r="D5" t="str">
-        <v>IMAGE CLASS MF249DW</v>
+        <v>Business Laptop</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -3219,10 +3219,10 @@
         <v/>
       </c>
       <c r="K5" t="str">
-        <v>Shared / Networked</v>
+        <v>Assigned</v>
       </c>
       <c r="L5" t="str">
-        <v>SHARED_NETWORK</v>
+        <v>USR-0016</v>
       </c>
       <c r="M5" t="str">
         <v>LOC-0001</v>
@@ -3231,12 +3231,12 @@
         <v/>
       </c>
       <c r="O5" t="str">
-        <v>AST-0060</v>
+        <v>AST-0061</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>KMN/CH/CP/005</v>
       </c>
       <c r="B6" t="str">
         <v>Printer</v>
@@ -3245,7 +3245,7 @@
         <v>CANON</v>
       </c>
       <c r="D6" t="str">
-        <v>IMAGE RUNNER 2006</v>
+        <v>IMAGE CLASS MF249DW</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -3278,115 +3278,115 @@
         <v/>
       </c>
       <c r="O6" t="str">
-        <v>AST-0059</v>
+        <v>AST-0060</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KMN/CH/CP/069</v>
+        <v/>
       </c>
       <c r="B7" t="str">
-        <v>Mouse</v>
+        <v>Printer</v>
       </c>
       <c r="C7" t="str">
-        <v>Standard</v>
+        <v>CANON</v>
       </c>
       <c r="D7" t="str">
-        <v>Optical USB Mouse</v>
+        <v>IMAGE RUNNER 2006</v>
       </c>
       <c r="E7" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>Standard Optical USB Mouse</v>
+        <v/>
       </c>
       <c r="G7" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-22</v>
       </c>
       <c r="H7">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I7" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-22</v>
       </c>
       <c r="J7" t="str">
-        <v>2027-09-07</v>
+        <v/>
       </c>
       <c r="K7" t="str">
-        <v>Assigned</v>
+        <v>Shared / Networked</v>
       </c>
       <c r="L7" t="str">
-        <v>USR-0014</v>
+        <v>SHARED_NETWORK</v>
       </c>
       <c r="M7" t="str">
         <v>LOC-0001</v>
       </c>
       <c r="N7" t="str">
-        <v>Issued during service REP-0004: HAVEN'T A MOUSE [Warranty: 1 Year]</v>
+        <v/>
       </c>
       <c r="O7" t="str">
-        <v>AST-0058</v>
+        <v>AST-0059</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>KMN/CH/CP/069</v>
       </c>
       <c r="B8" t="str">
-        <v>Printer</v>
+        <v>Mouse</v>
       </c>
       <c r="C8" t="str">
-        <v>CANON</v>
+        <v>Standard</v>
       </c>
       <c r="D8" t="str">
-        <v>MF645C ufr ii</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E8" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>Standard Optical USB Mouse</v>
       </c>
       <c r="G8" t="str">
-        <v>2026-09-21</v>
+        <v>2026-09-07</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I8" t="str">
-        <v>2026-09-21</v>
+        <v>2026-09-07</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>2027-09-07</v>
       </c>
       <c r="K8" t="str">
         <v>Assigned</v>
       </c>
       <c r="L8" t="str">
-        <v>USR-0008</v>
+        <v>USR-0014</v>
       </c>
       <c r="M8" t="str">
         <v>LOC-0001</v>
       </c>
       <c r="N8" t="str">
-        <v xml:space="preserve"> [Shared Network Office Printer]</v>
+        <v>Issued during service REP-0004: HAVEN'T A MOUSE [Warranty: 1 Year]</v>
       </c>
       <c r="O8" t="str">
-        <v>AST-0057</v>
+        <v>AST-0058</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>KMN/CH/CP/016</v>
+        <v/>
       </c>
       <c r="B9" t="str">
-        <v>Laptop</v>
+        <v>Printer</v>
       </c>
       <c r="C9" t="str">
-        <v>Dell</v>
+        <v>CANON</v>
       </c>
       <c r="D9" t="str">
-        <v>Business Laptop</v>
+        <v>MF645C ufr ii</v>
       </c>
       <c r="E9" t="str">
         <v/>
@@ -3410,30 +3410,30 @@
         <v>Assigned</v>
       </c>
       <c r="L9" t="str">
-        <v>USR-0015</v>
+        <v>USR-0008</v>
       </c>
       <c r="M9" t="str">
         <v>LOC-0001</v>
       </c>
       <c r="N9" t="str">
-        <v/>
+        <v xml:space="preserve"> [Shared Network Office Printer]</v>
       </c>
       <c r="O9" t="str">
-        <v>AST-0056</v>
+        <v>AST-0057</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>KMN/CH/CP/068</v>
+        <v>KMN/CH/CP/016</v>
       </c>
       <c r="B10" t="str">
-        <v>Mouse</v>
+        <v>Laptop</v>
       </c>
       <c r="C10" t="str">
-        <v>Standard</v>
+        <v>Dell</v>
       </c>
       <c r="D10" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Business Laptop</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -3466,21 +3466,21 @@
         <v/>
       </c>
       <c r="O10" t="str">
-        <v>AST-0055</v>
+        <v>AST-0056</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>KMN/CH/CP/022</v>
+        <v>KMN/CH/CP/068</v>
       </c>
       <c r="B11" t="str">
-        <v>Keyboard</v>
+        <v>Mouse</v>
       </c>
       <c r="C11" t="str">
-        <v>Dell</v>
+        <v>Standard</v>
       </c>
       <c r="D11" t="str">
-        <v>Standard Keyboard</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -3504,7 +3504,7 @@
         <v>Assigned</v>
       </c>
       <c r="L11" t="str">
-        <v>USR-0014</v>
+        <v>USR-0015</v>
       </c>
       <c r="M11" t="str">
         <v>LOC-0001</v>
@@ -3513,21 +3513,21 @@
         <v/>
       </c>
       <c r="O11" t="str">
-        <v>AST-0053</v>
+        <v>AST-0055</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>KMN/CH/CP/068</v>
+        <v>KMN/CH/CP/022</v>
       </c>
       <c r="B12" t="str">
-        <v>Desktop</v>
+        <v>Keyboard</v>
       </c>
       <c r="C12" t="str">
         <v>Dell</v>
       </c>
       <c r="D12" t="str">
-        <v>Desktop PC Workstation</v>
+        <v>Standard Keyboard</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -3557,33 +3557,24 @@
         <v>LOC-0001</v>
       </c>
       <c r="N12" t="str">
-        <v>[⚠️ Warning Logged 2026-09-10: S] [⚠️ Warning Logged 2026-09-07: G] [⚠️ Warning Logged 2026-08-04: p]</v>
+        <v/>
       </c>
       <c r="O12" t="str">
-        <v>AST-0052</v>
-      </c>
-      <c r="P12" t="str">
-        <v>Warning</v>
-      </c>
-      <c r="Q12" t="str">
-        <v>p</v>
-      </c>
-      <c r="R12" t="str">
-        <v>2026-08-04</v>
+        <v>AST-0053</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v/>
+        <v>KMN/CH/CP/068</v>
       </c>
       <c r="B13" t="str">
-        <v>UPS</v>
+        <v>Desktop</v>
       </c>
       <c r="C13" t="str">
-        <v>Office Standard</v>
+        <v>Dell</v>
       </c>
       <c r="D13" t="str">
-        <v>Office UPS Backup Unit</v>
+        <v>Desktop PC Workstation</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -3613,24 +3604,33 @@
         <v>LOC-0001</v>
       </c>
       <c r="N13" t="str">
-        <v/>
+        <v>[⚠️ Warning Logged 2026-09-10: S] [⚠️ Warning Logged 2026-09-07: G] [⚠️ Warning Logged 2026-08-04: p]</v>
       </c>
       <c r="O13" t="str">
-        <v>AST-0051</v>
+        <v>AST-0052</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Warning</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>p</v>
+      </c>
+      <c r="R13" t="str">
+        <v>2026-08-04</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>GAP/ATT/LE/001</v>
+        <v/>
       </c>
       <c r="B14" t="str">
-        <v>Lab Equipment</v>
+        <v>UPS</v>
       </c>
       <c r="C14" t="str">
-        <v>BRUKER</v>
+        <v>Office Standard</v>
       </c>
       <c r="D14" t="str">
-        <v>Laboratory Testing Machine</v>
+        <v>Office UPS Backup Unit</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -3654,7 +3654,7 @@
         <v>Assigned</v>
       </c>
       <c r="L14" t="str">
-        <v>USR-0013</v>
+        <v>USR-0014</v>
       </c>
       <c r="M14" t="str">
         <v>LOC-0001</v>
@@ -3663,21 +3663,21 @@
         <v/>
       </c>
       <c r="O14" t="str">
-        <v>AST-0050</v>
+        <v>AST-0051</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GAP/ATT/CP/011</v>
+        <v>GAP/ATT/LE/001</v>
       </c>
       <c r="B15" t="str">
-        <v>Laptop</v>
+        <v>Lab Equipment</v>
       </c>
       <c r="C15" t="str">
-        <v>Generic</v>
+        <v>BRUKER</v>
       </c>
       <c r="D15" t="str">
-        <v>Business Laptop</v>
+        <v>Laboratory Testing Machine</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -3707,24 +3707,24 @@
         <v>LOC-0001</v>
       </c>
       <c r="N15" t="str">
-        <v>NIR MACHINE LAPTOP</v>
+        <v/>
       </c>
       <c r="O15" t="str">
-        <v>AST-0049</v>
+        <v>AST-0050</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>GAP/ATT/CP/012</v>
+        <v>GAP/ATT/CP/011</v>
       </c>
       <c r="B16" t="str">
-        <v>UPS</v>
+        <v>Laptop</v>
       </c>
       <c r="C16" t="str">
-        <v>Office Standard</v>
+        <v>Generic</v>
       </c>
       <c r="D16" t="str">
-        <v>Office UPS Backup (GAP/ATT/CP/012)</v>
+        <v>Business Laptop</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -3754,24 +3754,24 @@
         <v>LOC-0001</v>
       </c>
       <c r="N16" t="str">
-        <v/>
+        <v>NIR MACHINE LAPTOP</v>
       </c>
       <c r="O16" t="str">
-        <v>AST-0048</v>
+        <v>AST-0049</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>KMN/CH/CP/041</v>
+        <v>GAP/ATT/CP/012</v>
       </c>
       <c r="B17" t="str">
-        <v>Mouse</v>
+        <v>UPS</v>
       </c>
       <c r="C17" t="str">
-        <v>Standard</v>
+        <v>Office Standard</v>
       </c>
       <c r="D17" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Office UPS Backup (GAP/ATT/CP/012)</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -3792,10 +3792,10 @@
         <v/>
       </c>
       <c r="K17" t="str">
-        <v>Available</v>
+        <v>Assigned</v>
       </c>
       <c r="L17" t="str">
-        <v/>
+        <v>USR-0013</v>
       </c>
       <c r="M17" t="str">
         <v>LOC-0001</v>
@@ -3804,21 +3804,21 @@
         <v/>
       </c>
       <c r="O17" t="str">
-        <v>AST-0047</v>
+        <v>AST-0048</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v/>
+        <v>KMN/CH/CP/041</v>
       </c>
       <c r="B18" t="str">
-        <v>Laptop</v>
+        <v>Mouse</v>
       </c>
       <c r="C18" t="str">
-        <v>Dell</v>
+        <v>Standard</v>
       </c>
       <c r="D18" t="str">
-        <v>INSPIRON 3502</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -3851,7 +3851,7 @@
         <v/>
       </c>
       <c r="O18" t="str">
-        <v>AST-0046</v>
+        <v>AST-0047</v>
       </c>
     </row>
     <row r="19">
@@ -3859,13 +3859,13 @@
         <v/>
       </c>
       <c r="B19" t="str">
-        <v>Mouse</v>
+        <v>Laptop</v>
       </c>
       <c r="C19" t="str">
-        <v>Standard</v>
+        <v>Dell</v>
       </c>
       <c r="D19" t="str">
-        <v>Optical USB Mouse</v>
+        <v>INSPIRON 3502</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -3886,10 +3886,10 @@
         <v/>
       </c>
       <c r="K19" t="str">
-        <v>Assigned</v>
+        <v>Available</v>
       </c>
       <c r="L19" t="str">
-        <v>USR-0011</v>
+        <v/>
       </c>
       <c r="M19" t="str">
         <v>LOC-0001</v>
@@ -3898,7 +3898,7 @@
         <v/>
       </c>
       <c r="O19" t="str">
-        <v>AST-0045</v>
+        <v>AST-0046</v>
       </c>
     </row>
     <row r="20">
@@ -3906,13 +3906,13 @@
         <v/>
       </c>
       <c r="B20" t="str">
-        <v>Laptop</v>
+        <v>Mouse</v>
       </c>
       <c r="C20" t="str">
-        <v>Dell</v>
+        <v>Standard</v>
       </c>
       <c r="D20" t="str">
-        <v>Business Laptop</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -3945,21 +3945,21 @@
         <v/>
       </c>
       <c r="O20" t="str">
-        <v>AST-0044</v>
+        <v>AST-0045</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>KMN/CH/CP/013</v>
+        <v/>
       </c>
       <c r="B21" t="str">
-        <v>UPS</v>
+        <v>Laptop</v>
       </c>
       <c r="C21" t="str">
-        <v>Office Standard</v>
+        <v>Dell</v>
       </c>
       <c r="D21" t="str">
-        <v>Office UPS Backup (KMN/CH/CP/013)</v>
+        <v>Business Laptop</v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -3983,7 +3983,7 @@
         <v>Assigned</v>
       </c>
       <c r="L21" t="str">
-        <v>USR-0010</v>
+        <v>USR-0011</v>
       </c>
       <c r="M21" t="str">
         <v>LOC-0001</v>
@@ -3992,21 +3992,21 @@
         <v/>
       </c>
       <c r="O21" t="str">
-        <v>AST-0043</v>
+        <v>AST-0044</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>KMN/CH/CP/013</v>
       </c>
       <c r="B22" t="str">
-        <v>Mouse</v>
+        <v>UPS</v>
       </c>
       <c r="C22" t="str">
-        <v>AOC</v>
+        <v>Office Standard</v>
       </c>
       <c r="D22" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Office UPS Backup (KMN/CH/CP/013)</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -4039,21 +4039,21 @@
         <v/>
       </c>
       <c r="O22" t="str">
-        <v>AST-0042</v>
+        <v>AST-0043</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>KMN/CH/CP/051</v>
+        <v/>
       </c>
       <c r="B23" t="str">
-        <v>Desktop</v>
+        <v>Mouse</v>
       </c>
       <c r="C23" t="str">
-        <v>Dell</v>
+        <v>AOC</v>
       </c>
       <c r="D23" t="str">
-        <v>Desktop PC Workstation</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E23" t="str">
         <v/>
@@ -4083,33 +4083,24 @@
         <v>LOC-0001</v>
       </c>
       <c r="N23" t="str">
-        <v>[⚠️ Warning Logged 2026-09-05: s] [⚠️ Warning Logged 2026-09-08: S]</v>
+        <v/>
       </c>
       <c r="O23" t="str">
-        <v>AST-0041</v>
-      </c>
-      <c r="P23" t="str">
-        <v>Warning</v>
-      </c>
-      <c r="Q23" t="str">
-        <v>S</v>
-      </c>
-      <c r="R23" t="str">
-        <v>2026-09-08</v>
+        <v>AST-0042</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>KMN/CH/CP/050</v>
+        <v>KMN/CH/CP/051</v>
       </c>
       <c r="B24" t="str">
-        <v>Keyboard</v>
+        <v>Desktop</v>
       </c>
       <c r="C24" t="str">
         <v>Dell</v>
       </c>
       <c r="D24" t="str">
-        <v>Standard Keyboard</v>
+        <v>Desktop PC Workstation</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -4139,24 +4130,33 @@
         <v>LOC-0001</v>
       </c>
       <c r="N24" t="str">
-        <v/>
+        <v>[⚠️ Warning Logged 2026-09-05: s] [⚠️ Warning Logged 2026-09-08: S]</v>
       </c>
       <c r="O24" t="str">
-        <v>AST-0040</v>
+        <v>AST-0041</v>
+      </c>
+      <c r="P24" t="str">
+        <v>Warning</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>S</v>
+      </c>
+      <c r="R24" t="str">
+        <v>2026-09-08</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>KMN/CH/CP054</v>
+        <v>KMN/CH/CP/050</v>
       </c>
       <c r="B25" t="str">
-        <v>Monitor</v>
+        <v>Keyboard</v>
       </c>
       <c r="C25" t="str">
         <v>Dell</v>
       </c>
       <c r="D25" t="str">
-        <v>Display Monitor</v>
+        <v>Standard Keyboard</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -4189,21 +4189,21 @@
         <v/>
       </c>
       <c r="O25" t="str">
-        <v>AST-0039</v>
+        <v>AST-0040</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>KMN/CH/CP/018</v>
+        <v>KMN/CH/CP054</v>
       </c>
       <c r="B26" t="str">
-        <v>UPS</v>
+        <v>Monitor</v>
       </c>
       <c r="C26" t="str">
-        <v>Office Standard</v>
+        <v>Dell</v>
       </c>
       <c r="D26" t="str">
-        <v>Office UPS Backup (KMN/CH/CP/018)</v>
+        <v>Display Monitor</v>
       </c>
       <c r="E26" t="str">
         <v/>
@@ -4227,7 +4227,7 @@
         <v>Assigned</v>
       </c>
       <c r="L26" t="str">
-        <v>USR-0009</v>
+        <v>USR-0010</v>
       </c>
       <c r="M26" t="str">
         <v>LOC-0001</v>
@@ -4236,21 +4236,21 @@
         <v/>
       </c>
       <c r="O26" t="str">
-        <v>AST-0038</v>
+        <v>AST-0039</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v/>
+        <v>KMN/CH/CP/018</v>
       </c>
       <c r="B27" t="str">
-        <v>Desktop</v>
+        <v>UPS</v>
       </c>
       <c r="C27" t="str">
-        <v>Generic</v>
+        <v>Office Standard</v>
       </c>
       <c r="D27" t="str">
-        <v>Desktop PC Workstation</v>
+        <v>Office UPS Backup (KMN/CH/CP/018)</v>
       </c>
       <c r="E27" t="str">
         <v/>
@@ -4283,7 +4283,7 @@
         <v/>
       </c>
       <c r="O27" t="str">
-        <v>AST-0037</v>
+        <v>AST-0038</v>
       </c>
     </row>
     <row r="28">
@@ -4291,13 +4291,13 @@
         <v/>
       </c>
       <c r="B28" t="str">
-        <v>Keyboard</v>
+        <v>Desktop</v>
       </c>
       <c r="C28" t="str">
-        <v>Standard</v>
+        <v>Generic</v>
       </c>
       <c r="D28" t="str">
-        <v>Keyboard</v>
+        <v>Desktop PC Workstation</v>
       </c>
       <c r="E28" t="str">
         <v/>
@@ -4330,7 +4330,7 @@
         <v/>
       </c>
       <c r="O28" t="str">
-        <v>AST-0036</v>
+        <v>AST-0037</v>
       </c>
     </row>
     <row r="29">
@@ -4338,13 +4338,13 @@
         <v/>
       </c>
       <c r="B29" t="str">
-        <v>Monitor</v>
+        <v>Keyboard</v>
       </c>
       <c r="C29" t="str">
-        <v>ASUS</v>
+        <v>Standard</v>
       </c>
       <c r="D29" t="str">
-        <v>Display Monitor</v>
+        <v>Keyboard</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -4377,21 +4377,21 @@
         <v/>
       </c>
       <c r="O29" t="str">
-        <v>AST-0035</v>
+        <v>AST-0036</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>KMN/CH/CP/032</v>
+        <v/>
       </c>
       <c r="B30" t="str">
-        <v>UPS</v>
+        <v>Monitor</v>
       </c>
       <c r="C30" t="str">
-        <v>Office Standard</v>
+        <v>ASUS</v>
       </c>
       <c r="D30" t="str">
-        <v>Office UPS Backup (KMN/CH/CP/032)</v>
+        <v>Display Monitor</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -4415,7 +4415,7 @@
         <v>Assigned</v>
       </c>
       <c r="L30" t="str">
-        <v>USR-0008</v>
+        <v>USR-0009</v>
       </c>
       <c r="M30" t="str">
         <v>LOC-0001</v>
@@ -4424,21 +4424,21 @@
         <v/>
       </c>
       <c r="O30" t="str">
-        <v>AST-0034</v>
+        <v>AST-0035</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v>KMN/CH/CP/032</v>
       </c>
       <c r="B31" t="str">
-        <v>Monitor</v>
+        <v>UPS</v>
       </c>
       <c r="C31" t="str">
-        <v>ACER</v>
+        <v>Office Standard</v>
       </c>
       <c r="D31" t="str">
-        <v>MONE</v>
+        <v>Office UPS Backup (KMN/CH/CP/032)</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -4471,7 +4471,7 @@
         <v/>
       </c>
       <c r="O31" t="str">
-        <v>AST-0033</v>
+        <v>AST-0034</v>
       </c>
     </row>
     <row r="32">
@@ -4479,13 +4479,13 @@
         <v/>
       </c>
       <c r="B32" t="str">
-        <v>Keyboard</v>
+        <v>Monitor</v>
       </c>
       <c r="C32" t="str">
-        <v>Dell</v>
+        <v>ACER</v>
       </c>
       <c r="D32" t="str">
-        <v>Standard Keyboard</v>
+        <v>MONE</v>
       </c>
       <c r="E32" t="str">
         <v/>
@@ -4518,21 +4518,21 @@
         <v/>
       </c>
       <c r="O32" t="str">
-        <v>AST-0032</v>
+        <v>AST-0033</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>KMN/CH/CP/033</v>
+        <v/>
       </c>
       <c r="B33" t="str">
-        <v>Desktop</v>
+        <v>Keyboard</v>
       </c>
       <c r="C33" t="str">
-        <v>ASUS</v>
+        <v>Dell</v>
       </c>
       <c r="D33" t="str">
-        <v>Desktop PC Workstation</v>
+        <v>Standard Keyboard</v>
       </c>
       <c r="E33" t="str">
         <v/>
@@ -4562,24 +4562,24 @@
         <v>LOC-0001</v>
       </c>
       <c r="N33" t="str">
-        <v>CPU KMN IT Tempory</v>
+        <v/>
       </c>
       <c r="O33" t="str">
-        <v>AST-0031</v>
+        <v>AST-0032</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>KMN/CH/CP/031</v>
+        <v>KMN/CH/CP/033</v>
       </c>
       <c r="B34" t="str">
-        <v>Mouse</v>
+        <v>Desktop</v>
       </c>
       <c r="C34" t="str">
-        <v>Standard</v>
+        <v>ASUS</v>
       </c>
       <c r="D34" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Desktop PC Workstation</v>
       </c>
       <c r="E34" t="str">
         <v/>
@@ -4609,24 +4609,24 @@
         <v>LOC-0001</v>
       </c>
       <c r="N34" t="str">
-        <v/>
+        <v>CPU KMN IT Tempory</v>
       </c>
       <c r="O34" t="str">
-        <v>AST-0030</v>
+        <v>AST-0031</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v/>
+        <v>KMN/CH/CP/031</v>
       </c>
       <c r="B35" t="str">
-        <v>UPS</v>
+        <v>Mouse</v>
       </c>
       <c r="C35" t="str">
-        <v>Office Standard</v>
+        <v>Standard</v>
       </c>
       <c r="D35" t="str">
-        <v>Office UPS Backup Unit</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E35" t="str">
         <v/>
@@ -4650,7 +4650,7 @@
         <v>Assigned</v>
       </c>
       <c r="L35" t="str">
-        <v>USR-0007</v>
+        <v>USR-0008</v>
       </c>
       <c r="M35" t="str">
         <v>LOC-0001</v>
@@ -4659,21 +4659,21 @@
         <v/>
       </c>
       <c r="O35" t="str">
-        <v>AST-0029</v>
+        <v>AST-0030</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>KMN/CH/CP/014</v>
+        <v/>
       </c>
       <c r="B36" t="str">
-        <v>Mouse</v>
+        <v>UPS</v>
       </c>
       <c r="C36" t="str">
-        <v>Standard</v>
+        <v>Office Standard</v>
       </c>
       <c r="D36" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Office UPS Backup Unit</v>
       </c>
       <c r="E36" t="str">
         <v/>
@@ -4706,21 +4706,21 @@
         <v/>
       </c>
       <c r="O36" t="str">
-        <v>AST-0028</v>
+        <v>AST-0029</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>KMN/CH/CP/015</v>
+        <v>KMN/CH/CP/014</v>
       </c>
       <c r="B37" t="str">
-        <v>Keyboard</v>
+        <v>Mouse</v>
       </c>
       <c r="C37" t="str">
-        <v>Dell</v>
+        <v>Standard</v>
       </c>
       <c r="D37" t="str">
-        <v>Standard Keyboard</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -4753,21 +4753,21 @@
         <v/>
       </c>
       <c r="O37" t="str">
-        <v>AST-0027</v>
+        <v>AST-0028</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v/>
+        <v>KMN/CH/CP/015</v>
       </c>
       <c r="B38" t="str">
-        <v>All-in-One</v>
+        <v>Keyboard</v>
       </c>
       <c r="C38" t="str">
-        <v>HP</v>
+        <v>Dell</v>
       </c>
       <c r="D38" t="str">
-        <v>PrO 200 G4 AIO-Desktop</v>
+        <v>Standard Keyboard</v>
       </c>
       <c r="E38" t="str">
         <v/>
@@ -4800,7 +4800,7 @@
         <v/>
       </c>
       <c r="O38" t="str">
-        <v>AST-0026</v>
+        <v>AST-0027</v>
       </c>
     </row>
     <row r="39">
@@ -4808,13 +4808,13 @@
         <v/>
       </c>
       <c r="B39" t="str">
-        <v>UPS</v>
+        <v>All-in-One</v>
       </c>
       <c r="C39" t="str">
-        <v>Office Standard</v>
+        <v>HP</v>
       </c>
       <c r="D39" t="str">
-        <v>Office UPS Backup Unit</v>
+        <v>PrO 200 G4 AIO-Desktop</v>
       </c>
       <c r="E39" t="str">
         <v/>
@@ -4838,7 +4838,7 @@
         <v>Assigned</v>
       </c>
       <c r="L39" t="str">
-        <v>USR-0006</v>
+        <v>USR-0007</v>
       </c>
       <c r="M39" t="str">
         <v>LOC-0001</v>
@@ -4847,7 +4847,7 @@
         <v/>
       </c>
       <c r="O39" t="str">
-        <v>AST-0025</v>
+        <v>AST-0026</v>
       </c>
     </row>
     <row r="40">
@@ -4855,13 +4855,13 @@
         <v/>
       </c>
       <c r="B40" t="str">
-        <v>Mouse</v>
+        <v>UPS</v>
       </c>
       <c r="C40" t="str">
-        <v>Standard</v>
+        <v>Office Standard</v>
       </c>
       <c r="D40" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Office UPS Backup Unit</v>
       </c>
       <c r="E40" t="str">
         <v/>
@@ -4894,7 +4894,7 @@
         <v/>
       </c>
       <c r="O40" t="str">
-        <v>AST-0024</v>
+        <v>AST-0025</v>
       </c>
     </row>
     <row r="41">
@@ -4902,13 +4902,13 @@
         <v/>
       </c>
       <c r="B41" t="str">
-        <v>Keyboard</v>
+        <v>Mouse</v>
       </c>
       <c r="C41" t="str">
         <v>Standard</v>
       </c>
       <c r="D41" t="str">
-        <v>Keyboard</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E41" t="str">
         <v/>
@@ -4941,21 +4941,21 @@
         <v/>
       </c>
       <c r="O41" t="str">
-        <v>AST-0023</v>
+        <v>AST-0024</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>KMN/CH/CP/009</v>
+        <v/>
       </c>
       <c r="B42" t="str">
-        <v>Laptop</v>
+        <v>Keyboard</v>
       </c>
       <c r="C42" t="str">
-        <v>ASUS</v>
+        <v>Standard</v>
       </c>
       <c r="D42" t="str">
-        <v>Business Laptop</v>
+        <v>Keyboard</v>
       </c>
       <c r="E42" t="str">
         <v/>
@@ -4988,21 +4988,21 @@
         <v/>
       </c>
       <c r="O42" t="str">
-        <v>AST-0022</v>
+        <v>AST-0023</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>KMN/CH/CP/010</v>
+        <v>KMN/CH/CP/009</v>
       </c>
       <c r="B43" t="str">
-        <v>Desktop</v>
+        <v>Laptop</v>
       </c>
       <c r="C43" t="str">
-        <v>HP</v>
+        <v>ASUS</v>
       </c>
       <c r="D43" t="str">
-        <v>Pro G4-AIO-Desktop</v>
+        <v>Business Laptop</v>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -5035,21 +5035,21 @@
         <v/>
       </c>
       <c r="O43" t="str">
-        <v>AST-0021</v>
+        <v>AST-0022</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v/>
+        <v>KMN/CH/CP/010</v>
       </c>
       <c r="B44" t="str">
-        <v>UPS</v>
+        <v>Desktop</v>
       </c>
       <c r="C44" t="str">
-        <v>Office Standard</v>
+        <v>HP</v>
       </c>
       <c r="D44" t="str">
-        <v>Office UPS Backup Unit</v>
+        <v>Pro G4-AIO-Desktop</v>
       </c>
       <c r="E44" t="str">
         <v/>
@@ -5073,7 +5073,7 @@
         <v>Assigned</v>
       </c>
       <c r="L44" t="str">
-        <v>USR-0005</v>
+        <v>USR-0006</v>
       </c>
       <c r="M44" t="str">
         <v>LOC-0001</v>
@@ -5082,7 +5082,7 @@
         <v/>
       </c>
       <c r="O44" t="str">
-        <v>AST-0020</v>
+        <v>AST-0021</v>
       </c>
     </row>
     <row r="45">
@@ -5090,13 +5090,13 @@
         <v/>
       </c>
       <c r="B45" t="str">
-        <v>Mouse</v>
+        <v>UPS</v>
       </c>
       <c r="C45" t="str">
-        <v>ASUS</v>
+        <v>Office Standard</v>
       </c>
       <c r="D45" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Office UPS Backup Unit</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -5129,7 +5129,7 @@
         <v/>
       </c>
       <c r="O45" t="str">
-        <v>AST-0019</v>
+        <v>AST-0020</v>
       </c>
     </row>
     <row r="46">
@@ -5137,13 +5137,13 @@
         <v/>
       </c>
       <c r="B46" t="str">
-        <v>Keyboard</v>
+        <v>Mouse</v>
       </c>
       <c r="C46" t="str">
         <v>ASUS</v>
       </c>
       <c r="D46" t="str">
-        <v>Standard Keyboard</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E46" t="str">
         <v/>
@@ -5176,7 +5176,7 @@
         <v/>
       </c>
       <c r="O46" t="str">
-        <v>AST-0018</v>
+        <v>AST-0019</v>
       </c>
     </row>
     <row r="47">
@@ -5184,13 +5184,13 @@
         <v/>
       </c>
       <c r="B47" t="str">
-        <v>All-in-One</v>
+        <v>Keyboard</v>
       </c>
       <c r="C47" t="str">
         <v>ASUS</v>
       </c>
       <c r="D47" t="str">
-        <v>All-in-One</v>
+        <v>Standard Keyboard</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -5223,7 +5223,7 @@
         <v/>
       </c>
       <c r="O47" t="str">
-        <v>AST-0017</v>
+        <v>AST-0018</v>
       </c>
     </row>
     <row r="48">
@@ -5231,13 +5231,13 @@
         <v/>
       </c>
       <c r="B48" t="str">
-        <v>UPS</v>
+        <v>All-in-One</v>
       </c>
       <c r="C48" t="str">
-        <v>Office Standard</v>
+        <v>ASUS</v>
       </c>
       <c r="D48" t="str">
-        <v>Office UPS Backup Unit</v>
+        <v>All-in-One</v>
       </c>
       <c r="E48" t="str">
         <v/>
@@ -5261,7 +5261,7 @@
         <v>Assigned</v>
       </c>
       <c r="L48" t="str">
-        <v>USR-0004</v>
+        <v>USR-0005</v>
       </c>
       <c r="M48" t="str">
         <v>LOC-0001</v>
@@ -5270,7 +5270,7 @@
         <v/>
       </c>
       <c r="O48" t="str">
-        <v>AST-0016</v>
+        <v>AST-0017</v>
       </c>
     </row>
     <row r="49">
@@ -5278,13 +5278,13 @@
         <v/>
       </c>
       <c r="B49" t="str">
-        <v>Mouse</v>
+        <v>UPS</v>
       </c>
       <c r="C49" t="str">
-        <v>Standard</v>
+        <v>Office Standard</v>
       </c>
       <c r="D49" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Office UPS Backup Unit</v>
       </c>
       <c r="E49" t="str">
         <v/>
@@ -5317,7 +5317,7 @@
         <v/>
       </c>
       <c r="O49" t="str">
-        <v>AST-0015</v>
+        <v>AST-0016</v>
       </c>
     </row>
     <row r="50">
@@ -5325,13 +5325,13 @@
         <v/>
       </c>
       <c r="B50" t="str">
-        <v>Keyboard</v>
+        <v>Mouse</v>
       </c>
       <c r="C50" t="str">
-        <v>Dell</v>
+        <v>Standard</v>
       </c>
       <c r="D50" t="str">
-        <v>Standard Keyboard</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E50" t="str">
         <v/>
@@ -5364,21 +5364,21 @@
         <v/>
       </c>
       <c r="O50" t="str">
-        <v>AST-0014</v>
+        <v>AST-0015</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>KMN/CH/CP/003</v>
+        <v/>
       </c>
       <c r="B51" t="str">
-        <v>All-in-One</v>
+        <v>Keyboard</v>
       </c>
       <c r="C51" t="str">
-        <v>HP</v>
+        <v>Dell</v>
       </c>
       <c r="D51" t="str">
-        <v>All-in-One</v>
+        <v>Standard Keyboard</v>
       </c>
       <c r="E51" t="str">
         <v/>
@@ -5411,21 +5411,21 @@
         <v/>
       </c>
       <c r="O51" t="str">
-        <v>AST-0013</v>
+        <v>AST-0014</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>KMN/CH/CP/063</v>
+        <v>KMN/CH/CP/003</v>
       </c>
       <c r="B52" t="str">
-        <v>Mouse</v>
+        <v>All-in-One</v>
       </c>
       <c r="C52" t="str">
-        <v>Standard</v>
+        <v>HP</v>
       </c>
       <c r="D52" t="str">
-        <v>Optical USB Mouse</v>
+        <v>All-in-One</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -5449,7 +5449,7 @@
         <v>Assigned</v>
       </c>
       <c r="L52" t="str">
-        <v>USR-0003</v>
+        <v>USR-0004</v>
       </c>
       <c r="M52" t="str">
         <v>LOC-0001</v>
@@ -5458,21 +5458,21 @@
         <v/>
       </c>
       <c r="O52" t="str">
-        <v>AST-0012</v>
+        <v>AST-0013</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>KMN/CH/CP/064</v>
+        <v>KMN/CH/CP/063</v>
       </c>
       <c r="B53" t="str">
-        <v>Laptop</v>
+        <v>Mouse</v>
       </c>
       <c r="C53" t="str">
-        <v>HP</v>
+        <v>Standard</v>
       </c>
       <c r="D53" t="str">
-        <v>Business Laptop</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E53" t="str">
         <v/>
@@ -5505,21 +5505,21 @@
         <v/>
       </c>
       <c r="O53" t="str">
-        <v>AST-0011</v>
+        <v>AST-0012</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>KMN/CH/CP/045</v>
+        <v>KMN/CH/CP/064</v>
       </c>
       <c r="B54" t="str">
-        <v>Desktop</v>
+        <v>Laptop</v>
       </c>
       <c r="C54" t="str">
-        <v>ASUS</v>
+        <v>HP</v>
       </c>
       <c r="D54" t="str">
-        <v>Desktop PC Workstation</v>
+        <v>Business Laptop</v>
       </c>
       <c r="E54" t="str">
         <v/>
@@ -5543,7 +5543,7 @@
         <v>Assigned</v>
       </c>
       <c r="L54" t="str">
-        <v>USR-0002</v>
+        <v>USR-0003</v>
       </c>
       <c r="M54" t="str">
         <v>LOC-0001</v>
@@ -5552,21 +5552,21 @@
         <v/>
       </c>
       <c r="O54" t="str">
-        <v>AST-0010</v>
+        <v>AST-0011</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>KMN/CH/CP/049</v>
+        <v>KMN/CH/CP/045</v>
       </c>
       <c r="B55" t="str">
-        <v>Mouse</v>
+        <v>Desktop</v>
       </c>
       <c r="C55" t="str">
-        <v>Standard</v>
+        <v>ASUS</v>
       </c>
       <c r="D55" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Desktop PC Workstation</v>
       </c>
       <c r="E55" t="str">
         <v/>
@@ -5587,33 +5587,33 @@
         <v/>
       </c>
       <c r="K55" t="str">
-        <v>Assigned</v>
+        <v>Available</v>
       </c>
       <c r="L55" t="str">
-        <v>USR-0002</v>
+        <v/>
       </c>
       <c r="M55" t="str">
-        <v>LOC-0001</v>
+        <v>LOC-0004</v>
       </c>
       <c r="N55" t="str">
         <v/>
       </c>
       <c r="O55" t="str">
-        <v>AST-0009</v>
+        <v>AST-0010</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>KMN/CH/CP/048</v>
+        <v>KMN/CH/CP/049</v>
       </c>
       <c r="B56" t="str">
-        <v>Keyboard</v>
+        <v>Mouse</v>
       </c>
       <c r="C56" t="str">
-        <v>Dell</v>
+        <v>Standard</v>
       </c>
       <c r="D56" t="str">
-        <v>Standard Keyboard</v>
+        <v>Optical USB Mouse</v>
       </c>
       <c r="E56" t="str">
         <v/>
@@ -5646,21 +5646,21 @@
         <v/>
       </c>
       <c r="O56" t="str">
-        <v>AST-0008</v>
+        <v>AST-0009</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>KMN/CH/CP/047</v>
+        <v>KMN/CH/CP/048</v>
       </c>
       <c r="B57" t="str">
-        <v>UPS</v>
+        <v>Keyboard</v>
       </c>
       <c r="C57" t="str">
-        <v>Office Standard</v>
+        <v>Dell</v>
       </c>
       <c r="D57" t="str">
-        <v>Office UPS Backup (KMN/CH/CP/047)</v>
+        <v>Standard Keyboard</v>
       </c>
       <c r="E57" t="str">
         <v/>
@@ -5693,21 +5693,21 @@
         <v/>
       </c>
       <c r="O57" t="str">
-        <v>AST-0007</v>
+        <v>AST-0008</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>KMN/CH/CP/046</v>
+        <v>KMN/CH/CP/047</v>
       </c>
       <c r="B58" t="str">
-        <v>Monitor</v>
+        <v>UPS</v>
       </c>
       <c r="C58" t="str">
-        <v>HP</v>
+        <v>Office Standard</v>
       </c>
       <c r="D58" t="str">
-        <v>Display Monitor</v>
+        <v>Office UPS Backup (KMN/CH/CP/047)</v>
       </c>
       <c r="E58" t="str">
         <v/>
@@ -5740,21 +5740,21 @@
         <v/>
       </c>
       <c r="O58" t="str">
-        <v>AST-0006</v>
+        <v>AST-0007</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v/>
+        <v>KMN/CH/CP/046</v>
       </c>
       <c r="B59" t="str">
-        <v>Printer</v>
+        <v>Monitor</v>
       </c>
       <c r="C59" t="str">
-        <v>EPSON</v>
+        <v>HP</v>
       </c>
       <c r="D59" t="str">
-        <v>Printer</v>
+        <v>Display Monitor</v>
       </c>
       <c r="E59" t="str">
         <v/>
@@ -5778,16 +5778,16 @@
         <v>Assigned</v>
       </c>
       <c r="L59" t="str">
-        <v>USR-0001</v>
+        <v>USR-0002</v>
       </c>
       <c r="M59" t="str">
         <v>LOC-0001</v>
       </c>
       <c r="N59" t="str">
-        <v xml:space="preserve"> [Shared Network Office Printer]</v>
+        <v/>
       </c>
       <c r="O59" t="str">
-        <v>AST-0005</v>
+        <v>AST-0006</v>
       </c>
     </row>
     <row r="60">
@@ -5795,13 +5795,13 @@
         <v/>
       </c>
       <c r="B60" t="str">
-        <v>UPS</v>
+        <v>Printer</v>
       </c>
       <c r="C60" t="str">
-        <v>Office Standard</v>
+        <v>CANON</v>
       </c>
       <c r="D60" t="str">
-        <v>Office UPS Backup Unit</v>
+        <v>G5070</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -5831,24 +5831,24 @@
         <v>LOC-0001</v>
       </c>
       <c r="N60" t="str">
-        <v/>
+        <v xml:space="preserve"> [Shared Network Office Printer]</v>
       </c>
       <c r="O60" t="str">
-        <v>AST-0004</v>
+        <v>AST-0005</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>KMN/CH/CP/028</v>
+        <v/>
       </c>
       <c r="B61" t="str">
-        <v>Keyboard</v>
+        <v>UPS</v>
       </c>
       <c r="C61" t="str">
-        <v>Dell</v>
+        <v>Office Standard</v>
       </c>
       <c r="D61" t="str">
-        <v>Standard Keyboard</v>
+        <v>Office UPS Backup Unit</v>
       </c>
       <c r="E61" t="str">
         <v/>
@@ -5881,21 +5881,21 @@
         <v/>
       </c>
       <c r="O61" t="str">
-        <v>AST-0003</v>
+        <v>AST-0004</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>KMN/CH/CP/030</v>
+        <v>KMN/CH/CP/028</v>
       </c>
       <c r="B62" t="str">
-        <v>Monitor</v>
+        <v>Keyboard</v>
       </c>
       <c r="C62" t="str">
-        <v>Generic</v>
+        <v>Dell</v>
       </c>
       <c r="D62" t="str">
-        <v>Display Monitor</v>
+        <v>Standard Keyboard</v>
       </c>
       <c r="E62" t="str">
         <v/>
@@ -5928,21 +5928,21 @@
         <v/>
       </c>
       <c r="O62" t="str">
-        <v>AST-0002</v>
+        <v>AST-0003</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>KMN/CH/CP/026</v>
+        <v>KMN/CH/CP/030</v>
       </c>
       <c r="B63" t="str">
-        <v>Mouse</v>
+        <v>Monitor</v>
       </c>
       <c r="C63" t="str">
-        <v>Standard</v>
+        <v>Generic</v>
       </c>
       <c r="D63" t="str">
-        <v>Optical USB Mouse</v>
+        <v>Display Monitor</v>
       </c>
       <c r="E63" t="str">
         <v/>
@@ -5975,12 +5975,59 @@
         <v/>
       </c>
       <c r="O63" t="str">
+        <v>AST-0002</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>KMN/CH/CP/026</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Mouse</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Optical USB Mouse</v>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="J64" t="str">
+        <v/>
+      </c>
+      <c r="K64" t="str">
+        <v>Assigned</v>
+      </c>
+      <c r="L64" t="str">
+        <v>USR-0001</v>
+      </c>
+      <c r="M64" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="N64" t="str">
+        <v/>
+      </c>
+      <c r="O64" t="str">
         <v>AST-0001</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R64"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5997,7 +6044,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L62"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6039,19 +6086,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ASN-0003</v>
+        <v>ASN-0061</v>
       </c>
       <c r="B2" t="str">
-        <v>AST-0005</v>
+        <v>AST-0064</v>
       </c>
       <c r="C2" t="str">
-        <v>USR-0001</v>
+        <v>USR-0002</v>
       </c>
       <c r="D2" t="str">
         <v>LOC-0001</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-09-22</v>
+        <v>2026-09-23</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -6060,7 +6107,7 @@
         <v>Current</v>
       </c>
       <c r="H2" t="str">
-        <v>Employee Handover / Device Swap</v>
+        <v>New Equipment Handover to Staff</v>
       </c>
       <c r="I2" t="str">
         <v>Good</v>
@@ -6074,13 +6121,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ASN-0002</v>
+        <v>ASN-0003</v>
       </c>
       <c r="B3" t="str">
-        <v>AST-0057</v>
+        <v>AST-0005</v>
       </c>
       <c r="C3" t="str">
-        <v>USR-0008</v>
+        <v>USR-0001</v>
       </c>
       <c r="D3" t="str">
         <v>LOC-0001</v>
@@ -6109,19 +6156,19 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ASN-0001</v>
+        <v>ASN-0002</v>
       </c>
       <c r="B4" t="str">
-        <v>AST-0058</v>
+        <v>AST-0057</v>
       </c>
       <c r="C4" t="str">
-        <v>USR-0014</v>
+        <v>USR-0008</v>
       </c>
       <c r="D4" t="str">
         <v>LOC-0001</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-22</v>
       </c>
       <c r="F4" t="str">
         <v/>
@@ -6130,24 +6177,2054 @@
         <v>Current</v>
       </c>
       <c r="H4" t="str">
+        <v>Employee Handover / Device Swap</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ASN-0001</v>
+      </c>
+      <c r="B5" t="str">
+        <v>AST-0058</v>
+      </c>
+      <c r="C5" t="str">
+        <v>USR-0014</v>
+      </c>
+      <c r="D5" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H5" t="str">
         <v>Newly Issued Peripheral (Peripheral) to employee</v>
       </c>
-      <c r="I4" t="str">
+      <c r="I5" t="str">
         <v>Brand New</v>
       </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4" t="str">
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
         <v>Issued during service REP-0004: HAVEN'T A MOUSE</v>
       </c>
-      <c r="L4" t="str">
+      <c r="L5" t="str">
         <v>INV-0003</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ASN-0004</v>
+      </c>
+      <c r="B6" t="str">
+        <v>AST-0063</v>
+      </c>
+      <c r="C6" t="str">
+        <v>USR-0016</v>
+      </c>
+      <c r="D6" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ASN-0005</v>
+      </c>
+      <c r="B7" t="str">
+        <v>AST-0062</v>
+      </c>
+      <c r="C7" t="str">
+        <v>USR-0016</v>
+      </c>
+      <c r="D7" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ASN-0006</v>
+      </c>
+      <c r="B8" t="str">
+        <v>AST-0061</v>
+      </c>
+      <c r="C8" t="str">
+        <v>USR-0016</v>
+      </c>
+      <c r="D8" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ASN-0007</v>
+      </c>
+      <c r="B9" t="str">
+        <v>AST-0060</v>
+      </c>
+      <c r="C9" t="str">
+        <v>SHARED_NETWORK</v>
+      </c>
+      <c r="D9" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Shared Network Hardware</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ASN-0008</v>
+      </c>
+      <c r="B10" t="str">
+        <v>AST-0059</v>
+      </c>
+      <c r="C10" t="str">
+        <v>SHARED_NETWORK</v>
+      </c>
+      <c r="D10" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Shared Network Hardware</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ASN-0009</v>
+      </c>
+      <c r="B11" t="str">
+        <v>AST-0056</v>
+      </c>
+      <c r="C11" t="str">
+        <v>USR-0015</v>
+      </c>
+      <c r="D11" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ASN-0010</v>
+      </c>
+      <c r="B12" t="str">
+        <v>AST-0055</v>
+      </c>
+      <c r="C12" t="str">
+        <v>USR-0015</v>
+      </c>
+      <c r="D12" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>ASN-0011</v>
+      </c>
+      <c r="B13" t="str">
+        <v>AST-0053</v>
+      </c>
+      <c r="C13" t="str">
+        <v>USR-0014</v>
+      </c>
+      <c r="D13" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>ASN-0012</v>
+      </c>
+      <c r="B14" t="str">
+        <v>AST-0052</v>
+      </c>
+      <c r="C14" t="str">
+        <v>USR-0014</v>
+      </c>
+      <c r="D14" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>ASN-0013</v>
+      </c>
+      <c r="B15" t="str">
+        <v>AST-0051</v>
+      </c>
+      <c r="C15" t="str">
+        <v>USR-0014</v>
+      </c>
+      <c r="D15" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>ASN-0014</v>
+      </c>
+      <c r="B16" t="str">
+        <v>AST-0050</v>
+      </c>
+      <c r="C16" t="str">
+        <v>USR-0013</v>
+      </c>
+      <c r="D16" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>ASN-0015</v>
+      </c>
+      <c r="B17" t="str">
+        <v>AST-0049</v>
+      </c>
+      <c r="C17" t="str">
+        <v>USR-0013</v>
+      </c>
+      <c r="D17" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>ASN-0016</v>
+      </c>
+      <c r="B18" t="str">
+        <v>AST-0048</v>
+      </c>
+      <c r="C18" t="str">
+        <v>USR-0013</v>
+      </c>
+      <c r="D18" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E18" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>ASN-0017</v>
+      </c>
+      <c r="B19" t="str">
+        <v>AST-0045</v>
+      </c>
+      <c r="C19" t="str">
+        <v>USR-0011</v>
+      </c>
+      <c r="D19" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E19" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>ASN-0018</v>
+      </c>
+      <c r="B20" t="str">
+        <v>AST-0044</v>
+      </c>
+      <c r="C20" t="str">
+        <v>USR-0011</v>
+      </c>
+      <c r="D20" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E20" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>ASN-0019</v>
+      </c>
+      <c r="B21" t="str">
+        <v>AST-0043</v>
+      </c>
+      <c r="C21" t="str">
+        <v>USR-0010</v>
+      </c>
+      <c r="D21" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>ASN-0020</v>
+      </c>
+      <c r="B22" t="str">
+        <v>AST-0042</v>
+      </c>
+      <c r="C22" t="str">
+        <v>USR-0010</v>
+      </c>
+      <c r="D22" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E22" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>ASN-0021</v>
+      </c>
+      <c r="B23" t="str">
+        <v>AST-0041</v>
+      </c>
+      <c r="C23" t="str">
+        <v>USR-0010</v>
+      </c>
+      <c r="D23" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E23" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>ASN-0022</v>
+      </c>
+      <c r="B24" t="str">
+        <v>AST-0040</v>
+      </c>
+      <c r="C24" t="str">
+        <v>USR-0010</v>
+      </c>
+      <c r="D24" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>ASN-0023</v>
+      </c>
+      <c r="B25" t="str">
+        <v>AST-0039</v>
+      </c>
+      <c r="C25" t="str">
+        <v>USR-0010</v>
+      </c>
+      <c r="D25" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>ASN-0024</v>
+      </c>
+      <c r="B26" t="str">
+        <v>AST-0038</v>
+      </c>
+      <c r="C26" t="str">
+        <v>USR-0009</v>
+      </c>
+      <c r="D26" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>ASN-0025</v>
+      </c>
+      <c r="B27" t="str">
+        <v>AST-0037</v>
+      </c>
+      <c r="C27" t="str">
+        <v>USR-0009</v>
+      </c>
+      <c r="D27" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>ASN-0026</v>
+      </c>
+      <c r="B28" t="str">
+        <v>AST-0036</v>
+      </c>
+      <c r="C28" t="str">
+        <v>USR-0009</v>
+      </c>
+      <c r="D28" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>ASN-0027</v>
+      </c>
+      <c r="B29" t="str">
+        <v>AST-0035</v>
+      </c>
+      <c r="C29" t="str">
+        <v>USR-0009</v>
+      </c>
+      <c r="D29" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E29" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>ASN-0028</v>
+      </c>
+      <c r="B30" t="str">
+        <v>AST-0034</v>
+      </c>
+      <c r="C30" t="str">
+        <v>USR-0008</v>
+      </c>
+      <c r="D30" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>ASN-0029</v>
+      </c>
+      <c r="B31" t="str">
+        <v>AST-0033</v>
+      </c>
+      <c r="C31" t="str">
+        <v>USR-0008</v>
+      </c>
+      <c r="D31" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E31" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>ASN-0030</v>
+      </c>
+      <c r="B32" t="str">
+        <v>AST-0032</v>
+      </c>
+      <c r="C32" t="str">
+        <v>USR-0008</v>
+      </c>
+      <c r="D32" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E32" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>ASN-0031</v>
+      </c>
+      <c r="B33" t="str">
+        <v>AST-0031</v>
+      </c>
+      <c r="C33" t="str">
+        <v>USR-0008</v>
+      </c>
+      <c r="D33" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E33" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>ASN-0032</v>
+      </c>
+      <c r="B34" t="str">
+        <v>AST-0030</v>
+      </c>
+      <c r="C34" t="str">
+        <v>USR-0008</v>
+      </c>
+      <c r="D34" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E34" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>ASN-0033</v>
+      </c>
+      <c r="B35" t="str">
+        <v>AST-0029</v>
+      </c>
+      <c r="C35" t="str">
+        <v>USR-0007</v>
+      </c>
+      <c r="D35" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E35" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>ASN-0034</v>
+      </c>
+      <c r="B36" t="str">
+        <v>AST-0028</v>
+      </c>
+      <c r="C36" t="str">
+        <v>USR-0007</v>
+      </c>
+      <c r="D36" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E36" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>ASN-0035</v>
+      </c>
+      <c r="B37" t="str">
+        <v>AST-0027</v>
+      </c>
+      <c r="C37" t="str">
+        <v>USR-0007</v>
+      </c>
+      <c r="D37" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E37" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>ASN-0036</v>
+      </c>
+      <c r="B38" t="str">
+        <v>AST-0026</v>
+      </c>
+      <c r="C38" t="str">
+        <v>USR-0007</v>
+      </c>
+      <c r="D38" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E38" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>ASN-0037</v>
+      </c>
+      <c r="B39" t="str">
+        <v>AST-0025</v>
+      </c>
+      <c r="C39" t="str">
+        <v>USR-0006</v>
+      </c>
+      <c r="D39" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E39" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>ASN-0038</v>
+      </c>
+      <c r="B40" t="str">
+        <v>AST-0024</v>
+      </c>
+      <c r="C40" t="str">
+        <v>USR-0006</v>
+      </c>
+      <c r="D40" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E40" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>ASN-0039</v>
+      </c>
+      <c r="B41" t="str">
+        <v>AST-0023</v>
+      </c>
+      <c r="C41" t="str">
+        <v>USR-0006</v>
+      </c>
+      <c r="D41" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E41" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+      <c r="K41" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>ASN-0040</v>
+      </c>
+      <c r="B42" t="str">
+        <v>AST-0022</v>
+      </c>
+      <c r="C42" t="str">
+        <v>USR-0006</v>
+      </c>
+      <c r="D42" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E42" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>ASN-0041</v>
+      </c>
+      <c r="B43" t="str">
+        <v>AST-0021</v>
+      </c>
+      <c r="C43" t="str">
+        <v>USR-0006</v>
+      </c>
+      <c r="D43" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E43" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>ASN-0042</v>
+      </c>
+      <c r="B44" t="str">
+        <v>AST-0020</v>
+      </c>
+      <c r="C44" t="str">
+        <v>USR-0005</v>
+      </c>
+      <c r="D44" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E44" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I44" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J44" t="str">
+        <v/>
+      </c>
+      <c r="K44" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>ASN-0043</v>
+      </c>
+      <c r="B45" t="str">
+        <v>AST-0019</v>
+      </c>
+      <c r="C45" t="str">
+        <v>USR-0005</v>
+      </c>
+      <c r="D45" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E45" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I45" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+      <c r="K45" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>ASN-0044</v>
+      </c>
+      <c r="B46" t="str">
+        <v>AST-0018</v>
+      </c>
+      <c r="C46" t="str">
+        <v>USR-0005</v>
+      </c>
+      <c r="D46" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E46" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I46" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+      <c r="K46" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>ASN-0045</v>
+      </c>
+      <c r="B47" t="str">
+        <v>AST-0017</v>
+      </c>
+      <c r="C47" t="str">
+        <v>USR-0005</v>
+      </c>
+      <c r="D47" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E47" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H47" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I47" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+      <c r="K47" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>ASN-0046</v>
+      </c>
+      <c r="B48" t="str">
+        <v>AST-0016</v>
+      </c>
+      <c r="C48" t="str">
+        <v>USR-0004</v>
+      </c>
+      <c r="D48" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E48" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H48" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+      <c r="K48" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>ASN-0047</v>
+      </c>
+      <c r="B49" t="str">
+        <v>AST-0015</v>
+      </c>
+      <c r="C49" t="str">
+        <v>USR-0004</v>
+      </c>
+      <c r="D49" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E49" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H49" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+      <c r="K49" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>ASN-0048</v>
+      </c>
+      <c r="B50" t="str">
+        <v>AST-0014</v>
+      </c>
+      <c r="C50" t="str">
+        <v>USR-0004</v>
+      </c>
+      <c r="D50" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E50" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H50" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+      <c r="K50" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>ASN-0049</v>
+      </c>
+      <c r="B51" t="str">
+        <v>AST-0013</v>
+      </c>
+      <c r="C51" t="str">
+        <v>USR-0004</v>
+      </c>
+      <c r="D51" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E51" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H51" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I51" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+      <c r="K51" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>ASN-0050</v>
+      </c>
+      <c r="B52" t="str">
+        <v>AST-0012</v>
+      </c>
+      <c r="C52" t="str">
+        <v>USR-0003</v>
+      </c>
+      <c r="D52" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E52" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H52" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I52" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>ASN-0051</v>
+      </c>
+      <c r="B53" t="str">
+        <v>AST-0011</v>
+      </c>
+      <c r="C53" t="str">
+        <v>USR-0003</v>
+      </c>
+      <c r="D53" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E53" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H53" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I53" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+      <c r="K53" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>ASN-0052</v>
+      </c>
+      <c r="B54" t="str">
+        <v>AST-0010</v>
+      </c>
+      <c r="C54" t="str">
+        <v>USR-0002</v>
+      </c>
+      <c r="D54" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E54" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F54" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Returned</v>
+      </c>
+      <c r="H54" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I54" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J54" t="str">
+        <v>Fair / Cosmetic Wear</v>
+      </c>
+      <c r="K54" t="str">
+        <v>Initial active assignment from inventory baseline. [Equipment Removed / Replaced - Returned to Storage (Available)]</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>ASN-0053</v>
+      </c>
+      <c r="B55" t="str">
+        <v>AST-0009</v>
+      </c>
+      <c r="C55" t="str">
+        <v>USR-0002</v>
+      </c>
+      <c r="D55" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E55" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H55" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I55" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+      <c r="K55" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>ASN-0054</v>
+      </c>
+      <c r="B56" t="str">
+        <v>AST-0008</v>
+      </c>
+      <c r="C56" t="str">
+        <v>USR-0002</v>
+      </c>
+      <c r="D56" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E56" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H56" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I56" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+      <c r="K56" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>ASN-0055</v>
+      </c>
+      <c r="B57" t="str">
+        <v>AST-0007</v>
+      </c>
+      <c r="C57" t="str">
+        <v>USR-0002</v>
+      </c>
+      <c r="D57" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E57" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H57" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I57" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+      <c r="K57" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>ASN-0056</v>
+      </c>
+      <c r="B58" t="str">
+        <v>AST-0006</v>
+      </c>
+      <c r="C58" t="str">
+        <v>USR-0002</v>
+      </c>
+      <c r="D58" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E58" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+      <c r="G58" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H58" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I58" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+      <c r="K58" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>ASN-0057</v>
+      </c>
+      <c r="B59" t="str">
+        <v>AST-0004</v>
+      </c>
+      <c r="C59" t="str">
+        <v>USR-0001</v>
+      </c>
+      <c r="D59" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E59" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+      <c r="G59" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H59" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I59" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
+      <c r="K59" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>ASN-0058</v>
+      </c>
+      <c r="B60" t="str">
+        <v>AST-0003</v>
+      </c>
+      <c r="C60" t="str">
+        <v>USR-0001</v>
+      </c>
+      <c r="D60" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E60" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+      <c r="G60" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H60" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I60" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J60" t="str">
+        <v/>
+      </c>
+      <c r="K60" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>ASN-0059</v>
+      </c>
+      <c r="B61" t="str">
+        <v>AST-0002</v>
+      </c>
+      <c r="C61" t="str">
+        <v>USR-0001</v>
+      </c>
+      <c r="D61" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E61" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H61" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I61" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J61" t="str">
+        <v/>
+      </c>
+      <c r="K61" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>ASN-0060</v>
+      </c>
+      <c r="B62" t="str">
+        <v>AST-0001</v>
+      </c>
+      <c r="C62" t="str">
+        <v>USR-0001</v>
+      </c>
+      <c r="D62" t="str">
+        <v>LOC-0001</v>
+      </c>
+      <c r="E62" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+      <c r="G62" t="str">
+        <v>Current</v>
+      </c>
+      <c r="H62" t="str">
+        <v>Initial Device Deployment</v>
+      </c>
+      <c r="I62" t="str">
+        <v>Good</v>
+      </c>
+      <c r="J62" t="str">
+        <v/>
+      </c>
+      <c r="K62" t="str">
+        <v>Initial active assignment from inventory baseline.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L62"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: implement AC unit management module with interactive floor plans, maintenance modals, and services
</commit_message>
<xml_diff>
--- a/database/IT_Asset_Database.xlsx
+++ b/database/IT_Asset_Database.xlsx
@@ -17,7 +17,11 @@
     <sheet name="Invoices" sheetId="12" r:id="rId12"/>
     <sheet name="Suppliers" sheetId="13" r:id="rId13"/>
     <sheet name="CCTVBills" sheetId="14" r:id="rId14"/>
-    <sheet name="LegacyRawImport" sheetId="15" r:id="rId15"/>
+    <sheet name="ACUnits" sheetId="15" r:id="rId15"/>
+    <sheet name="ACServices" sheetId="16" r:id="rId16"/>
+    <sheet name="ACRepairs" sheetId="17" r:id="rId17"/>
+    <sheet name="ACReplacements" sheetId="18" r:id="rId18"/>
+    <sheet name="LegacyRawImport" sheetId="19" r:id="rId19"/>
   </sheets>
 </workbook>
 </file>
@@ -2475,7 +2479,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
@@ -2743,8 +2753,1473 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:W14"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>UnitID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>UnitNumber</v>
+      </c>
+      <c r="C1" t="str">
+        <v>UnitCode</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Floor</v>
+      </c>
+      <c r="E1" t="str">
+        <v>RoomName</v>
+      </c>
+      <c r="F1" t="str">
+        <v>WallPosition</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Brand</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Model</v>
+      </c>
+      <c r="I1" t="str">
+        <v>CapacityBTU</v>
+      </c>
+      <c r="J1" t="str">
+        <v>RefrigerantType</v>
+      </c>
+      <c r="K1" t="str">
+        <v>PowerRating</v>
+      </c>
+      <c r="L1" t="str">
+        <v>PurchaseDate</v>
+      </c>
+      <c r="M1" t="str">
+        <v>PurchasePrice</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Supplier</v>
+      </c>
+      <c r="O1" t="str">
+        <v>WarrantyUntil</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>WorkMode</v>
+      </c>
+      <c r="R1" t="str">
+        <v>TargetTemp</v>
+      </c>
+      <c r="S1" t="str">
+        <v>CoordX</v>
+      </c>
+      <c r="T1" t="str">
+        <v>CoordY</v>
+      </c>
+      <c r="U1" t="str">
+        <v>LastServiceDate</v>
+      </c>
+      <c r="V1" t="str">
+        <v>NextServiceDue</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>AC-0001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>GF-AC-01</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Ground Floor</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Main Operations Hall (North-West)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Top Wall (North)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Panasonic</v>
+      </c>
+      <c r="H2" t="str">
+        <v>CS-S18TKH Inverter</v>
+      </c>
+      <c r="I2" t="str">
+        <v>18,000 BTU</v>
+      </c>
+      <c r="J2" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K2" t="str">
+        <v>1.5 kW</v>
+      </c>
+      <c r="L2" t="str">
+        <v>2024-02-15</v>
+      </c>
+      <c r="M2">
+        <v>195000</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Singer Sri Lanka PLC</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2029-02-15</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Eco Cooling</v>
+      </c>
+      <c r="R2">
+        <v>22</v>
+      </c>
+      <c r="S2">
+        <v>280</v>
+      </c>
+      <c r="T2">
+        <v>108</v>
+      </c>
+      <c r="U2" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="V2" t="str">
+        <v>2026-10-10</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Primary cooling unit for ground floor front desk and admin workstations</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>AC-0002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>02</v>
+      </c>
+      <c r="C3" t="str">
+        <v>GF-AC-02</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ground Floor</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Main Operations Hall (North-East)</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Top Wall (North)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Panasonic</v>
+      </c>
+      <c r="H3" t="str">
+        <v>CS-S18TKH Inverter</v>
+      </c>
+      <c r="I3" t="str">
+        <v>18,000 BTU</v>
+      </c>
+      <c r="J3" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K3" t="str">
+        <v>1.5 kW</v>
+      </c>
+      <c r="L3" t="str">
+        <v>2024-02-15</v>
+      </c>
+      <c r="M3">
+        <v>195000</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Singer Sri Lanka PLC</v>
+      </c>
+      <c r="O3" t="str">
+        <v>2029-02-15</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Normal Cooling</v>
+      </c>
+      <c r="R3">
+        <v>23</v>
+      </c>
+      <c r="S3">
+        <v>620</v>
+      </c>
+      <c r="T3">
+        <v>108</v>
+      </c>
+      <c r="U3" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="V3" t="str">
+        <v>2026-10-10</v>
+      </c>
+      <c r="W3" t="str">
+        <v>Covers east workstations and client reception seating</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>AC-0003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>03</v>
+      </c>
+      <c r="C4" t="str">
+        <v>GF-AC-03</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Ground Floor</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Main Operations Hall (South-West)</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Bottom Wall (South)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Daikin</v>
+      </c>
+      <c r="H4" t="str">
+        <v>FTKF50 Inverter</v>
+      </c>
+      <c r="I4" t="str">
+        <v>18,000 BTU</v>
+      </c>
+      <c r="J4" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K4" t="str">
+        <v>1.45 kW</v>
+      </c>
+      <c r="L4" t="str">
+        <v>2023-11-20</v>
+      </c>
+      <c r="M4">
+        <v>185000</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Abans PLC</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2028-11-20</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Needs Service</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Low Power</v>
+      </c>
+      <c r="R4">
+        <v>24</v>
+      </c>
+      <c r="S4">
+        <v>280</v>
+      </c>
+      <c r="T4">
+        <v>542</v>
+      </c>
+      <c r="U4" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="V4" t="str">
+        <v>2026-07-12</v>
+      </c>
+      <c r="W4" t="str">
+        <v>Filter cleaning and chemical condenser wash scheduled. Minor blower dust.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>AC-0004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>04</v>
+      </c>
+      <c r="C5" t="str">
+        <v>GF-AC-04</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Ground Floor</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Main Operations Hall (South-East)</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Bottom Wall (South)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Daikin</v>
+      </c>
+      <c r="H5" t="str">
+        <v>FTKF50 Inverter</v>
+      </c>
+      <c r="I5" t="str">
+        <v>18,000 BTU</v>
+      </c>
+      <c r="J5" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K5" t="str">
+        <v>1.45 kW</v>
+      </c>
+      <c r="L5" t="str">
+        <v>2023-11-20</v>
+      </c>
+      <c r="M5">
+        <v>185000</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Abans PLC</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2028-11-20</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Normal Cooling</v>
+      </c>
+      <c r="R5">
+        <v>22</v>
+      </c>
+      <c r="S5">
+        <v>620</v>
+      </c>
+      <c r="T5">
+        <v>542</v>
+      </c>
+      <c r="U5" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="V5" t="str">
+        <v>2026-10-10</v>
+      </c>
+      <c r="W5" t="str">
+        <v>Covers southern operations rows and filing section</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>AC-0005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>05</v>
+      </c>
+      <c r="C6" t="str">
+        <v>1F-AC-05</v>
+      </c>
+      <c r="D6" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E6" t="str">
+        <v>1st Floor Operations Hall (North)</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Long East Wall</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Mitsubishi</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Heavy Duty SRK24CXS</v>
+      </c>
+      <c r="I6" t="str">
+        <v>24,000 BTU</v>
+      </c>
+      <c r="J6" t="str">
+        <v>R410A</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2.1 kW</v>
+      </c>
+      <c r="L6" t="str">
+        <v>2023-08-10</v>
+      </c>
+      <c r="M6">
+        <v>245000</v>
+      </c>
+      <c r="N6" t="str">
+        <v>United Tractors / CoolAir Lanka</v>
+      </c>
+      <c r="O6" t="str">
+        <v>2028-08-10</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Turbo Cooling</v>
+      </c>
+      <c r="R6">
+        <v>21</v>
+      </c>
+      <c r="S6">
+        <v>752</v>
+      </c>
+      <c r="T6">
+        <v>240</v>
+      </c>
+      <c r="U6" t="str">
+        <v>2026-05-18</v>
+      </c>
+      <c r="V6" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="W6" t="str">
+        <v>High-capacity unit covering upper floor main workstation wing</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>AC-0006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>06</v>
+      </c>
+      <c r="C7" t="str">
+        <v>1F-AC-06</v>
+      </c>
+      <c r="D7" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E7" t="str">
+        <v>1st Floor Operations Hall (Center)</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Long East Wall</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Mitsubishi</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Heavy Duty SRK24CXS</v>
+      </c>
+      <c r="I7" t="str">
+        <v>24,000 BTU</v>
+      </c>
+      <c r="J7" t="str">
+        <v>R410A</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2.1 kW</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2023-08-10</v>
+      </c>
+      <c r="M7">
+        <v>245000</v>
+      </c>
+      <c r="N7" t="str">
+        <v>United Tractors / CoolAir Lanka</v>
+      </c>
+      <c r="O7" t="str">
+        <v>2028-08-10</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>Normal Cooling</v>
+      </c>
+      <c r="R7">
+        <v>22</v>
+      </c>
+      <c r="S7">
+        <v>752</v>
+      </c>
+      <c r="T7">
+        <v>360</v>
+      </c>
+      <c r="U7" t="str">
+        <v>2026-05-18</v>
+      </c>
+      <c r="V7" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="W7" t="str">
+        <v>Center wing cooling unit</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>AC-0007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>07</v>
+      </c>
+      <c r="C8" t="str">
+        <v>1F-AC-07</v>
+      </c>
+      <c r="D8" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E8" t="str">
+        <v>1st Floor Operations Hall (South)</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Long East Wall</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Mitsubishi</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Heavy Duty SRK24CXS</v>
+      </c>
+      <c r="I8" t="str">
+        <v>24,000 BTU</v>
+      </c>
+      <c r="J8" t="str">
+        <v>R410A</v>
+      </c>
+      <c r="K8" t="str">
+        <v>2.1 kW</v>
+      </c>
+      <c r="L8" t="str">
+        <v>2023-08-10</v>
+      </c>
+      <c r="M8">
+        <v>245000</v>
+      </c>
+      <c r="N8" t="str">
+        <v>United Tractors / CoolAir Lanka</v>
+      </c>
+      <c r="O8" t="str">
+        <v>2028-08-10</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Normal Cooling</v>
+      </c>
+      <c r="R8">
+        <v>22</v>
+      </c>
+      <c r="S8">
+        <v>752</v>
+      </c>
+      <c r="T8">
+        <v>480</v>
+      </c>
+      <c r="U8" t="str">
+        <v>2026-05-18</v>
+      </c>
+      <c r="V8" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="W8" t="str">
+        <v>South corridor cooling unit</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>AC-0008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>08</v>
+      </c>
+      <c r="C9" t="str">
+        <v>1F-AC-08</v>
+      </c>
+      <c r="D9" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Corner Conference &amp; Meeting Room</v>
+      </c>
+      <c r="F9" t="str">
+        <v>North Wall (Corner)</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Panasonic</v>
+      </c>
+      <c r="H9" t="str">
+        <v>CS-S18TKH Inverter</v>
+      </c>
+      <c r="I9" t="str">
+        <v>18,000 BTU</v>
+      </c>
+      <c r="J9" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K9" t="str">
+        <v>1.5 kW</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2024-01-14</v>
+      </c>
+      <c r="M9">
+        <v>190000</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Singer Sri Lanka PLC</v>
+      </c>
+      <c r="O9" t="str">
+        <v>2029-01-14</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>Eco Cooling</v>
+      </c>
+      <c r="R9">
+        <v>23</v>
+      </c>
+      <c r="S9">
+        <v>670</v>
+      </c>
+      <c r="T9">
+        <v>88</v>
+      </c>
+      <c r="U9" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="V9" t="str">
+        <v>2026-11-02</v>
+      </c>
+      <c r="W9" t="str">
+        <v>Dedicated conference room cooling</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>AC-0009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>09</v>
+      </c>
+      <c r="C10" t="str">
+        <v>1F-AC-09</v>
+      </c>
+      <c r="D10" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Executive Office 1</v>
+      </c>
+      <c r="F10" t="str">
+        <v>North Wall</v>
+      </c>
+      <c r="G10" t="str">
+        <v>LG</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Dual Inverter V13WIN</v>
+      </c>
+      <c r="I10" t="str">
+        <v>12,000 BTU</v>
+      </c>
+      <c r="J10" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K10" t="str">
+        <v>1.0 kW</v>
+      </c>
+      <c r="L10" t="str">
+        <v>2024-04-05</v>
+      </c>
+      <c r="M10">
+        <v>155000</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Abans PLC</v>
+      </c>
+      <c r="O10" t="str">
+        <v>2029-04-05</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>Quiet / Normal</v>
+      </c>
+      <c r="R10">
+        <v>24</v>
+      </c>
+      <c r="S10">
+        <v>515</v>
+      </c>
+      <c r="T10">
+        <v>88</v>
+      </c>
+      <c r="U10" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="V10" t="str">
+        <v>2026-11-02</v>
+      </c>
+      <c r="W10" t="str">
+        <v>Director office unit</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>AC-0010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>10</v>
+      </c>
+      <c r="C11" t="str">
+        <v>1F-AC-10</v>
+      </c>
+      <c r="D11" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Executive Office 2</v>
+      </c>
+      <c r="F11" t="str">
+        <v>North Wall</v>
+      </c>
+      <c r="G11" t="str">
+        <v>LG</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Dual Inverter V13WIN</v>
+      </c>
+      <c r="I11" t="str">
+        <v>12,000 BTU</v>
+      </c>
+      <c r="J11" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K11" t="str">
+        <v>1.0 kW</v>
+      </c>
+      <c r="L11" t="str">
+        <v>2024-04-05</v>
+      </c>
+      <c r="M11">
+        <v>155000</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Abans PLC</v>
+      </c>
+      <c r="O11" t="str">
+        <v>2029-04-05</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Under Repair</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>Off / Error</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>385</v>
+      </c>
+      <c r="T11">
+        <v>88</v>
+      </c>
+      <c r="U11" t="str">
+        <v>2026-04-10</v>
+      </c>
+      <c r="V11" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="W11" t="str">
+        <v>Compressor capacitor faulty, fan motor noisy. Service technician called.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>AC-0011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>11</v>
+      </c>
+      <c r="C12" t="str">
+        <v>1F-AC-11</v>
+      </c>
+      <c r="D12" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Accounts &amp; Audit Room</v>
+      </c>
+      <c r="F12" t="str">
+        <v>North Wall (Side Block)</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Gree</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Fairy Inverter GWH12AC</v>
+      </c>
+      <c r="I12" t="str">
+        <v>12,000 BTU</v>
+      </c>
+      <c r="J12" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K12" t="str">
+        <v>1.05 kW</v>
+      </c>
+      <c r="L12" t="str">
+        <v>2023-09-15</v>
+      </c>
+      <c r="M12">
+        <v>145000</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Gree Lanka / Softlogic</v>
+      </c>
+      <c r="O12" t="str">
+        <v>2028-09-15</v>
+      </c>
+      <c r="P12" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>Eco Cooling</v>
+      </c>
+      <c r="R12">
+        <v>23</v>
+      </c>
+      <c r="S12">
+        <v>162</v>
+      </c>
+      <c r="T12">
+        <v>288</v>
+      </c>
+      <c r="U12" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="V12" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="W12" t="str">
+        <v>Accounts staff room cooling unit</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>AC-0012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>12</v>
+      </c>
+      <c r="C13" t="str">
+        <v>1F-AC-12</v>
+      </c>
+      <c r="D13" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E13" t="str">
+        <v>IT &amp; Server Equipment Room</v>
+      </c>
+      <c r="F13" t="str">
+        <v>North Wall (Side Block)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Daikin</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Heavy Duty FTKF50</v>
+      </c>
+      <c r="I13" t="str">
+        <v>18,000 BTU</v>
+      </c>
+      <c r="J13" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K13" t="str">
+        <v>1.5 kW</v>
+      </c>
+      <c r="L13" t="str">
+        <v>2023-06-01</v>
+      </c>
+      <c r="M13">
+        <v>210000</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Abans PLC</v>
+      </c>
+      <c r="O13" t="str">
+        <v>2028-06-01</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>Continuous 24/7</v>
+      </c>
+      <c r="R13">
+        <v>19</v>
+      </c>
+      <c r="S13">
+        <v>250</v>
+      </c>
+      <c r="T13">
+        <v>288</v>
+      </c>
+      <c r="U13" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="V13" t="str">
+        <v>2026-11-01</v>
+      </c>
+      <c r="W13" t="str">
+        <v>Critical server room cooling unit running 24/7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>AC-0013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>13</v>
+      </c>
+      <c r="C14" t="str">
+        <v>1F-AC-13</v>
+      </c>
+      <c r="D14" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Senior Manager Office</v>
+      </c>
+      <c r="F14" t="str">
+        <v>North Wall (Side Block)</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Gree</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Fairy Inverter GWH12AC</v>
+      </c>
+      <c r="I14" t="str">
+        <v>12,000 BTU</v>
+      </c>
+      <c r="J14" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K14" t="str">
+        <v>1.05 kW</v>
+      </c>
+      <c r="L14" t="str">
+        <v>2023-09-15</v>
+      </c>
+      <c r="M14">
+        <v>145000</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Gree Lanka / Softlogic</v>
+      </c>
+      <c r="O14" t="str">
+        <v>2028-09-15</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>Normal Cooling</v>
+      </c>
+      <c r="R14">
+        <v>23</v>
+      </c>
+      <c r="S14">
+        <v>337</v>
+      </c>
+      <c r="T14">
+        <v>288</v>
+      </c>
+      <c r="U14" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="V14" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="W14" t="str">
+        <v>Manager office individual split AC</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:W14"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ServiceID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>UnitID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ServiceDate</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ServiceType</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Cost</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Technician</v>
+      </c>
+      <c r="G1" t="str">
+        <v>InvoiceNo</v>
+      </c>
+      <c r="H1" t="str">
+        <v>GasRefillPSI</v>
+      </c>
+      <c r="I1" t="str">
+        <v>FilterCleaned</v>
+      </c>
+      <c r="J1" t="str">
+        <v>CoilCleaned</v>
+      </c>
+      <c r="K1" t="str">
+        <v>NextServiceDue</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ACS-0001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>AC-0001</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Routine Maintenance</v>
+      </c>
+      <c r="E2">
+        <v>5500</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Lanka Cool Tech (Pvt) Ltd</v>
+      </c>
+      <c r="G2" t="str">
+        <v>INV-AC-102</v>
+      </c>
+      <c r="H2" t="str">
+        <v>135 PSI (OK)</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2026-10-10</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Standard quarterly cleaning and indoor blower pressure wash</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ACS-0002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>AC-0002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Routine Maintenance</v>
+      </c>
+      <c r="E3">
+        <v>5500</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Lanka Cool Tech (Pvt) Ltd</v>
+      </c>
+      <c r="G3" t="str">
+        <v>INV-AC-102</v>
+      </c>
+      <c r="H3" t="str">
+        <v>140 PSI (OK)</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2026-10-10</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Quarterly routine servicing</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ACS-0003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AC-0003</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Routine Maintenance</v>
+      </c>
+      <c r="E4">
+        <v>5500</v>
+      </c>
+      <c r="F4" t="str">
+        <v>CoolAir Solutions</v>
+      </c>
+      <c r="G4" t="str">
+        <v>INV-AC-088</v>
+      </c>
+      <c r="H4" t="str">
+        <v>120 PSI</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4" t="str">
+        <v>2026-07-12</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Routine cleaning. Recommended chemical wash on next service.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ACS-0004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>AC-0005</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2026-05-18</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Chemical Wash &amp; Gas Top-up</v>
+      </c>
+      <c r="E5">
+        <v>12500</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Lanka Cool Tech (Pvt) Ltd</v>
+      </c>
+      <c r="G5" t="str">
+        <v>INV-AC-095</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Topped up R410A (150 PSI)</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Chemical wash of outdoor condenser and indoor evaporator coil</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ACS-0005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>AC-0012</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Server Room Heavy Service</v>
+      </c>
+      <c r="E6">
+        <v>9500</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Daikin Authorized Service (Abans)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>ABN-SRV-4421</v>
+      </c>
+      <c r="H6" t="str">
+        <v>145 PSI (Optimal)</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2026-11-01</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Preventative high-priority maintenance for 24/7 server room cooling</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>RepairID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>UnitID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>IssueDate</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ResolvedDate</v>
+      </c>
+      <c r="E1" t="str">
+        <v>IssueDescription</v>
+      </c>
+      <c r="F1" t="str">
+        <v>PartsReplaced</v>
+      </c>
+      <c r="G1" t="str">
+        <v>RepairCost</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Technician</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="J1" t="str">
+        <v>InvoiceNo</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ACR-0001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>AC-0010</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>Indoor unit blowing warm air and outdoor unit making clicking noise</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Compressor Capacitor 45uF, Indoor Fan Motor Capacitor 2.5uF</v>
+      </c>
+      <c r="G2">
+        <v>18500</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Chilaw Refrigeration &amp; Electricals</v>
+      </c>
+      <c r="I2" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>Capacitor tested blown. Part ordered, expected fix within 24 hours.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ACR-0002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>AC-0003</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2025-11-04</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2025-11-06</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Water leakage from indoor unit condensate tray</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Drain pipe replaced and tray re-leveled</v>
+      </c>
+      <c r="G3">
+        <v>4500</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Lanka Cool Tech (Pvt) Ltd</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="J3" t="str">
+        <v>REP-AC-2025-11</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Drain pipe unclogged and re-routed to exterior gutter</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ReplacementID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>SpotCode</v>
+      </c>
+      <c r="C1" t="str">
+        <v>RoomName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Floor</v>
+      </c>
+      <c r="E1" t="str">
+        <v>OldUnitBrand</v>
+      </c>
+      <c r="F1" t="str">
+        <v>OldUnitModel</v>
+      </c>
+      <c r="G1" t="str">
+        <v>OldUnitPurchaseYear</v>
+      </c>
+      <c r="H1" t="str">
+        <v>OldUnitLifetimeServiceCost</v>
+      </c>
+      <c r="I1" t="str">
+        <v>OldUnitLifetimeRepairCost</v>
+      </c>
+      <c r="J1" t="str">
+        <v>RemovalDate</v>
+      </c>
+      <c r="K1" t="str">
+        <v>RemovalReason</v>
+      </c>
+      <c r="L1" t="str">
+        <v>FinalCondition</v>
+      </c>
+      <c r="M1" t="str">
+        <v>NewUnitID</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ACREP-0001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>1F-AC-12</v>
+      </c>
+      <c r="C2" t="str">
+        <v>IT &amp; Server Equipment Room</v>
+      </c>
+      <c r="D2" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Singer</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Old Non-Inverter 12000 BTU</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2019</v>
+      </c>
+      <c r="H2">
+        <v>48000</v>
+      </c>
+      <c r="I2">
+        <v>65000</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2023-06-01</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Repeated compressor failures, upgraded to Daikin 18,000 BTU Inverter for high server load</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Scrapped / Salvaged for Copper</v>
+      </c>
+      <c r="M2" t="str">
+        <v>AC-0012</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Successfully upgraded server room to high-reliability Daikin unit.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
@@ -6035,7 +7510,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
feat: add comprehensive AC unit management module with views, floor plans, and modals
</commit_message>
<xml_diff>
--- a/database/IT_Asset_Database.xlsx
+++ b/database/IT_Asset_Database.xlsx
@@ -2753,7 +2753,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W14"/>
+  <dimension ref="A1:W17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2840,10 +2840,10 @@
         <v>Ground Floor</v>
       </c>
       <c r="E2" t="str">
-        <v>Main Operations Hall (North-West)</v>
+        <v>Reception (Front Lobby)</v>
       </c>
       <c r="F2" t="str">
-        <v>Top Wall (North)</v>
+        <v>East Wall (Reception)</v>
       </c>
       <c r="G2" t="str">
         <v>Panasonic</v>
@@ -2882,10 +2882,10 @@
         <v>22</v>
       </c>
       <c r="S2">
-        <v>280</v>
+        <v>752</v>
       </c>
       <c r="T2">
-        <v>108</v>
+        <v>440</v>
       </c>
       <c r="U2" t="str">
         <v>2026-06-10</v>
@@ -2894,7 +2894,7 @@
         <v>2026-10-10</v>
       </c>
       <c r="W2" t="str">
-        <v>Primary cooling unit for ground floor front desk and admin workstations</v>
+        <v>Ground floor front reception cooling</v>
       </c>
     </row>
     <row r="3">
@@ -2911,10 +2911,10 @@
         <v>Ground Floor</v>
       </c>
       <c r="E3" t="str">
-        <v>Main Operations Hall (North-East)</v>
+        <v>Ground Operations Hall (East)</v>
       </c>
       <c r="F3" t="str">
-        <v>Top Wall (North)</v>
+        <v>East Wall (Main Hall)</v>
       </c>
       <c r="G3" t="str">
         <v>Panasonic</v>
@@ -2953,10 +2953,10 @@
         <v>23</v>
       </c>
       <c r="S3">
-        <v>620</v>
+        <v>752</v>
       </c>
       <c r="T3">
-        <v>108</v>
+        <v>245</v>
       </c>
       <c r="U3" t="str">
         <v>2026-06-10</v>
@@ -2965,7 +2965,7 @@
         <v>2026-10-10</v>
       </c>
       <c r="W3" t="str">
-        <v>Covers east workstations and client reception seating</v>
+        <v>Main hall east zone cooling unit</v>
       </c>
     </row>
     <row r="4">
@@ -2982,61 +2982,61 @@
         <v>Ground Floor</v>
       </c>
       <c r="E4" t="str">
-        <v>Main Operations Hall (South-West)</v>
+        <v>Ground Operations Hall (West Upper)</v>
       </c>
       <c r="F4" t="str">
-        <v>Bottom Wall (South)</v>
+        <v>West Wall (Upper)</v>
       </c>
       <c r="G4" t="str">
-        <v>Daikin</v>
+        <v>Mitsubishi</v>
       </c>
       <c r="H4" t="str">
-        <v>FTKF50 Inverter</v>
+        <v>Heavy Duty SRK24CXS</v>
       </c>
       <c r="I4" t="str">
-        <v>18,000 BTU</v>
+        <v>24,000 BTU</v>
       </c>
       <c r="J4" t="str">
-        <v>R32</v>
+        <v>R410A</v>
       </c>
       <c r="K4" t="str">
-        <v>1.45 kW</v>
+        <v>2.1 kW</v>
       </c>
       <c r="L4" t="str">
-        <v>2023-11-20</v>
+        <v>2023-08-10</v>
       </c>
       <c r="M4">
-        <v>185000</v>
+        <v>245000</v>
       </c>
       <c r="N4" t="str">
-        <v>Abans PLC</v>
+        <v>United Tractors / CoolAir Lanka</v>
       </c>
       <c r="O4" t="str">
-        <v>2028-11-20</v>
+        <v>2028-08-10</v>
       </c>
       <c r="P4" t="str">
-        <v>Needs Service</v>
+        <v>Active</v>
       </c>
       <c r="Q4" t="str">
-        <v>Low Power</v>
+        <v>Turbo Cooling</v>
       </c>
       <c r="R4">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="S4">
-        <v>280</v>
+        <v>208</v>
       </c>
       <c r="T4">
-        <v>542</v>
+        <v>270</v>
       </c>
       <c r="U4" t="str">
-        <v>2026-03-12</v>
+        <v>2026-05-18</v>
       </c>
       <c r="V4" t="str">
-        <v>2026-07-12</v>
+        <v>2026-09-18</v>
       </c>
       <c r="W4" t="str">
-        <v>Filter cleaning and chemical condenser wash scheduled. Minor blower dust.</v>
+        <v>Main hall west upper zone cooling unit</v>
       </c>
     </row>
     <row r="5">
@@ -3053,40 +3053,40 @@
         <v>Ground Floor</v>
       </c>
       <c r="E5" t="str">
-        <v>Main Operations Hall (South-East)</v>
+        <v>Ground Operations Hall (West Lower)</v>
       </c>
       <c r="F5" t="str">
-        <v>Bottom Wall (South)</v>
+        <v>West Wall (Lower)</v>
       </c>
       <c r="G5" t="str">
-        <v>Daikin</v>
+        <v>Mitsubishi</v>
       </c>
       <c r="H5" t="str">
-        <v>FTKF50 Inverter</v>
+        <v>Heavy Duty SRK24CXS</v>
       </c>
       <c r="I5" t="str">
-        <v>18,000 BTU</v>
+        <v>24,000 BTU</v>
       </c>
       <c r="J5" t="str">
-        <v>R32</v>
+        <v>R410A</v>
       </c>
       <c r="K5" t="str">
-        <v>1.45 kW</v>
+        <v>2.1 kW</v>
       </c>
       <c r="L5" t="str">
-        <v>2023-11-20</v>
+        <v>2023-08-10</v>
       </c>
       <c r="M5">
-        <v>185000</v>
+        <v>245000</v>
       </c>
       <c r="N5" t="str">
-        <v>Abans PLC</v>
+        <v>United Tractors / CoolAir Lanka</v>
       </c>
       <c r="O5" t="str">
-        <v>2028-11-20</v>
+        <v>2028-08-10</v>
       </c>
       <c r="P5" t="str">
-        <v>Active</v>
+        <v>Needs Service</v>
       </c>
       <c r="Q5" t="str">
         <v>Normal Cooling</v>
@@ -3095,19 +3095,19 @@
         <v>22</v>
       </c>
       <c r="S5">
-        <v>620</v>
+        <v>208</v>
       </c>
       <c r="T5">
-        <v>542</v>
+        <v>415</v>
       </c>
       <c r="U5" t="str">
-        <v>2026-06-10</v>
+        <v>2026-03-12</v>
       </c>
       <c r="V5" t="str">
-        <v>2026-10-10</v>
+        <v>2026-07-12</v>
       </c>
       <c r="W5" t="str">
-        <v>Covers southern operations rows and filing section</v>
+        <v>Scheduled for chemical condenser wash</v>
       </c>
     </row>
     <row r="6">
@@ -3118,16 +3118,16 @@
         <v>05</v>
       </c>
       <c r="C6" t="str">
-        <v>1F-AC-05</v>
+        <v>GF-AC-05</v>
       </c>
       <c r="D6" t="str">
-        <v>First Floor</v>
+        <v>Ground Floor</v>
       </c>
       <c r="E6" t="str">
-        <v>1st Floor Operations Hall (North)</v>
+        <v>Boss Office (Executive Suite)</v>
       </c>
       <c r="F6" t="str">
-        <v>Long East Wall</v>
+        <v>West Wall (Boss Office)</v>
       </c>
       <c r="G6" t="str">
         <v>Mitsubishi</v>
@@ -3166,10 +3166,10 @@
         <v>21</v>
       </c>
       <c r="S6">
-        <v>752</v>
+        <v>208</v>
       </c>
       <c r="T6">
-        <v>240</v>
+        <v>628</v>
       </c>
       <c r="U6" t="str">
         <v>2026-05-18</v>
@@ -3178,7 +3178,7 @@
         <v>2026-09-18</v>
       </c>
       <c r="W6" t="str">
-        <v>High-capacity unit covering upper floor main workstation wing</v>
+        <v>Ground floor Boss office executive suite cooling unit</v>
       </c>
     </row>
     <row r="7">
@@ -3189,16 +3189,16 @@
         <v>06</v>
       </c>
       <c r="C7" t="str">
-        <v>1F-AC-06</v>
+        <v>GF-AC-06</v>
       </c>
       <c r="D7" t="str">
-        <v>First Floor</v>
+        <v>Ground Floor</v>
       </c>
       <c r="E7" t="str">
-        <v>1st Floor Operations Hall (Center)</v>
+        <v>HR Office (Human Resources)</v>
       </c>
       <c r="F7" t="str">
-        <v>Long East Wall</v>
+        <v>West Wall (HR Office)</v>
       </c>
       <c r="G7" t="str">
         <v>Mitsubishi</v>
@@ -3237,19 +3237,19 @@
         <v>22</v>
       </c>
       <c r="S7">
-        <v>752</v>
+        <v>208</v>
       </c>
       <c r="T7">
-        <v>360</v>
+        <v>742</v>
       </c>
       <c r="U7" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-10</v>
       </c>
       <c r="V7" t="str">
-        <v>2026-09-18</v>
+        <v>2026-10-10</v>
       </c>
       <c r="W7" t="str">
-        <v>Center wing cooling unit</v>
+        <v>Ground floor HR department cooling unit</v>
       </c>
     </row>
     <row r="8">
@@ -3260,16 +3260,16 @@
         <v>07</v>
       </c>
       <c r="C8" t="str">
-        <v>1F-AC-07</v>
+        <v>GF-AC-07</v>
       </c>
       <c r="D8" t="str">
-        <v>First Floor</v>
+        <v>Ground Floor</v>
       </c>
       <c r="E8" t="str">
-        <v>1st Floor Operations Hall (South)</v>
+        <v>Other Office (Accounts &amp; Operations)</v>
       </c>
       <c r="F8" t="str">
-        <v>Long East Wall</v>
+        <v>West Wall (Other Office)</v>
       </c>
       <c r="G8" t="str">
         <v>Mitsubishi</v>
@@ -3308,19 +3308,19 @@
         <v>22</v>
       </c>
       <c r="S8">
-        <v>752</v>
+        <v>208</v>
       </c>
       <c r="T8">
-        <v>480</v>
+        <v>860</v>
       </c>
       <c r="U8" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-10</v>
       </c>
       <c r="V8" t="str">
-        <v>2026-09-18</v>
+        <v>2026-10-10</v>
       </c>
       <c r="W8" t="str">
-        <v>South corridor cooling unit</v>
+        <v>Ground floor Other Office (Accounts &amp; Operations) cooling unit</v>
       </c>
     </row>
     <row r="9">
@@ -3331,67 +3331,67 @@
         <v>08</v>
       </c>
       <c r="C9" t="str">
-        <v>1F-AC-08</v>
+        <v>1F-AC-14</v>
       </c>
       <c r="D9" t="str">
         <v>First Floor</v>
       </c>
       <c r="E9" t="str">
-        <v>Corner Conference &amp; Meeting Room</v>
+        <v>1st Floor Operations Hall (North)</v>
       </c>
       <c r="F9" t="str">
-        <v>North Wall (Corner)</v>
+        <v>Long East Wall</v>
       </c>
       <c r="G9" t="str">
-        <v>Panasonic</v>
+        <v>Mitsubishi</v>
       </c>
       <c r="H9" t="str">
-        <v>CS-S18TKH Inverter</v>
+        <v>Heavy Duty SRK24CXS</v>
       </c>
       <c r="I9" t="str">
-        <v>18,000 BTU</v>
+        <v>24,000 BTU</v>
       </c>
       <c r="J9" t="str">
-        <v>R32</v>
+        <v>R410A</v>
       </c>
       <c r="K9" t="str">
-        <v>1.5 kW</v>
+        <v>2.1 kW</v>
       </c>
       <c r="L9" t="str">
-        <v>2024-01-14</v>
+        <v>2023-08-10</v>
       </c>
       <c r="M9">
-        <v>190000</v>
+        <v>245000</v>
       </c>
       <c r="N9" t="str">
-        <v>Singer Sri Lanka PLC</v>
+        <v>United Tractors / CoolAir Lanka</v>
       </c>
       <c r="O9" t="str">
-        <v>2029-01-14</v>
+        <v>2028-08-10</v>
       </c>
       <c r="P9" t="str">
         <v>Active</v>
       </c>
       <c r="Q9" t="str">
-        <v>Eco Cooling</v>
+        <v>Turbo Cooling</v>
       </c>
       <c r="R9">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="S9">
-        <v>670</v>
+        <v>752</v>
       </c>
       <c r="T9">
-        <v>88</v>
+        <v>240</v>
       </c>
       <c r="U9" t="str">
-        <v>2026-07-02</v>
+        <v>2026-05-18</v>
       </c>
       <c r="V9" t="str">
-        <v>2026-11-02</v>
+        <v>2026-09-18</v>
       </c>
       <c r="W9" t="str">
-        <v>Dedicated conference room cooling</v>
+        <v>High-capacity unit covering upper floor main workstation wing</v>
       </c>
     </row>
     <row r="10">
@@ -3402,67 +3402,67 @@
         <v>09</v>
       </c>
       <c r="C10" t="str">
-        <v>1F-AC-09</v>
+        <v>1F-AC-15</v>
       </c>
       <c r="D10" t="str">
         <v>First Floor</v>
       </c>
       <c r="E10" t="str">
-        <v>Executive Office 1</v>
+        <v>1st Floor Operations Hall (Center)</v>
       </c>
       <c r="F10" t="str">
-        <v>North Wall</v>
+        <v>Long East Wall</v>
       </c>
       <c r="G10" t="str">
-        <v>LG</v>
+        <v>Mitsubishi</v>
       </c>
       <c r="H10" t="str">
-        <v>Dual Inverter V13WIN</v>
+        <v>Heavy Duty SRK24CXS</v>
       </c>
       <c r="I10" t="str">
-        <v>12,000 BTU</v>
+        <v>24,000 BTU</v>
       </c>
       <c r="J10" t="str">
-        <v>R32</v>
+        <v>R410A</v>
       </c>
       <c r="K10" t="str">
-        <v>1.0 kW</v>
+        <v>2.1 kW</v>
       </c>
       <c r="L10" t="str">
-        <v>2024-04-05</v>
+        <v>2023-08-10</v>
       </c>
       <c r="M10">
-        <v>155000</v>
+        <v>245000</v>
       </c>
       <c r="N10" t="str">
-        <v>Abans PLC</v>
+        <v>United Tractors / CoolAir Lanka</v>
       </c>
       <c r="O10" t="str">
-        <v>2029-04-05</v>
+        <v>2028-08-10</v>
       </c>
       <c r="P10" t="str">
         <v>Active</v>
       </c>
       <c r="Q10" t="str">
-        <v>Quiet / Normal</v>
+        <v>Normal Cooling</v>
       </c>
       <c r="R10">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="S10">
-        <v>515</v>
+        <v>752</v>
       </c>
       <c r="T10">
-        <v>88</v>
+        <v>360</v>
       </c>
       <c r="U10" t="str">
-        <v>2026-07-02</v>
+        <v>2026-05-18</v>
       </c>
       <c r="V10" t="str">
-        <v>2026-11-02</v>
+        <v>2026-09-18</v>
       </c>
       <c r="W10" t="str">
-        <v>Director office unit</v>
+        <v>Center wing cooling unit</v>
       </c>
     </row>
     <row r="11">
@@ -3473,67 +3473,67 @@
         <v>10</v>
       </c>
       <c r="C11" t="str">
-        <v>1F-AC-10</v>
+        <v>1F-AC-16</v>
       </c>
       <c r="D11" t="str">
         <v>First Floor</v>
       </c>
       <c r="E11" t="str">
-        <v>Executive Office 2</v>
+        <v>1st Floor Operations Hall (South)</v>
       </c>
       <c r="F11" t="str">
-        <v>North Wall</v>
+        <v>Long East Wall</v>
       </c>
       <c r="G11" t="str">
-        <v>LG</v>
+        <v>Mitsubishi</v>
       </c>
       <c r="H11" t="str">
-        <v>Dual Inverter V13WIN</v>
+        <v>Heavy Duty SRK24CXS</v>
       </c>
       <c r="I11" t="str">
-        <v>12,000 BTU</v>
+        <v>24,000 BTU</v>
       </c>
       <c r="J11" t="str">
-        <v>R32</v>
+        <v>R410A</v>
       </c>
       <c r="K11" t="str">
-        <v>1.0 kW</v>
+        <v>2.1 kW</v>
       </c>
       <c r="L11" t="str">
-        <v>2024-04-05</v>
+        <v>2023-08-10</v>
       </c>
       <c r="M11">
-        <v>155000</v>
+        <v>245000</v>
       </c>
       <c r="N11" t="str">
-        <v>Abans PLC</v>
+        <v>United Tractors / CoolAir Lanka</v>
       </c>
       <c r="O11" t="str">
-        <v>2029-04-05</v>
+        <v>2028-08-10</v>
       </c>
       <c r="P11" t="str">
-        <v>Under Repair</v>
+        <v>Active</v>
       </c>
       <c r="Q11" t="str">
-        <v>Off / Error</v>
+        <v>Normal Cooling</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="S11">
-        <v>385</v>
+        <v>752</v>
       </c>
       <c r="T11">
-        <v>88</v>
+        <v>480</v>
       </c>
       <c r="U11" t="str">
-        <v>2026-04-10</v>
+        <v>2026-05-18</v>
       </c>
       <c r="V11" t="str">
-        <v>2026-08-10</v>
+        <v>2026-09-18</v>
       </c>
       <c r="W11" t="str">
-        <v>Compressor capacitor faulty, fan motor noisy. Service technician called.</v>
+        <v>South corridor cooling unit</v>
       </c>
     </row>
     <row r="12">
@@ -3544,43 +3544,43 @@
         <v>11</v>
       </c>
       <c r="C12" t="str">
-        <v>1F-AC-11</v>
+        <v>1F-AC-08</v>
       </c>
       <c r="D12" t="str">
         <v>First Floor</v>
       </c>
       <c r="E12" t="str">
-        <v>Accounts &amp; Audit Room</v>
+        <v>Corner Conference &amp; Meeting Room</v>
       </c>
       <c r="F12" t="str">
-        <v>North Wall (Side Block)</v>
+        <v>North Wall (Corner)</v>
       </c>
       <c r="G12" t="str">
-        <v>Gree</v>
+        <v>Panasonic</v>
       </c>
       <c r="H12" t="str">
-        <v>Fairy Inverter GWH12AC</v>
+        <v>CS-S18TKH Inverter</v>
       </c>
       <c r="I12" t="str">
-        <v>12,000 BTU</v>
+        <v>18,000 BTU</v>
       </c>
       <c r="J12" t="str">
         <v>R32</v>
       </c>
       <c r="K12" t="str">
-        <v>1.05 kW</v>
+        <v>1.5 kW</v>
       </c>
       <c r="L12" t="str">
-        <v>2023-09-15</v>
+        <v>2024-01-14</v>
       </c>
       <c r="M12">
-        <v>145000</v>
+        <v>190000</v>
       </c>
       <c r="N12" t="str">
-        <v>Gree Lanka / Softlogic</v>
+        <v>Singer Sri Lanka PLC</v>
       </c>
       <c r="O12" t="str">
-        <v>2028-09-15</v>
+        <v>2029-01-14</v>
       </c>
       <c r="P12" t="str">
         <v>Active</v>
@@ -3592,19 +3592,19 @@
         <v>23</v>
       </c>
       <c r="S12">
-        <v>162</v>
+        <v>670</v>
       </c>
       <c r="T12">
-        <v>288</v>
+        <v>88</v>
       </c>
       <c r="U12" t="str">
-        <v>2026-06-25</v>
+        <v>2026-07-02</v>
       </c>
       <c r="V12" t="str">
-        <v>2026-10-25</v>
+        <v>2026-11-02</v>
       </c>
       <c r="W12" t="str">
-        <v>Accounts staff room cooling unit</v>
+        <v>Dedicated conference room cooling</v>
       </c>
     </row>
     <row r="13">
@@ -3615,67 +3615,67 @@
         <v>12</v>
       </c>
       <c r="C13" t="str">
-        <v>1F-AC-12</v>
+        <v>1F-AC-09</v>
       </c>
       <c r="D13" t="str">
         <v>First Floor</v>
       </c>
       <c r="E13" t="str">
-        <v>IT &amp; Server Equipment Room</v>
+        <v>Executive Office 1</v>
       </c>
       <c r="F13" t="str">
-        <v>North Wall (Side Block)</v>
+        <v>North Wall</v>
       </c>
       <c r="G13" t="str">
-        <v>Daikin</v>
+        <v>LG</v>
       </c>
       <c r="H13" t="str">
-        <v>Heavy Duty FTKF50</v>
+        <v>Dual Inverter V13WIN</v>
       </c>
       <c r="I13" t="str">
-        <v>18,000 BTU</v>
+        <v>12,000 BTU</v>
       </c>
       <c r="J13" t="str">
         <v>R32</v>
       </c>
       <c r="K13" t="str">
-        <v>1.5 kW</v>
+        <v>1.0 kW</v>
       </c>
       <c r="L13" t="str">
-        <v>2023-06-01</v>
+        <v>2024-04-05</v>
       </c>
       <c r="M13">
-        <v>210000</v>
+        <v>155000</v>
       </c>
       <c r="N13" t="str">
         <v>Abans PLC</v>
       </c>
       <c r="O13" t="str">
-        <v>2028-06-01</v>
+        <v>2029-04-05</v>
       </c>
       <c r="P13" t="str">
         <v>Active</v>
       </c>
       <c r="Q13" t="str">
-        <v>Continuous 24/7</v>
+        <v>Quiet / Normal</v>
       </c>
       <c r="R13">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="S13">
-        <v>250</v>
+        <v>515</v>
       </c>
       <c r="T13">
-        <v>288</v>
+        <v>88</v>
       </c>
       <c r="U13" t="str">
-        <v>2026-08-01</v>
+        <v>2026-07-02</v>
       </c>
       <c r="V13" t="str">
-        <v>2026-11-01</v>
+        <v>2026-11-02</v>
       </c>
       <c r="W13" t="str">
-        <v>Critical server room cooling unit running 24/7</v>
+        <v>Director office unit</v>
       </c>
     </row>
     <row r="14">
@@ -3686,22 +3686,22 @@
         <v>13</v>
       </c>
       <c r="C14" t="str">
-        <v>1F-AC-13</v>
+        <v>1F-AC-10</v>
       </c>
       <c r="D14" t="str">
         <v>First Floor</v>
       </c>
       <c r="E14" t="str">
-        <v>Senior Manager Office</v>
+        <v>Executive Office 2</v>
       </c>
       <c r="F14" t="str">
-        <v>North Wall (Side Block)</v>
+        <v>North Wall</v>
       </c>
       <c r="G14" t="str">
-        <v>Gree</v>
+        <v>LG</v>
       </c>
       <c r="H14" t="str">
-        <v>Fairy Inverter GWH12AC</v>
+        <v>Dual Inverter V13WIN</v>
       </c>
       <c r="I14" t="str">
         <v>12,000 BTU</v>
@@ -3710,48 +3710,261 @@
         <v>R32</v>
       </c>
       <c r="K14" t="str">
+        <v>1.0 kW</v>
+      </c>
+      <c r="L14" t="str">
+        <v>2024-04-05</v>
+      </c>
+      <c r="M14">
+        <v>155000</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Abans PLC</v>
+      </c>
+      <c r="O14" t="str">
+        <v>2029-04-05</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Under Repair</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>Off / Error</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>385</v>
+      </c>
+      <c r="T14">
+        <v>88</v>
+      </c>
+      <c r="U14" t="str">
+        <v>2026-04-10</v>
+      </c>
+      <c r="V14" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="W14" t="str">
+        <v>Compressor capacitor faulty, fan motor noisy. Service technician called.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>AC-0014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>14</v>
+      </c>
+      <c r="C15" t="str">
+        <v>1F-AC-11</v>
+      </c>
+      <c r="D15" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Accounts &amp; Audit Room</v>
+      </c>
+      <c r="F15" t="str">
+        <v>North Wall (Side Block)</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Gree</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Fairy Inverter GWH12AC</v>
+      </c>
+      <c r="I15" t="str">
+        <v>12,000 BTU</v>
+      </c>
+      <c r="J15" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K15" t="str">
         <v>1.05 kW</v>
       </c>
-      <c r="L14" t="str">
+      <c r="L15" t="str">
         <v>2023-09-15</v>
       </c>
-      <c r="M14">
+      <c r="M15">
         <v>145000</v>
       </c>
-      <c r="N14" t="str">
+      <c r="N15" t="str">
         <v>Gree Lanka / Softlogic</v>
       </c>
-      <c r="O14" t="str">
+      <c r="O15" t="str">
         <v>2028-09-15</v>
       </c>
-      <c r="P14" t="str">
+      <c r="P15" t="str">
         <v>Active</v>
       </c>
-      <c r="Q14" t="str">
+      <c r="Q15" t="str">
+        <v>Eco Cooling</v>
+      </c>
+      <c r="R15">
+        <v>23</v>
+      </c>
+      <c r="S15">
+        <v>162</v>
+      </c>
+      <c r="T15">
+        <v>288</v>
+      </c>
+      <c r="U15" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="V15" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="W15" t="str">
+        <v>Accounts staff room cooling unit</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>AC-0015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>15</v>
+      </c>
+      <c r="C16" t="str">
+        <v>1F-AC-12</v>
+      </c>
+      <c r="D16" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E16" t="str">
+        <v>IT &amp; Server Equipment Room</v>
+      </c>
+      <c r="F16" t="str">
+        <v>North Wall (Side Block)</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Daikin</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Heavy Duty FTKF50</v>
+      </c>
+      <c r="I16" t="str">
+        <v>18,000 BTU</v>
+      </c>
+      <c r="J16" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K16" t="str">
+        <v>1.5 kW</v>
+      </c>
+      <c r="L16" t="str">
+        <v>2023-06-01</v>
+      </c>
+      <c r="M16">
+        <v>210000</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Abans PLC</v>
+      </c>
+      <c r="O16" t="str">
+        <v>2028-06-01</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>Continuous 24/7</v>
+      </c>
+      <c r="R16">
+        <v>19</v>
+      </c>
+      <c r="S16">
+        <v>250</v>
+      </c>
+      <c r="T16">
+        <v>288</v>
+      </c>
+      <c r="U16" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="V16" t="str">
+        <v>2026-11-01</v>
+      </c>
+      <c r="W16" t="str">
+        <v>Critical server room cooling unit running 24/7</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>AC-0016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>16</v>
+      </c>
+      <c r="C17" t="str">
+        <v>1F-AC-13</v>
+      </c>
+      <c r="D17" t="str">
+        <v>First Floor</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Senior Manager Office</v>
+      </c>
+      <c r="F17" t="str">
+        <v>North Wall (Side Block)</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Gree</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Fairy Inverter GWH12AC</v>
+      </c>
+      <c r="I17" t="str">
+        <v>12,000 BTU</v>
+      </c>
+      <c r="J17" t="str">
+        <v>R32</v>
+      </c>
+      <c r="K17" t="str">
+        <v>1.05 kW</v>
+      </c>
+      <c r="L17" t="str">
+        <v>2023-09-15</v>
+      </c>
+      <c r="M17">
+        <v>145000</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Gree Lanka / Softlogic</v>
+      </c>
+      <c r="O17" t="str">
+        <v>2028-09-15</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Active</v>
+      </c>
+      <c r="Q17" t="str">
         <v>Normal Cooling</v>
       </c>
-      <c r="R14">
+      <c r="R17">
         <v>23</v>
       </c>
-      <c r="S14">
+      <c r="S17">
         <v>337</v>
       </c>
-      <c r="T14">
+      <c r="T17">
         <v>288</v>
       </c>
-      <c r="U14" t="str">
+      <c r="U17" t="str">
         <v>2026-06-25</v>
       </c>
-      <c r="V14" t="str">
+      <c r="V17" t="str">
         <v>2026-10-25</v>
       </c>
-      <c r="W14" t="str">
+      <c r="W17" t="str">
         <v>Manager office individual split AC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: add IT asset database Excel file
</commit_message>
<xml_diff>
--- a/database/IT_Asset_Database.xlsx
+++ b/database/IT_Asset_Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\AnjeloPrograms\ITSystem\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C24B18-6321-48AB-8050-E2F6058211F8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B4C07A-0CC2-405B-A9D9-0B50BD653B30}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2859" uniqueCount="777">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2829" uniqueCount="755">
   <si>
     <t>Name</t>
   </si>
@@ -1963,12 +1963,6 @@
     <t>East Wall (Reception)</t>
   </si>
   <si>
-    <t>Panasonic</t>
-  </si>
-  <si>
-    <t>CS-S18TKH Inverter</t>
-  </si>
-  <si>
     <t>18,000 BTU</t>
   </si>
   <si>
@@ -2002,12 +1996,6 @@
     <t>03</t>
   </si>
   <si>
-    <t>Mitsubishi</t>
-  </si>
-  <si>
-    <t>Heavy Duty SRK24CXS</t>
-  </si>
-  <si>
     <t>24,000 BTU</t>
   </si>
   <si>
@@ -2086,9 +2074,6 @@
     <t>First Floor</t>
   </si>
   <si>
-    <t>1st Floor Operations Hall (North)</t>
-  </si>
-  <si>
     <t>Long East Wall</t>
   </si>
   <si>
@@ -2101,12 +2086,6 @@
     <t>09</t>
   </si>
   <si>
-    <t>1F-AC-15</t>
-  </si>
-  <si>
-    <t>1st Floor Operations Hall (Center)</t>
-  </si>
-  <si>
     <t>Center wing cooling unit</t>
   </si>
   <si>
@@ -2116,12 +2095,6 @@
     <t>10</t>
   </si>
   <si>
-    <t>1F-AC-16</t>
-  </si>
-  <si>
-    <t>1st Floor Operations Hall (South)</t>
-  </si>
-  <si>
     <t>South corridor cooling unit</t>
   </si>
   <si>
@@ -2131,12 +2104,6 @@
     <t>11</t>
   </si>
   <si>
-    <t>1F-AC-08</t>
-  </si>
-  <si>
-    <t>Corner Conference &amp; Meeting Room</t>
-  </si>
-  <si>
     <t>North Wall (Corner)</t>
   </si>
   <si>
@@ -2152,21 +2119,12 @@
     <t>12</t>
   </si>
   <si>
-    <t>1F-AC-09</t>
-  </si>
-  <si>
-    <t>Executive Office 1</t>
-  </si>
-  <si>
     <t>North Wall</t>
   </si>
   <si>
     <t>LG</t>
   </si>
   <si>
-    <t>Dual Inverter V13WIN</t>
-  </si>
-  <si>
     <t>12,000 BTU</t>
   </si>
   <si>
@@ -2182,9 +2140,6 @@
     <t>13</t>
   </si>
   <si>
-    <t>1F-AC-10</t>
-  </si>
-  <si>
     <t>Executive Office 2</t>
   </si>
   <si>
@@ -2197,69 +2152,12 @@
     <t>14</t>
   </si>
   <si>
-    <t>1F-AC-11</t>
-  </si>
-  <si>
-    <t>Accounts &amp; Audit Room</t>
-  </si>
-  <si>
-    <t>North Wall (Side Block)</t>
-  </si>
-  <si>
-    <t>Gree</t>
-  </si>
-  <si>
-    <t>Fairy Inverter GWH12AC</t>
-  </si>
-  <si>
     <t>2026-10-25</t>
   </si>
   <si>
     <t>Accounts staff room cooling unit</t>
   </si>
   <si>
-    <t>AC-0015</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>1F-AC-12</t>
-  </si>
-  <si>
-    <t>IT &amp; Server Equipment Room</t>
-  </si>
-  <si>
-    <t>Daikin</t>
-  </si>
-  <si>
-    <t>Heavy Duty FTKF50</t>
-  </si>
-  <si>
-    <t>Continuous 24/7</t>
-  </si>
-  <si>
-    <t>2026-11-01</t>
-  </si>
-  <si>
-    <t>Critical server room cooling unit running 24/7</t>
-  </si>
-  <si>
-    <t>AC-0016</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>1F-AC-13</t>
-  </si>
-  <si>
-    <t>Senior Manager Office</t>
-  </si>
-  <si>
-    <t>Manager office individual split AC</t>
-  </si>
-  <si>
     <t>ServiceID</t>
   </si>
   <si>
@@ -2369,6 +2267,42 @@
   </si>
   <si>
     <t>Other Office (Recovery &amp; Operations)</t>
+  </si>
+  <si>
+    <t>CHW/AC/008</t>
+  </si>
+  <si>
+    <t>CHW/AC/009</t>
+  </si>
+  <si>
+    <t>CHW/AC/010</t>
+  </si>
+  <si>
+    <t>CHW/AC/011</t>
+  </si>
+  <si>
+    <t>CHW/AC/012</t>
+  </si>
+  <si>
+    <t>CHW/AC/013</t>
+  </si>
+  <si>
+    <t>CHW/AC/014</t>
+  </si>
+  <si>
+    <t>Nadun's Office (North)</t>
+  </si>
+  <si>
+    <t>1st Floor Operations Hall (Center Nadun's Lobbby)</t>
+  </si>
+  <si>
+    <t>Auditorium</t>
+  </si>
+  <si>
+    <t>New Lab</t>
+  </si>
+  <si>
+    <t>LAB</t>
   </si>
 </sst>
 </file>
@@ -2747,9 +2681,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2784,7 +2718,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2819,7 +2753,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -2854,7 +2788,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -2889,7 +2823,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -2924,7 +2858,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -2959,7 +2893,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -2994,7 +2928,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>42</v>
       </c>
@@ -3029,7 +2963,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -3064,7 +2998,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>49</v>
       </c>
@@ -3099,7 +3033,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>52</v>
       </c>
@@ -3134,7 +3068,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -3169,7 +3103,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>58</v>
       </c>
@@ -3204,7 +3138,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>61</v>
       </c>
@@ -3239,7 +3173,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>65</v>
       </c>
@@ -3274,7 +3208,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>68</v>
       </c>
@@ -3309,7 +3243,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>71</v>
       </c>
@@ -3355,9 +3289,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:S7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>460</v>
       </c>
@@ -3416,7 +3350,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>472</v>
       </c>
@@ -3475,7 +3409,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>480</v>
       </c>
@@ -3534,7 +3468,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>483</v>
       </c>
@@ -3593,7 +3527,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>487</v>
       </c>
@@ -3652,7 +3586,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>491</v>
       </c>
@@ -3711,7 +3645,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>494</v>
       </c>
@@ -3781,9 +3715,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:M15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>497</v>
       </c>
@@ -3824,7 +3758,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>502</v>
       </c>
@@ -3865,7 +3799,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>506</v>
       </c>
@@ -3906,7 +3840,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>512</v>
       </c>
@@ -3947,7 +3881,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>519</v>
       </c>
@@ -3988,7 +3922,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>519</v>
       </c>
@@ -4029,7 +3963,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>527</v>
       </c>
@@ -4070,7 +4004,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>530</v>
       </c>
@@ -4111,7 +4045,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>532</v>
       </c>
@@ -4152,7 +4086,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>536</v>
       </c>
@@ -4193,7 +4127,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>537</v>
       </c>
@@ -4234,7 +4168,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>539</v>
       </c>
@@ -4275,7 +4209,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>540</v>
       </c>
@@ -4316,7 +4250,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>542</v>
       </c>
@@ -4357,7 +4291,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>544</v>
       </c>
@@ -4409,9 +4343,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:N9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>401</v>
       </c>
@@ -4455,7 +4389,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>440</v>
       </c>
@@ -4499,7 +4433,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>408</v>
       </c>
@@ -4543,7 +4477,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>412</v>
       </c>
@@ -4587,7 +4521,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>415</v>
       </c>
@@ -4631,7 +4565,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>420</v>
       </c>
@@ -4675,7 +4609,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>305</v>
       </c>
@@ -4719,7 +4653,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>450</v>
       </c>
@@ -4763,7 +4697,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>453</v>
       </c>
@@ -4818,9 +4752,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>285</v>
       </c>
@@ -4836,9 +4770,9 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:T4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>587</v>
       </c>
@@ -4900,7 +4834,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>510</v>
       </c>
@@ -4962,7 +4896,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>517</v>
       </c>
@@ -5024,7 +4958,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>522</v>
       </c>
@@ -5096,8 +5030,8 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:W17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:W15"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="11.75" customWidth="1"/>
     <col min="4" max="4" width="13.625" customWidth="1"/>
@@ -5114,7 +5048,7 @@
     <col min="22" max="22" width="14.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>622</v>
       </c>
@@ -5185,7 +5119,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>637</v>
       </c>
@@ -5193,7 +5127,7 @@
         <v>638</v>
       </c>
       <c r="C2" t="s">
-        <v>761</v>
+        <v>727</v>
       </c>
       <c r="D2" t="s">
         <v>95</v>
@@ -5205,13 +5139,13 @@
         <v>640</v>
       </c>
       <c r="G2" t="s">
-        <v>762</v>
+        <v>728</v>
       </c>
       <c r="H2" t="s">
-        <v>763</v>
+        <v>729</v>
       </c>
       <c r="I2" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="J2" t="s">
         <v>131</v>
@@ -5223,7 +5157,7 @@
         <v>16</v>
       </c>
       <c r="Q2" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="R2">
         <v>22</v>
@@ -5238,39 +5172,39 @@
         <v>46274</v>
       </c>
       <c r="V2" t="s">
+        <v>643</v>
+      </c>
+      <c r="W2" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>645</v>
       </c>
-      <c r="W2" t="s">
+      <c r="B3" t="s">
         <v>646</v>
       </c>
-    </row>
-    <row r="3" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>647</v>
-      </c>
-      <c r="B3" t="s">
-        <v>648</v>
-      </c>
       <c r="C3" t="s">
-        <v>764</v>
+        <v>730</v>
       </c>
       <c r="D3" t="s">
         <v>95</v>
       </c>
       <c r="E3" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="F3" t="s">
-        <v>770</v>
+        <v>736</v>
       </c>
       <c r="G3" t="s">
-        <v>707</v>
+        <v>694</v>
       </c>
       <c r="H3" t="s">
-        <v>763</v>
+        <v>729</v>
       </c>
       <c r="I3" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="J3" t="s">
         <v>131</v>
@@ -5282,7 +5216,7 @@
         <v>16</v>
       </c>
       <c r="Q3" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="R3">
         <v>23</v>
@@ -5297,39 +5231,39 @@
         <v>46274</v>
       </c>
       <c r="V3" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="W3" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>650</v>
+      </c>
+      <c r="B4" t="s">
         <v>651</v>
       </c>
-    </row>
-    <row r="4" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>652</v>
-      </c>
-      <c r="B4" t="s">
-        <v>653</v>
-      </c>
       <c r="C4" t="s">
-        <v>765</v>
+        <v>731</v>
       </c>
       <c r="D4" t="s">
         <v>95</v>
       </c>
       <c r="E4" t="s">
-        <v>771</v>
+        <v>737</v>
       </c>
       <c r="F4" t="s">
-        <v>772</v>
+        <v>738</v>
       </c>
       <c r="G4" t="s">
-        <v>707</v>
+        <v>694</v>
       </c>
       <c r="H4" t="s">
-        <v>773</v>
+        <v>739</v>
       </c>
       <c r="I4" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="J4" t="s">
         <v>131</v>
@@ -5341,7 +5275,7 @@
         <v>16</v>
       </c>
       <c r="Q4" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="R4">
         <v>21</v>
@@ -5356,39 +5290,39 @@
         <v>46274</v>
       </c>
       <c r="V4" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="W4" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="B5" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="C5" t="s">
-        <v>766</v>
+        <v>732</v>
       </c>
       <c r="D5" t="s">
         <v>95</v>
       </c>
       <c r="E5" t="s">
-        <v>774</v>
+        <v>740</v>
       </c>
       <c r="F5" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="G5" t="s">
-        <v>707</v>
+        <v>694</v>
       </c>
       <c r="H5" t="s">
-        <v>773</v>
+        <v>739</v>
       </c>
       <c r="I5" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="J5" t="s">
         <v>131</v>
@@ -5400,7 +5334,7 @@
         <v>16</v>
       </c>
       <c r="Q5" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="R5">
         <v>22</v>
@@ -5415,39 +5349,39 @@
         <v>46274</v>
       </c>
       <c r="V5" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="W5" t="s">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>665</v>
+        <v>661</v>
       </c>
       <c r="B6" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="C6" t="s">
-        <v>767</v>
+        <v>733</v>
       </c>
       <c r="D6" t="s">
         <v>95</v>
       </c>
       <c r="E6" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="F6" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="G6" t="s">
-        <v>762</v>
+        <v>728</v>
       </c>
       <c r="H6" t="s">
-        <v>773</v>
+        <v>739</v>
       </c>
       <c r="I6" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="J6" t="s">
         <v>131</v>
@@ -5459,7 +5393,7 @@
         <v>16</v>
       </c>
       <c r="Q6" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="R6">
         <v>21</v>
@@ -5474,39 +5408,39 @@
         <v>46274</v>
       </c>
       <c r="V6" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="W6" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="B7" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="C7" t="s">
-        <v>768</v>
+        <v>734</v>
       </c>
       <c r="D7" t="s">
         <v>95</v>
       </c>
       <c r="E7" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="F7" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="G7" t="s">
-        <v>775</v>
+        <v>741</v>
       </c>
       <c r="H7" t="s">
-        <v>763</v>
+        <v>729</v>
       </c>
       <c r="I7" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="J7" t="s">
         <v>131</v>
@@ -5518,7 +5452,7 @@
         <v>16</v>
       </c>
       <c r="Q7" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="R7">
         <v>22</v>
@@ -5533,39 +5467,39 @@
         <v>46274</v>
       </c>
       <c r="V7" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="W7" t="s">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="B8" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="C8" t="s">
-        <v>769</v>
+        <v>735</v>
       </c>
       <c r="D8" t="s">
         <v>95</v>
       </c>
       <c r="E8" t="s">
-        <v>776</v>
+        <v>742</v>
       </c>
       <c r="F8" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="G8" t="s">
-        <v>762</v>
+        <v>728</v>
       </c>
       <c r="H8" t="s">
-        <v>773</v>
+        <v>739</v>
       </c>
       <c r="I8" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="J8" t="s">
         <v>131</v>
@@ -5577,7 +5511,7 @@
         <v>16</v>
       </c>
       <c r="Q8" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="R8">
         <v>22</v>
@@ -5592,36 +5526,39 @@
         <v>46274</v>
       </c>
       <c r="V8" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="W8" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>675</v>
+      </c>
+      <c r="B9" t="s">
+        <v>676</v>
+      </c>
+      <c r="C9" t="s">
+        <v>743</v>
+      </c>
+      <c r="D9" t="s">
+        <v>677</v>
+      </c>
+      <c r="E9" t="s">
+        <v>750</v>
+      </c>
+      <c r="F9" t="s">
         <v>678</v>
       </c>
-    </row>
-    <row r="9" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>679</v>
-      </c>
-      <c r="B9" t="s">
-        <v>680</v>
-      </c>
-      <c r="D9" t="s">
-        <v>681</v>
-      </c>
-      <c r="E9" t="s">
-        <v>682</v>
-      </c>
-      <c r="F9" t="s">
-        <v>683</v>
-      </c>
       <c r="G9" t="s">
-        <v>654</v>
+        <v>694</v>
       </c>
       <c r="H9" t="s">
-        <v>655</v>
+        <v>739</v>
       </c>
       <c r="I9" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="J9" t="s">
         <v>131</v>
@@ -5633,7 +5570,7 @@
         <v>16</v>
       </c>
       <c r="Q9" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="R9">
         <v>21</v>
@@ -5648,39 +5585,39 @@
         <v>46274</v>
       </c>
       <c r="V9" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="W9" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>685</v>
+        <v>680</v>
       </c>
       <c r="B10" t="s">
-        <v>686</v>
+        <v>681</v>
       </c>
       <c r="C10" t="s">
-        <v>687</v>
+        <v>744</v>
       </c>
       <c r="D10" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="E10" t="s">
-        <v>688</v>
+        <v>751</v>
       </c>
       <c r="F10" t="s">
-        <v>683</v>
+        <v>678</v>
       </c>
       <c r="G10" t="s">
-        <v>654</v>
+        <v>694</v>
       </c>
       <c r="H10" t="s">
-        <v>655</v>
+        <v>739</v>
       </c>
       <c r="I10" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="J10" t="s">
         <v>131</v>
@@ -5692,7 +5629,7 @@
         <v>16</v>
       </c>
       <c r="Q10" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="R10">
         <v>22</v>
@@ -5707,39 +5644,39 @@
         <v>46274</v>
       </c>
       <c r="V10" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="W10" t="s">
-        <v>689</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>690</v>
+        <v>683</v>
       </c>
       <c r="B11" t="s">
-        <v>691</v>
+        <v>684</v>
       </c>
       <c r="C11" t="s">
-        <v>692</v>
+        <v>745</v>
       </c>
       <c r="D11" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="E11" t="s">
-        <v>693</v>
+        <v>752</v>
       </c>
       <c r="F11" t="s">
-        <v>683</v>
+        <v>678</v>
       </c>
       <c r="G11" t="s">
-        <v>654</v>
+        <v>741</v>
       </c>
       <c r="H11" t="s">
-        <v>655</v>
+        <v>739</v>
       </c>
       <c r="I11" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="J11" t="s">
         <v>131</v>
@@ -5751,7 +5688,7 @@
         <v>16</v>
       </c>
       <c r="Q11" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="R11">
         <v>22</v>
@@ -5766,39 +5703,39 @@
         <v>46274</v>
       </c>
       <c r="V11" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="W11" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>686</v>
+      </c>
+      <c r="B12" t="s">
+        <v>687</v>
+      </c>
+      <c r="C12" t="s">
+        <v>746</v>
+      </c>
+      <c r="D12" t="s">
+        <v>677</v>
+      </c>
+      <c r="E12" t="s">
+        <v>752</v>
+      </c>
+      <c r="F12" t="s">
+        <v>688</v>
+      </c>
+      <c r="G12" t="s">
         <v>694</v>
       </c>
-    </row>
-    <row r="12" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>695</v>
-      </c>
-      <c r="B12" t="s">
-        <v>696</v>
-      </c>
-      <c r="C12" t="s">
-        <v>697</v>
-      </c>
-      <c r="D12" t="s">
-        <v>681</v>
-      </c>
-      <c r="E12" t="s">
-        <v>698</v>
-      </c>
-      <c r="F12" t="s">
-        <v>699</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
+        <v>739</v>
+      </c>
+      <c r="I12" t="s">
         <v>641</v>
-      </c>
-      <c r="H12" t="s">
-        <v>642</v>
-      </c>
-      <c r="I12" t="s">
-        <v>643</v>
       </c>
       <c r="J12" t="s">
         <v>131</v>
@@ -5810,7 +5747,7 @@
         <v>16</v>
       </c>
       <c r="Q12" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="R12">
         <v>23</v>
@@ -5825,39 +5762,39 @@
         <v>46274</v>
       </c>
       <c r="V12" t="s">
-        <v>700</v>
+        <v>689</v>
       </c>
       <c r="W12" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>702</v>
+        <v>691</v>
       </c>
       <c r="B13" t="s">
-        <v>703</v>
+        <v>692</v>
       </c>
       <c r="C13" t="s">
-        <v>704</v>
+        <v>747</v>
       </c>
       <c r="D13" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="E13" t="s">
-        <v>705</v>
+        <v>752</v>
       </c>
       <c r="F13" t="s">
-        <v>706</v>
+        <v>693</v>
       </c>
       <c r="G13" t="s">
-        <v>707</v>
+        <v>694</v>
       </c>
       <c r="H13" t="s">
-        <v>708</v>
+        <v>739</v>
       </c>
       <c r="I13" t="s">
-        <v>709</v>
+        <v>695</v>
       </c>
       <c r="J13" t="s">
         <v>131</v>
@@ -5869,7 +5806,7 @@
         <v>16</v>
       </c>
       <c r="Q13" t="s">
-        <v>710</v>
+        <v>696</v>
       </c>
       <c r="R13">
         <v>24</v>
@@ -5884,39 +5821,39 @@
         <v>46274</v>
       </c>
       <c r="V13" t="s">
+        <v>689</v>
+      </c>
+      <c r="W13" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>698</v>
+      </c>
+      <c r="B14" t="s">
+        <v>699</v>
+      </c>
+      <c r="C14" t="s">
+        <v>748</v>
+      </c>
+      <c r="D14" t="s">
+        <v>677</v>
+      </c>
+      <c r="E14" t="s">
         <v>700</v>
       </c>
-      <c r="W13" t="s">
-        <v>711</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>712</v>
-      </c>
-      <c r="B14" t="s">
-        <v>713</v>
-      </c>
-      <c r="C14" t="s">
-        <v>714</v>
-      </c>
-      <c r="D14" t="s">
-        <v>681</v>
-      </c>
-      <c r="E14" t="s">
-        <v>715</v>
-      </c>
       <c r="F14" t="s">
-        <v>706</v>
+        <v>693</v>
       </c>
       <c r="G14" t="s">
-        <v>707</v>
+        <v>694</v>
       </c>
       <c r="H14" t="s">
-        <v>708</v>
+        <v>739</v>
       </c>
       <c r="I14" t="s">
-        <v>709</v>
+        <v>695</v>
       </c>
       <c r="J14" t="s">
         <v>131</v>
@@ -5928,7 +5865,7 @@
         <v>16</v>
       </c>
       <c r="Q14" t="s">
-        <v>710</v>
+        <v>696</v>
       </c>
       <c r="R14">
         <v>0</v>
@@ -5946,36 +5883,33 @@
         <v>63</v>
       </c>
       <c r="W14" t="s">
-        <v>716</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>717</v>
+        <v>702</v>
       </c>
       <c r="B15" t="s">
-        <v>718</v>
+        <v>703</v>
       </c>
       <c r="C15" t="s">
-        <v>719</v>
+        <v>749</v>
       </c>
       <c r="D15" t="s">
-        <v>681</v>
+        <v>753</v>
       </c>
       <c r="E15" t="s">
-        <v>720</v>
-      </c>
-      <c r="F15" t="s">
-        <v>721</v>
+        <v>754</v>
       </c>
       <c r="G15" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="H15" t="s">
-        <v>723</v>
+        <v>739</v>
       </c>
       <c r="I15" t="s">
-        <v>709</v>
+        <v>695</v>
       </c>
       <c r="J15" t="s">
         <v>131</v>
@@ -5987,7 +5921,7 @@
         <v>16</v>
       </c>
       <c r="Q15" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="R15">
         <v>23</v>
@@ -6002,134 +5936,16 @@
         <v>46274</v>
       </c>
       <c r="V15" t="s">
-        <v>724</v>
+        <v>704</v>
       </c>
       <c r="W15" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>726</v>
-      </c>
-      <c r="B16" t="s">
-        <v>727</v>
-      </c>
-      <c r="C16" t="s">
-        <v>728</v>
-      </c>
-      <c r="D16" t="s">
-        <v>681</v>
-      </c>
-      <c r="E16" t="s">
-        <v>729</v>
-      </c>
-      <c r="F16" t="s">
-        <v>721</v>
-      </c>
-      <c r="G16" t="s">
-        <v>730</v>
-      </c>
-      <c r="H16" t="s">
-        <v>731</v>
-      </c>
-      <c r="I16" t="s">
-        <v>643</v>
-      </c>
-      <c r="J16" t="s">
-        <v>131</v>
-      </c>
-      <c r="K16" t="s">
-        <v>131</v>
-      </c>
-      <c r="P16" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>732</v>
-      </c>
-      <c r="R16">
-        <v>19</v>
-      </c>
-      <c r="S16">
-        <v>250</v>
-      </c>
-      <c r="T16">
-        <v>288</v>
-      </c>
-      <c r="U16" s="1">
-        <v>46274</v>
-      </c>
-      <c r="V16" t="s">
-        <v>733</v>
-      </c>
-      <c r="W16" t="s">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>735</v>
-      </c>
-      <c r="B17" t="s">
-        <v>736</v>
-      </c>
-      <c r="C17" t="s">
-        <v>737</v>
-      </c>
-      <c r="D17" t="s">
-        <v>681</v>
-      </c>
-      <c r="E17" t="s">
-        <v>738</v>
-      </c>
-      <c r="F17" t="s">
-        <v>721</v>
-      </c>
-      <c r="G17" t="s">
-        <v>722</v>
-      </c>
-      <c r="H17" t="s">
-        <v>723</v>
-      </c>
-      <c r="I17" t="s">
-        <v>709</v>
-      </c>
-      <c r="J17" t="s">
-        <v>131</v>
-      </c>
-      <c r="K17" t="s">
-        <v>131</v>
-      </c>
-      <c r="P17" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>650</v>
-      </c>
-      <c r="R17">
-        <v>23</v>
-      </c>
-      <c r="S17">
-        <v>337</v>
-      </c>
-      <c r="T17">
-        <v>288</v>
-      </c>
-      <c r="U17" s="1">
-        <v>46274</v>
-      </c>
-      <c r="V17" t="s">
-        <v>724</v>
-      </c>
-      <c r="W17" t="s">
-        <v>739</v>
+        <v>705</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:W1 A8:B8 A2:B2 D2:F2 A3:B3 D3:E3 A17:I17 A9:B9 D9:I9 I2 P2 R2:T2 V2:W2 V3:W3 A4:B4 V4:W4 A5:B5 V5:W5 A6:B6 V6:W6 A7:B7 V7:W7 V8:W8 V9:W9 A10:I10 V10:W10 A11:I11 V11:W11 A12:I12 V12:W12 A13:I13 V13:W13 A14:I14 V14:W14 A15:I15 V15:W15 A16:I16 V16:W16 V17:W17 D8 D4 D5 D6:F6 D7:F7 I3 P3:T3 P17:T17 P9:T9 P10:T10 P11:T11 P12:T12 P13:T13 R14:T14 P15:T15 P16:T16 P8:T8 P4:T4 Q5:T5 P6:T6 P7:T7 I4 F5 I6 F8" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:W1 A8:B8 A2:B2 D2:F2 A3:B3 D3:E3 A9:B9 D9 I2 P2 R2:T2 V2:W2 V3:W3 A4:B4 V4:W4 A5:B5 V5:W5 A6:B6 V6:W6 A7:B7 V7:W7 V8:W8 V9:W9 A10:B10 V10:W10 A11:B11 V11:W11 A12:B12 V12:W12 A13:B13 V13:W13 A14:B14 V14:W14 A15:B15 V15:W15 D8 D4 D5 D6:F6 D7:F7 I3 P3:T3 P9:T9 P10:T10 P11:T11 P12:T12 P13:T13 R14:T14 P15:T15 P8:T8 P4:T4 Q5:T5 P6:T6 P7:T7 I4 F5 I6 D10 D11 D12 D13 D14:G14 I9 I10 I11 I12 I13 I14 I15 F10 F11 F12 F13:G13" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6137,20 +5953,20 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>740</v>
+        <v>706</v>
       </c>
       <c r="B1" t="s">
         <v>622</v>
       </c>
       <c r="C1" t="s">
-        <v>741</v>
+        <v>707</v>
       </c>
       <c r="D1" t="s">
-        <v>742</v>
+        <v>708</v>
       </c>
       <c r="E1" t="s">
         <v>468</v>
@@ -6159,16 +5975,16 @@
         <v>429</v>
       </c>
       <c r="G1" t="s">
-        <v>743</v>
+        <v>709</v>
       </c>
       <c r="H1" t="s">
-        <v>744</v>
+        <v>710</v>
       </c>
       <c r="I1" t="s">
-        <v>745</v>
+        <v>711</v>
       </c>
       <c r="J1" t="s">
-        <v>746</v>
+        <v>712</v>
       </c>
       <c r="K1" t="s">
         <v>636</v>
@@ -6188,9 +6004,9 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>422</v>
       </c>
@@ -6198,13 +6014,13 @@
         <v>622</v>
       </c>
       <c r="C1" t="s">
-        <v>747</v>
+        <v>713</v>
       </c>
       <c r="D1" t="s">
-        <v>748</v>
+        <v>714</v>
       </c>
       <c r="E1" t="s">
-        <v>749</v>
+        <v>715</v>
       </c>
       <c r="F1" t="s">
         <v>427</v>
@@ -6219,7 +6035,7 @@
         <v>7</v>
       </c>
       <c r="J1" t="s">
-        <v>743</v>
+        <v>709</v>
       </c>
       <c r="K1" t="s">
         <v>9</v>
@@ -6236,14 +6052,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:N1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>750</v>
+        <v>716</v>
       </c>
       <c r="B1" t="s">
-        <v>751</v>
+        <v>717</v>
       </c>
       <c r="C1" t="s">
         <v>625</v>
@@ -6252,31 +6068,31 @@
         <v>91</v>
       </c>
       <c r="E1" t="s">
-        <v>752</v>
+        <v>718</v>
       </c>
       <c r="F1" t="s">
-        <v>753</v>
+        <v>719</v>
       </c>
       <c r="G1" t="s">
-        <v>754</v>
+        <v>720</v>
       </c>
       <c r="H1" t="s">
-        <v>755</v>
+        <v>721</v>
       </c>
       <c r="I1" t="s">
-        <v>756</v>
+        <v>722</v>
       </c>
       <c r="J1" t="s">
-        <v>757</v>
+        <v>723</v>
       </c>
       <c r="K1" t="s">
-        <v>758</v>
+        <v>724</v>
       </c>
       <c r="L1" t="s">
-        <v>759</v>
+        <v>725</v>
       </c>
       <c r="M1" t="s">
-        <v>760</v>
+        <v>726</v>
       </c>
       <c r="N1" t="s">
         <v>9</v>
@@ -6293,9 +6109,9 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>285</v>
       </c>
@@ -6311,9 +6127,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -6327,7 +6143,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -6341,7 +6157,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -6355,7 +6171,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -6369,7 +6185,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -6383,7 +6199,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -6397,7 +6213,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -6422,9 +6238,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>88</v>
       </c>
@@ -6447,7 +6263,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -6470,7 +6286,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>98</v>
       </c>
@@ -6493,7 +6309,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>104</v>
       </c>
@@ -6516,7 +6332,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>108</v>
       </c>
@@ -6550,9 +6366,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:R64"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>112</v>
       </c>
@@ -6608,7 +6424,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>128</v>
       </c>
@@ -6655,7 +6471,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -6702,7 +6518,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>139</v>
       </c>
@@ -6749,7 +6565,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>144</v>
       </c>
@@ -6796,7 +6612,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>148</v>
       </c>
@@ -6843,7 +6659,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -6890,7 +6706,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>156</v>
       </c>
@@ -6937,7 +6753,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -6984,7 +6800,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>164</v>
       </c>
@@ -7031,7 +6847,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>166</v>
       </c>
@@ -7078,7 +6894,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>168</v>
       </c>
@@ -7125,7 +6941,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>166</v>
       </c>
@@ -7181,7 +6997,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -7228,7 +7044,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>182</v>
       </c>
@@ -7275,7 +7091,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>187</v>
       </c>
@@ -7322,7 +7138,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>191</v>
       </c>
@@ -7369,7 +7185,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>194</v>
       </c>
@@ -7416,7 +7232,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -7463,7 +7279,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -7510,7 +7326,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -7557,7 +7373,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>201</v>
       </c>
@@ -7604,7 +7420,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -7651,7 +7467,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>206</v>
       </c>
@@ -7707,7 +7523,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>211</v>
       </c>
@@ -7754,7 +7570,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>213</v>
       </c>
@@ -7801,7 +7617,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>217</v>
       </c>
@@ -7848,7 +7664,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -7895,7 +7711,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>14</v>
       </c>
@@ -7942,7 +7758,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>14</v>
       </c>
@@ -7989,7 +7805,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>224</v>
       </c>
@@ -8036,7 +7852,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>14</v>
       </c>
@@ -8083,7 +7899,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="33" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>14</v>
       </c>
@@ -8130,7 +7946,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="34" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>231</v>
       </c>
@@ -8177,7 +7993,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="35" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>234</v>
       </c>
@@ -8224,7 +8040,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="36" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -8271,7 +8087,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="37" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>237</v>
       </c>
@@ -8318,7 +8134,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="38" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>239</v>
       </c>
@@ -8365,7 +8181,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="39" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -8412,7 +8228,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="40" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>14</v>
       </c>
@@ -8459,7 +8275,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="41" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>14</v>
       </c>
@@ -8506,7 +8322,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="42" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>14</v>
       </c>
@@ -8553,7 +8369,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>247</v>
       </c>
@@ -8600,7 +8416,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="44" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>249</v>
       </c>
@@ -8647,7 +8463,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="45" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>14</v>
       </c>
@@ -8694,7 +8510,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="46" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>14</v>
       </c>
@@ -8741,7 +8557,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="47" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>14</v>
       </c>
@@ -8788,7 +8604,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="48" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>14</v>
       </c>
@@ -8835,7 +8651,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="49" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>14</v>
       </c>
@@ -8882,7 +8698,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="50" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>14</v>
       </c>
@@ -8929,7 +8745,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="51" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>14</v>
       </c>
@@ -8976,7 +8792,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="52" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>259</v>
       </c>
@@ -9023,7 +8839,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="53" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>261</v>
       </c>
@@ -9070,7 +8886,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="54" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>263</v>
       </c>
@@ -9117,7 +8933,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="55" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>265</v>
       </c>
@@ -9164,7 +8980,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="56" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>267</v>
       </c>
@@ -9211,7 +9027,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="57" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>269</v>
       </c>
@@ -9258,7 +9074,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="58" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>271</v>
       </c>
@@ -9305,7 +9121,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="59" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>274</v>
       </c>
@@ -9352,7 +9168,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="60" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>14</v>
       </c>
@@ -9399,7 +9215,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="61" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>14</v>
       </c>
@@ -9446,7 +9262,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="62" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>279</v>
       </c>
@@ -9493,7 +9309,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="63" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>281</v>
       </c>
@@ -9540,7 +9356,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="64" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>283</v>
       </c>
@@ -9598,9 +9414,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>285</v>
       </c>
@@ -9616,9 +9432,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:L62"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>286</v>
       </c>
@@ -9656,7 +9472,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>294</v>
       </c>
@@ -9691,7 +9507,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>298</v>
       </c>
@@ -9726,7 +9542,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>300</v>
       </c>
@@ -9761,7 +9577,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>301</v>
       </c>
@@ -9799,7 +9615,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>306</v>
       </c>
@@ -9834,7 +9650,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>309</v>
       </c>
@@ -9869,7 +9685,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>310</v>
       </c>
@@ -9904,7 +9720,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>311</v>
       </c>
@@ -9939,7 +9755,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>313</v>
       </c>
@@ -9974,7 +9790,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>314</v>
       </c>
@@ -10009,7 +9825,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>315</v>
       </c>
@@ -10044,7 +9860,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>316</v>
       </c>
@@ -10079,7 +9895,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>317</v>
       </c>
@@ -10114,7 +9930,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>318</v>
       </c>
@@ -10149,7 +9965,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>319</v>
       </c>
@@ -10184,7 +10000,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>320</v>
       </c>
@@ -10219,7 +10035,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>321</v>
       </c>
@@ -10254,7 +10070,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>322</v>
       </c>
@@ -10289,7 +10105,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>323</v>
       </c>
@@ -10324,7 +10140,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>324</v>
       </c>
@@ -10359,7 +10175,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>325</v>
       </c>
@@ -10394,7 +10210,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>326</v>
       </c>
@@ -10429,7 +10245,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>327</v>
       </c>
@@ -10464,7 +10280,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>328</v>
       </c>
@@ -10499,7 +10315,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>329</v>
       </c>
@@ -10534,7 +10350,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>330</v>
       </c>
@@ -10569,7 +10385,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>331</v>
       </c>
@@ -10604,7 +10420,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>332</v>
       </c>
@@ -10639,7 +10455,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>333</v>
       </c>
@@ -10674,7 +10490,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>334</v>
       </c>
@@ -10709,7 +10525,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>335</v>
       </c>
@@ -10744,7 +10560,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>336</v>
       </c>
@@ -10779,7 +10595,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>337</v>
       </c>
@@ -10814,7 +10630,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>338</v>
       </c>
@@ -10849,7 +10665,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>339</v>
       </c>
@@ -10884,7 +10700,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>340</v>
       </c>
@@ -10919,7 +10735,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>341</v>
       </c>
@@ -10954,7 +10770,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>342</v>
       </c>
@@ -10989,7 +10805,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>343</v>
       </c>
@@ -11024,7 +10840,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>344</v>
       </c>
@@ -11059,7 +10875,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>345</v>
       </c>
@@ -11094,7 +10910,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>346</v>
       </c>
@@ -11129,7 +10945,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>347</v>
       </c>
@@ -11164,7 +10980,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>348</v>
       </c>
@@ -11199,7 +11015,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>349</v>
       </c>
@@ -11234,7 +11050,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>350</v>
       </c>
@@ -11269,7 +11085,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>351</v>
       </c>
@@ -11304,7 +11120,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>352</v>
       </c>
@@ -11339,7 +11155,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>353</v>
       </c>
@@ -11374,7 +11190,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>354</v>
       </c>
@@ -11409,7 +11225,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>355</v>
       </c>
@@ -11444,7 +11260,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>356</v>
       </c>
@@ -11479,7 +11295,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>357</v>
       </c>
@@ -11514,7 +11330,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>361</v>
       </c>
@@ -11549,7 +11365,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>362</v>
       </c>
@@ -11584,7 +11400,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>363</v>
       </c>
@@ -11619,7 +11435,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>364</v>
       </c>
@@ -11654,7 +11470,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>365</v>
       </c>
@@ -11689,7 +11505,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>366</v>
       </c>
@@ -11724,7 +11540,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>367</v>
       </c>
@@ -11759,7 +11575,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>368</v>
       </c>
@@ -11805,9 +11621,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>369</v>
       </c>
@@ -11839,7 +11655,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>374</v>
       </c>
@@ -11871,7 +11687,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>379</v>
       </c>
@@ -11903,7 +11719,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>382</v>
       </c>
@@ -11935,7 +11751,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>384</v>
       </c>
@@ -11967,7 +11783,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>389</v>
       </c>
@@ -12010,9 +11826,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>393</v>
       </c>
@@ -12053,7 +11869,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>403</v>
       </c>
@@ -12094,7 +11910,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>410</v>
       </c>
@@ -12135,7 +11951,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>413</v>
       </c>
@@ -12176,7 +11992,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>417</v>
       </c>
@@ -12217,7 +12033,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>421</v>
       </c>
@@ -12269,9 +12085,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:Q6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>422</v>
       </c>
@@ -12324,7 +12140,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>435</v>
       </c>
@@ -12377,7 +12193,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>441</v>
       </c>
@@ -12430,7 +12246,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>445</v>
       </c>
@@ -12483,7 +12299,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>451</v>
       </c>
@@ -12536,7 +12352,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>454</v>
       </c>

</xml_diff>

<commit_message>
feat: add relational database seed data and Excel database files
</commit_message>
<xml_diff>
--- a/database/IT_Asset_Database.xlsx
+++ b/database/IT_Asset_Database.xlsx
@@ -2071,7 +2071,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2119,22 +2119,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ACS-0005</v>
+        <v>ACS-0006</v>
       </c>
       <c r="B2" t="str">
-        <v>ACS-0005</v>
+        <v>ACS-0006</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-09-09</v>
+        <v>2026-07-13</v>
       </c>
       <c r="D2" t="str">
-        <v>Saman Ref Enginering</v>
+        <v>Saman Ref. Engineering (Ruchira)</v>
       </c>
       <c r="E2">
-        <v>2500</v>
+        <v>20000</v>
       </c>
       <c r="F2" t="str">
-        <v>AC-0002</v>
+        <v>AC-0005</v>
       </c>
       <c r="G2" t="str">
         <v/>
@@ -2143,7 +2143,7 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>ACS-0005</v>
+        <v>ACS-0006</v>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -2155,30 +2155,30 @@
         <v/>
       </c>
       <c r="M2" t="str">
-        <v>2026-09-09</v>
+        <v>2026-07-13</v>
       </c>
       <c r="N2" t="str">
-        <v xml:space="preserve">[AC Service - AC-0002] Routine Maintenance: </v>
+        <v>[AC Service - AC-0005] Replacement &amp; Installation: Abans AC එකක් Cool එක මදි කියල Haier 240000 AC එකට මාරු කරා</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ACS-0004</v>
+        <v>ACS-0005</v>
       </c>
       <c r="B3" t="str">
-        <v>ACS-0004</v>
+        <v>ACS-0005</v>
       </c>
       <c r="C3" t="str">
         <v>2026-09-09</v>
       </c>
       <c r="D3" t="str">
-        <v>Saman Ref Engineering</v>
+        <v>Saman Ref Enginering</v>
       </c>
       <c r="E3">
         <v>2500</v>
       </c>
       <c r="F3" t="str">
-        <v>AC-0001</v>
+        <v>AC-0002</v>
       </c>
       <c r="G3" t="str">
         <v/>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>ACS-0004</v>
+        <v>ACS-0005</v>
       </c>
       <c r="J3" t="str">
         <v/>
@@ -2202,15 +2202,15 @@
         <v>2026-09-09</v>
       </c>
       <c r="N3" t="str">
-        <v xml:space="preserve">[AC Service - AC-0001] Routine Maintenance: </v>
+        <v xml:space="preserve">[AC Service - AC-0002] Routine Maintenance: </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ACS-0003</v>
+        <v>ACS-0004</v>
       </c>
       <c r="B4" t="str">
-        <v>ACS-0003</v>
+        <v>ACS-0004</v>
       </c>
       <c r="C4" t="str">
         <v>2026-09-09</v>
@@ -2222,7 +2222,7 @@
         <v>2500</v>
       </c>
       <c r="F4" t="str">
-        <v>AC-0004</v>
+        <v>AC-0001</v>
       </c>
       <c r="G4" t="str">
         <v/>
@@ -2231,7 +2231,7 @@
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>ACS-0003</v>
+        <v>ACS-0004</v>
       </c>
       <c r="J4" t="str">
         <v/>
@@ -2246,15 +2246,15 @@
         <v>2026-09-09</v>
       </c>
       <c r="N4" t="str">
-        <v xml:space="preserve">[AC Service - AC-0004] Routine Maintenance: </v>
+        <v xml:space="preserve">[AC Service - AC-0001] Routine Maintenance: </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ACS-0002</v>
+        <v>ACS-0003</v>
       </c>
       <c r="B5" t="str">
-        <v>ACS-0002</v>
+        <v>ACS-0003</v>
       </c>
       <c r="C5" t="str">
         <v>2026-09-09</v>
@@ -2266,7 +2266,7 @@
         <v>2500</v>
       </c>
       <c r="F5" t="str">
-        <v>AC-0003</v>
+        <v>AC-0004</v>
       </c>
       <c r="G5" t="str">
         <v/>
@@ -2275,7 +2275,7 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>ACS-0002</v>
+        <v>ACS-0003</v>
       </c>
       <c r="J5" t="str">
         <v/>
@@ -2290,18 +2290,18 @@
         <v>2026-09-09</v>
       </c>
       <c r="N5" t="str">
-        <v xml:space="preserve">[AC Service - AC-0003] Routine Maintenance: </v>
+        <v xml:space="preserve">[AC Service - AC-0004] Routine Maintenance: </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ACS-0001</v>
+        <v>ACS-0002</v>
       </c>
       <c r="B6" t="str">
-        <v>ACS-0001</v>
+        <v>ACS-0002</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-05-26</v>
+        <v>2026-09-09</v>
       </c>
       <c r="D6" t="str">
         <v>Saman Ref Engineering</v>
@@ -2310,7 +2310,7 @@
         <v>2500</v>
       </c>
       <c r="F6" t="str">
-        <v>AC-0001</v>
+        <v>AC-0003</v>
       </c>
       <c r="G6" t="str">
         <v/>
@@ -2319,7 +2319,7 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>ACS-0001</v>
+        <v>ACS-0002</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -2331,30 +2331,30 @@
         <v/>
       </c>
       <c r="M6" t="str">
-        <v>2026-05-26</v>
+        <v>2026-09-09</v>
       </c>
       <c r="N6" t="str">
-        <v xml:space="preserve">[AC Service - AC-0001] Emergency Service: </v>
+        <v xml:space="preserve">[AC Service - AC-0003] Routine Maintenance: </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ACR-0001</v>
+        <v>ACS-0001</v>
       </c>
       <c r="B7" t="str">
-        <v>ACR-0001</v>
+        <v>ACS-0001</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-09-25</v>
+        <v>2026-05-26</v>
       </c>
       <c r="D7" t="str">
-        <v>Saman Ref Engineer</v>
+        <v>Saman Ref Engineering</v>
       </c>
       <c r="E7">
         <v>2500</v>
       </c>
       <c r="F7" t="str">
-        <v>AC-0006</v>
+        <v>AC-0001</v>
       </c>
       <c r="G7" t="str">
         <v/>
@@ -2363,7 +2363,7 @@
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>ACR-0001</v>
+        <v>ACS-0001</v>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -2375,30 +2375,30 @@
         <v/>
       </c>
       <c r="M7" t="str">
-        <v>2026-09-25</v>
+        <v>2026-05-26</v>
       </c>
       <c r="N7" t="str">
-        <v>[AC Repair - AC-0006] Drain leak Repair</v>
+        <v xml:space="preserve">[AC Service - AC-0001] Emergency Service: </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>INV-0008</v>
+        <v>ACR-0001</v>
       </c>
       <c r="B8" t="str">
-        <v>04_08_2026_</v>
+        <v>ACR-0001</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-08-04</v>
+        <v>2026-09-25</v>
       </c>
       <c r="D8" t="str">
-        <v>KMN IT Solution</v>
+        <v>Saman Ref Engineer</v>
       </c>
       <c r="E8">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="F8" t="str">
-        <v>AST-0052</v>
+        <v>AC-0006</v>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -2407,107 +2407,107 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>ACR-0001</v>
       </c>
       <c r="J8" t="str">
-        <v>04.08.2026..pdf</v>
+        <v/>
       </c>
       <c r="K8" t="str">
-        <v>/invoices/04.08.2026..pdf</v>
+        <v/>
       </c>
       <c r="L8" t="str">
-        <v>545 KB</v>
+        <v/>
       </c>
       <c r="M8" t="str">
-        <v>2026-09-23</v>
+        <v>2026-09-25</v>
       </c>
       <c r="N8" t="str">
-        <v xml:space="preserve">Invoice for repair/service: Power cable not worked </v>
+        <v>[AC Repair - AC-0006] Drain leak Repair</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>INV-0007</v>
+        <v>INV-0008</v>
       </c>
       <c r="B9" t="str">
-        <v>kmn_aqua</v>
+        <v>04_08_2026_</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-09-17</v>
+        <v>2026-08-04</v>
       </c>
       <c r="D9" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E9">
-        <v>4800</v>
+        <v>1000</v>
       </c>
       <c r="F9" t="str">
-        <v>AST-0057</v>
+        <v>AST-0052</v>
       </c>
       <c r="G9" t="str">
         <v/>
       </c>
       <c r="H9" t="str">
-        <v>AST-0057</v>
+        <v/>
       </c>
       <c r="I9" t="str">
         <v/>
       </c>
       <c r="J9" t="str">
-        <v>17.09.26.pdf</v>
+        <v>04.08.2026..pdf</v>
       </c>
       <c r="K9" t="str">
-        <v>/invoices/17.09.26.pdf</v>
+        <v>/invoices/04.08.2026..pdf</v>
       </c>
       <c r="L9" t="str">
         <v>545 KB</v>
       </c>
       <c r="M9" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-23</v>
       </c>
       <c r="N9" t="str">
-        <v>Black Toner for printer</v>
+        <v xml:space="preserve">Invoice for repair/service: Power cable not worked </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>INV-0006</v>
+        <v>INV-0007</v>
       </c>
       <c r="B10" t="str">
-        <v>23_07_2026_</v>
+        <v>kmn_aqua</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-07-23</v>
+        <v>2026-09-17</v>
       </c>
       <c r="D10" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E10">
-        <v>8000</v>
+        <v>4800</v>
       </c>
       <c r="F10" t="str">
-        <v>AST-0059</v>
+        <v>AST-0057</v>
       </c>
       <c r="G10" t="str">
         <v/>
       </c>
       <c r="H10" t="str">
-        <v>AST-0059</v>
+        <v>AST-0057</v>
       </c>
       <c r="I10" t="str">
         <v/>
       </c>
       <c r="J10" t="str">
-        <v>23.07.2026..pdf</v>
+        <v>17.09.26.pdf</v>
       </c>
       <c r="K10" t="str">
-        <v>/invoices/23.07.2026..pdf</v>
+        <v>/invoices/17.09.26.pdf</v>
       </c>
       <c r="L10" t="str">
-        <v>633 KB</v>
+        <v>545 KB</v>
       </c>
       <c r="M10" t="str">
-        <v>2026-07-23</v>
+        <v>2026-09-17</v>
       </c>
       <c r="N10" t="str">
         <v>Black Toner for printer</v>
@@ -2515,69 +2515,69 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>INV-0005</v>
+        <v>INV-0006</v>
       </c>
       <c r="B11" t="str">
-        <v>14.08.2026.</v>
+        <v>23_07_2026_</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-08-14</v>
+        <v>2026-07-23</v>
       </c>
       <c r="D11" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E11">
-        <v>9200</v>
+        <v>8000</v>
       </c>
       <c r="F11" t="str">
-        <v>AST-0060</v>
+        <v>AST-0059</v>
       </c>
       <c r="G11" t="str">
         <v/>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>AST-0059</v>
       </c>
       <c r="I11" t="str">
         <v/>
       </c>
       <c r="J11" t="str">
-        <v>14.08.2026..pdf</v>
+        <v>23.07.2026..pdf</v>
       </c>
       <c r="K11" t="str">
-        <v>/invoices/14.08.2026..pdf</v>
+        <v>/invoices/23.07.2026..pdf</v>
       </c>
       <c r="L11" t="str">
-        <v>641 KB</v>
+        <v>633 KB</v>
       </c>
       <c r="M11" t="str">
-        <v>2026-09-22</v>
+        <v>2026-07-23</v>
       </c>
       <c r="N11" t="str">
-        <v>Uploaded Invoice: 14.08.2026..pdf</v>
+        <v>Black Toner for printer</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>INV-0004</v>
+        <v>INV-0005</v>
       </c>
       <c r="B12" t="str">
-        <v>01.07.2026.</v>
+        <v>14.08.2026.</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-07-01</v>
+        <v>2026-08-14</v>
       </c>
       <c r="D12" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E12">
-        <v>5650</v>
+        <v>9200</v>
       </c>
       <c r="F12" t="str">
-        <v>AST-0063</v>
+        <v>AST-0060</v>
       </c>
       <c r="G12" t="str">
-        <v>USR-0016</v>
+        <v/>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -2586,42 +2586,42 @@
         <v/>
       </c>
       <c r="J12" t="str">
-        <v>01.07.2026..pdf</v>
+        <v>14.08.2026..pdf</v>
       </c>
       <c r="K12" t="str">
-        <v>/invoices/01.07.2026..pdf</v>
+        <v>/invoices/14.08.2026..pdf</v>
       </c>
       <c r="L12" t="str">
-        <v>494 KB</v>
+        <v>641 KB</v>
       </c>
       <c r="M12" t="str">
         <v>2026-09-22</v>
       </c>
       <c r="N12" t="str">
-        <v>ADD TO TONNER 680 BLACK AND COLOUR</v>
+        <v>Uploaded Invoice: 14.08.2026..pdf</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>INV-0003</v>
+        <v>INV-0004</v>
       </c>
       <c r="B13" t="str">
-        <v>07_09_2026_</v>
+        <v>01.07.2026.</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-09-07</v>
+        <v>2026-07-01</v>
       </c>
       <c r="D13" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E13">
-        <v>1000</v>
+        <v>5650</v>
       </c>
       <c r="F13" t="str">
-        <v>AST-0052</v>
+        <v>AST-0063</v>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>USR-0016</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -2630,36 +2630,36 @@
         <v/>
       </c>
       <c r="J13" t="str">
-        <v>07.09.2026..pdf</v>
+        <v>01.07.2026..pdf</v>
       </c>
       <c r="K13" t="str">
-        <v>/invoices/07.09.2026..pdf</v>
+        <v>/invoices/01.07.2026..pdf</v>
       </c>
       <c r="L13" t="str">
-        <v>638 KB</v>
+        <v>494 KB</v>
       </c>
       <c r="M13" t="str">
         <v>2026-09-22</v>
       </c>
       <c r="N13" t="str">
-        <v>Invoice for repair/service: HAVEN'T A MOUSE</v>
+        <v>ADD TO TONNER 680 BLACK AND COLOUR</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>INV-0002</v>
+        <v>INV-0003</v>
       </c>
       <c r="B14" t="str">
-        <v>10_09_2026_</v>
+        <v>07_09_2026_</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-07</v>
       </c>
       <c r="D14" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E14">
-        <v>30000</v>
+        <v>1000</v>
       </c>
       <c r="F14" t="str">
         <v>AST-0052</v>
@@ -2674,39 +2674,39 @@
         <v/>
       </c>
       <c r="J14" t="str">
-        <v>10.09.2026..pdf</v>
+        <v>07.09.2026..pdf</v>
       </c>
       <c r="K14" t="str">
-        <v>/invoices/10.09.2026..pdf</v>
+        <v>/invoices/07.09.2026..pdf</v>
       </c>
       <c r="L14" t="str">
-        <v>633 KB</v>
+        <v>638 KB</v>
       </c>
       <c r="M14" t="str">
         <v>2026-09-22</v>
       </c>
       <c r="N14" t="str">
-        <v>Invoice for repair/service: STUCK &amp; SLOW</v>
+        <v>Invoice for repair/service: HAVEN'T A MOUSE</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>INV-0001</v>
+        <v>INV-0002</v>
       </c>
       <c r="B15" t="str">
-        <v>05_09_2026_</v>
+        <v>10_09_2026_</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-10</v>
       </c>
       <c r="D15" t="str">
         <v>KMN IT Solution</v>
       </c>
       <c r="E15">
-        <v>36000</v>
+        <v>30000</v>
       </c>
       <c r="F15" t="str">
-        <v>AST-0041</v>
+        <v>AST-0052</v>
       </c>
       <c r="G15" t="str">
         <v/>
@@ -2718,13 +2718,13 @@
         <v/>
       </c>
       <c r="J15" t="str">
-        <v>05.09.2026..pdf</v>
+        <v>10.09.2026..pdf</v>
       </c>
       <c r="K15" t="str">
-        <v>/invoices/05.09.2026..pdf</v>
+        <v>/invoices/10.09.2026..pdf</v>
       </c>
       <c r="L15" t="str">
-        <v>639 KB</v>
+        <v>633 KB</v>
       </c>
       <c r="M15" t="str">
         <v>2026-09-22</v>
@@ -2733,9 +2733,53 @@
         <v>Invoice for repair/service: STUCK &amp; SLOW</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>INV-0001</v>
+      </c>
+      <c r="B16" t="str">
+        <v>05_09_2026_</v>
+      </c>
+      <c r="C16" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="D16" t="str">
+        <v>KMN IT Solution</v>
+      </c>
+      <c r="E16">
+        <v>36000</v>
+      </c>
+      <c r="F16" t="str">
+        <v>AST-0041</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v>05.09.2026..pdf</v>
+      </c>
+      <c r="K16" t="str">
+        <v>/invoices/05.09.2026..pdf</v>
+      </c>
+      <c r="L16" t="str">
+        <v>639 KB</v>
+      </c>
+      <c r="M16" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Invoice for repair/service: STUCK &amp; SLOW</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3017,7 +3061,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:T15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3077,6 +3121,9 @@
       <c r="S1" t="str">
         <v>Notes</v>
       </c>
+      <c r="T1" t="str">
+        <v>PurchaseDate</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -3119,7 +3166,7 @@
         <v>Eco Cooling</v>
       </c>
       <c r="N2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="O2">
         <v>752</v>
@@ -3364,13 +3411,16 @@
         <v>628</v>
       </c>
       <c r="Q6" t="str">
-        <v>2026-09-09</v>
+        <v>2026-07-13</v>
       </c>
       <c r="R6" t="str">
         <v>2026-09-18</v>
       </c>
       <c r="S6" t="str">
-        <v>Ground floor Boss office executive suite cooling unit</v>
+        <v>Haier 24,000 BTU Dual Inverter installed on 2026-07-13. Replaced old Abans AC which was moved due to low cooling.</v>
+      </c>
+      <c r="T6" t="str">
+        <v>2026-07-13</v>
       </c>
     </row>
     <row r="7">
@@ -3903,14 +3953,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4149,22 +4199,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ACS-0001</v>
+        <v>ACS-0006</v>
       </c>
       <c r="B6" t="str">
-        <v>AC-0001</v>
+        <v>AC-0005</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-05-26</v>
+        <v>2026-07-13</v>
       </c>
       <c r="D6" t="str">
-        <v>Emergency Service</v>
+        <v>Replacement &amp; Installation</v>
       </c>
       <c r="E6">
-        <v>2500</v>
+        <v>20000</v>
       </c>
       <c r="F6" t="str">
-        <v>Saman Ref Engineering</v>
+        <v>Saman Ref. Engineering (Ruchira)</v>
       </c>
       <c r="G6" t="str">
         <v/>
@@ -4182,7 +4232,7 @@
         <v/>
       </c>
       <c r="L6" t="str">
-        <v/>
+        <v>Abans AC එකක් Cool එක මදි කියල Haier 240000 AC එකට මාරු කරා (Old Abans AC moved due to low cooling, replaced with Haier 24,000 BTU)</v>
       </c>
       <c r="M6" t="str">
         <v/>
@@ -4191,12 +4241,59 @@
         <v/>
       </c>
       <c r="O6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ACS-0001</v>
+      </c>
+      <c r="B7" t="str">
+        <v>AC-0001</v>
+      </c>
+      <c r="C7" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Emergency Service</v>
+      </c>
+      <c r="E7">
+        <v>2500</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Saman Ref Engineering</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4302,16 +4399,111 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>ID</v>
+        <v>ReplacementID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>SpotCode</v>
+      </c>
+      <c r="C1" t="str">
+        <v>RoomName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Floor</v>
+      </c>
+      <c r="E1" t="str">
+        <v>OldUnitBrand</v>
+      </c>
+      <c r="F1" t="str">
+        <v>OldUnitModel</v>
+      </c>
+      <c r="G1" t="str">
+        <v>OldUnitPurchaseYear</v>
+      </c>
+      <c r="H1" t="str">
+        <v>OldUnitLifetimeServiceCost</v>
+      </c>
+      <c r="I1" t="str">
+        <v>OldUnitLifetimeRepairCost</v>
+      </c>
+      <c r="J1" t="str">
+        <v>RemovalDate</v>
+      </c>
+      <c r="K1" t="str">
+        <v>RemovalReason</v>
+      </c>
+      <c r="L1" t="str">
+        <v>FinalCondition</v>
+      </c>
+      <c r="M1" t="str">
+        <v>NewUnitID</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Technician</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Cost</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ACREP-0001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>CHW/AC/005</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Boss Office (Executive Suite)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Ground Floor</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Abans</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Abans AC (Relocated)</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2026-07-13</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Abans AC cooling insufficient, replaced with Haier 240000 AC (Abans AC එකක් Cool එක මදි කියල Haier 240000 AC එකට මාරු කරා)</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Moved / Relocated</v>
+      </c>
+      <c r="M2" t="str">
+        <v>AC-0005</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Saman Ref. Engineering (Ruchira)</v>
+      </c>
+      <c r="O2">
+        <v>20000</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Abans AC එකක් Cool එක මදි කියල Haier 240000 AC එකට මාරු කරා. Technician: Saman Ref. Engineering (Ruchira), Cost: Rs. 20,000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>